<commit_message>
Update funding data 2026-09-13
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$210</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M210"/>
+  <dimension ref="A1:M209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 12/09/2026 09:42 - 203 convocatorias - 11 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 13/09/2026 10:44 - 202 convocatorias - 11 nuevas</t>
         </is>
       </c>
     </row>
@@ -9802,11 +9802,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L197" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L197" s="6" t="inlineStr"/>
       <c r="M197" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -9814,21 +9810,21 @@
       </c>
     </row>
     <row r="198" ht="28" customHeight="1">
-      <c r="A198" s="16" t="inlineStr">
+      <c r="A198" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="199" ht="40" customHeight="1">
-      <c r="A199" s="17" t="inlineStr">
+      <c r="A199" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>EUS-47015</t>
+          <t>EUS-71187</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
@@ -9864,7 +9860,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L199" s="15" t="inlineStr">
+      <c r="L199" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -9876,14 +9872,14 @@
       </c>
     </row>
     <row r="200" ht="40" customHeight="1">
-      <c r="A200" s="17" t="inlineStr">
+      <c r="A200" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t>EUS-18875</t>
+          <t>EUS-18280</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
@@ -9919,7 +9915,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L200" s="15" t="inlineStr">
+      <c r="L200" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -9931,14 +9927,14 @@
       </c>
     </row>
     <row r="201" ht="40" customHeight="1">
-      <c r="A201" s="17" t="inlineStr">
+      <c r="A201" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>EUS-03901</t>
+          <t>EUS-83528</t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
@@ -9974,7 +9970,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L201" s="15" t="inlineStr">
+      <c r="L201" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -9986,14 +9982,14 @@
       </c>
     </row>
     <row r="202" ht="40" customHeight="1">
-      <c r="A202" s="17" t="inlineStr">
+      <c r="A202" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>EUS-17248</t>
+          <t>EUS-58263</t>
         </is>
       </c>
       <c r="C202" s="6" t="inlineStr">
@@ -10029,7 +10025,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L202" s="15" t="inlineStr">
+      <c r="L202" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10041,14 +10037,14 @@
       </c>
     </row>
     <row r="203" ht="40" customHeight="1">
-      <c r="A203" s="17" t="inlineStr">
+      <c r="A203" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B203" s="6" t="inlineStr">
         <is>
-          <t>EUS-36047</t>
+          <t>EUS-37780</t>
         </is>
       </c>
       <c r="C203" s="6" t="inlineStr">
@@ -10084,7 +10080,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L203" s="15" t="inlineStr">
+      <c r="L203" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10096,19 +10092,19 @@
       </c>
     </row>
     <row r="204" ht="40" customHeight="1">
-      <c r="A204" s="17" t="inlineStr">
+      <c r="A204" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B204" s="6" t="inlineStr">
         <is>
-          <t>EUS-38592</t>
+          <t>EUS-87782</t>
         </is>
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino 1800 natural,para mobiliario urbano. (pto 21036009)</t>
+          <t>Servicio de limpieza a prestar en las instalaciones del CENTRO DE DESARROLLO EMPRESARIAL DE LA MARGEN IZQUIERDA, S.A. (BIC BIZKAIA EZKERRALDEA) sitas en 48901 Barakaldo (Bizkaia), Avda. Altos Hornos d</t>
         </is>
       </c>
       <c r="D204" s="6" t="inlineStr">
@@ -10139,7 +10135,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L204" s="6" t="inlineStr"/>
+      <c r="L204" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M204" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -10147,19 +10147,19 @@
       </c>
     </row>
     <row r="205" ht="40" customHeight="1">
-      <c r="A205" s="17" t="inlineStr">
+      <c r="A205" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B205" s="6" t="inlineStr">
         <is>
-          <t>EUS-51365</t>
+          <t>EUS-48229</t>
         </is>
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de proyector digital para el Zornotza Aretoa</t>
+          <t>Servicio de mantenimiento integral del edificio e instalaciones de Azkuna Zentroa</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
@@ -10190,7 +10190,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L205" s="15" t="inlineStr">
+      <c r="L205" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10202,19 +10202,19 @@
       </c>
     </row>
     <row r="206" ht="40" customHeight="1">
-      <c r="A206" s="17" t="inlineStr">
+      <c r="A206" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>EUS-28575</t>
+          <t>EUS-84876</t>
         </is>
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>Suministro, colocación, integración y puesta en marcha de equipos de los sistemas de seguridad del edificio Koldo Mitxelena.</t>
+          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino 1800 natural,para mobiliario urbano. (pto 21036009)</t>
         </is>
       </c>
       <c r="D206" s="6" t="inlineStr">
@@ -10245,7 +10245,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L206" s="6" t="inlineStr"/>
+      <c r="L206" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M206" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -10253,19 +10257,19 @@
       </c>
     </row>
     <row r="207" ht="40" customHeight="1">
-      <c r="A207" s="17" t="inlineStr">
+      <c r="A207" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B207" s="6" t="inlineStr">
         <is>
-          <t>EUS-74130</t>
+          <t>EUS-51515</t>
         </is>
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>Levantamiento Topográfico de la Red de saneamiento y pluviales, así como inventario de arquetas del conjunto edificado del Hospital Universitario Donostia</t>
+          <t>Servicio de alquiler de proyector digital para el Zornotza Aretoa</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
@@ -10296,7 +10300,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L207" s="15" t="inlineStr">
+      <c r="L207" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10308,19 +10312,19 @@
       </c>
     </row>
     <row r="208" ht="40" customHeight="1">
-      <c r="A208" s="17" t="inlineStr">
+      <c r="A208" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B208" s="6" t="inlineStr">
         <is>
-          <t>EUS-74639</t>
+          <t>EUS-20770</t>
         </is>
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>Obras de adecuación a la protección contra incendios en el Edificio Anexo del Hospital de Leza</t>
+          <t>Suministro, colocación, integración y puesta en marcha de equipos de los sistemas de seguridad del edificio Koldo Mitxelena.</t>
         </is>
       </c>
       <c r="D208" s="6" t="inlineStr">
@@ -10351,7 +10355,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L208" s="15" t="inlineStr">
+      <c r="L208" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10363,19 +10367,19 @@
       </c>
     </row>
     <row r="209" ht="40" customHeight="1">
-      <c r="A209" s="17" t="inlineStr">
+      <c r="A209" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B209" s="6" t="inlineStr">
         <is>
-          <t>EUS-61809</t>
+          <t>EUS-12021</t>
         </is>
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>Transporte adaptado alumna.</t>
+          <t>Levantamiento Topográfico de la Red de saneamiento y pluviales, así como inventario de arquetas del conjunto edificado del Hospital Universitario Donostia</t>
         </is>
       </c>
       <c r="D209" s="6" t="inlineStr">
@@ -10406,7 +10410,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L209" s="15" t="inlineStr">
+      <c r="L209" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -10417,63 +10421,8 @@
         </is>
       </c>
     </row>
-    <row r="210" ht="40" customHeight="1">
-      <c r="A210" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B210" s="6" t="inlineStr">
-        <is>
-          <t>EUS-93696</t>
-        </is>
-      </c>
-      <c r="C210" s="6" t="inlineStr">
-        <is>
-          <t>Instalación paneles solares 10% instalación legalización</t>
-        </is>
-      </c>
-      <c r="D210" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E210" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F210" s="6" t="inlineStr"/>
-      <c r="G210" s="6" t="inlineStr"/>
-      <c r="H210" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I210" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J210" s="6" t="inlineStr"/>
-      <c r="K210" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L210" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M210" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M210"/>
+  <autoFilter ref="A4:M209"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -10684,7 +10633,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M210" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10696,7 +10644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3044"/>
+  <dimension ref="A1:F3029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -49814,7 +49762,7 @@
     <row r="2866" ht="30" customHeight="1">
       <c r="A2866" s="18" t="inlineStr">
         <is>
-          <t>FICHA 192: EUS-47015</t>
+          <t>FICHA 192: EUS-71187</t>
         </is>
       </c>
       <c r="B2866" s="19" t="n"/>
@@ -49863,7 +49811,7 @@
       </c>
       <c r="B2869" s="21" t="inlineStr">
         <is>
-          <t>EUS-47015</t>
+          <t>EUS-71187</t>
         </is>
       </c>
       <c r="C2869" s="22" t="n"/>
@@ -50026,7 +49974,7 @@
     <row r="2881" ht="30" customHeight="1">
       <c r="A2881" s="18" t="inlineStr">
         <is>
-          <t>FICHA 193: EUS-18875</t>
+          <t>FICHA 193: EUS-18280</t>
         </is>
       </c>
       <c r="B2881" s="19" t="n"/>
@@ -50075,7 +50023,7 @@
       </c>
       <c r="B2884" s="21" t="inlineStr">
         <is>
-          <t>EUS-18875</t>
+          <t>EUS-18280</t>
         </is>
       </c>
       <c r="C2884" s="22" t="n"/>
@@ -50238,7 +50186,7 @@
     <row r="2896" ht="30" customHeight="1">
       <c r="A2896" s="18" t="inlineStr">
         <is>
-          <t>FICHA 194: EUS-03901</t>
+          <t>FICHA 194: EUS-83528</t>
         </is>
       </c>
       <c r="B2896" s="19" t="n"/>
@@ -50287,7 +50235,7 @@
       </c>
       <c r="B2899" s="21" t="inlineStr">
         <is>
-          <t>EUS-03901</t>
+          <t>EUS-83528</t>
         </is>
       </c>
       <c r="C2899" s="22" t="n"/>
@@ -50450,7 +50398,7 @@
     <row r="2911" ht="30" customHeight="1">
       <c r="A2911" s="18" t="inlineStr">
         <is>
-          <t>FICHA 195: EUS-17248</t>
+          <t>FICHA 195: EUS-58263</t>
         </is>
       </c>
       <c r="B2911" s="19" t="n"/>
@@ -50499,7 +50447,7 @@
       </c>
       <c r="B2914" s="21" t="inlineStr">
         <is>
-          <t>EUS-17248</t>
+          <t>EUS-58263</t>
         </is>
       </c>
       <c r="C2914" s="22" t="n"/>
@@ -50662,7 +50610,7 @@
     <row r="2926" ht="30" customHeight="1">
       <c r="A2926" s="18" t="inlineStr">
         <is>
-          <t>FICHA 196: EUS-36047</t>
+          <t>FICHA 196: EUS-37780</t>
         </is>
       </c>
       <c r="B2926" s="19" t="n"/>
@@ -50711,7 +50659,7 @@
       </c>
       <c r="B2929" s="21" t="inlineStr">
         <is>
-          <t>EUS-36047</t>
+          <t>EUS-37780</t>
         </is>
       </c>
       <c r="C2929" s="22" t="n"/>
@@ -50874,7 +50822,7 @@
     <row r="2941" ht="30" customHeight="1">
       <c r="A2941" s="18" t="inlineStr">
         <is>
-          <t>FICHA 197: EUS-38592</t>
+          <t>FICHA 197: EUS-87782</t>
         </is>
       </c>
       <c r="B2941" s="19" t="n"/>
@@ -50907,7 +50855,7 @@
       </c>
       <c r="B2943" s="21" t="inlineStr">
         <is>
-          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino 1800 natural,para mobiliario urbano. (pto 21036009)</t>
+          <t>Servicio de limpieza a prestar en las instalaciones del CENTRO DE DESARROLLO EMPRESARIAL DE LA MARGEN IZQUIERDA, S.A. (BIC BIZKAIA EZKERRALDEA) sitas en 48901 Barakaldo (Bizkaia), Avda. Altos Hornos d</t>
         </is>
       </c>
       <c r="C2943" s="22" t="n"/>
@@ -50923,7 +50871,7 @@
       </c>
       <c r="B2944" s="21" t="inlineStr">
         <is>
-          <t>EUS-38592</t>
+          <t>EUS-87782</t>
         </is>
       </c>
       <c r="C2944" s="22" t="n"/>
@@ -51075,7 +51023,7 @@
       </c>
       <c r="B2954" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/o-pto-21036009-suministro-bancos-modelo-neobarcino-1800-natural-mobiliario-urbano-pto-21036009/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-prestar-instalaciones-del-centro-desarrollo-empresarial-margen-izquierda-s-bic-bizkaia-ezkerraldea-sitas-48901-barakaldo-bizkaia-avda-altos-hornos-vizcaya-33/expjaso740813/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2954" s="22" t="n"/>
@@ -51086,7 +51034,7 @@
     <row r="2956" ht="30" customHeight="1">
       <c r="A2956" s="18" t="inlineStr">
         <is>
-          <t>FICHA 198: EUS-51365</t>
+          <t>FICHA 198: EUS-48229</t>
         </is>
       </c>
       <c r="B2956" s="19" t="n"/>
@@ -51111,7 +51059,7 @@
       <c r="E2957" s="22" t="n"/>
       <c r="F2957" s="22" t="n"/>
     </row>
-    <row r="2958" ht="20" customHeight="1">
+    <row r="2958" ht="45" customHeight="1">
       <c r="A2958" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -51119,7 +51067,7 @@
       </c>
       <c r="B2958" s="21" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de proyector digital para el Zornotza Aretoa</t>
+          <t>Servicio de mantenimiento integral del edificio e instalaciones de Azkuna Zentroa</t>
         </is>
       </c>
       <c r="C2958" s="22" t="n"/>
@@ -51135,7 +51083,7 @@
       </c>
       <c r="B2959" s="21" t="inlineStr">
         <is>
-          <t>EUS-51365</t>
+          <t>EUS-48229</t>
         </is>
       </c>
       <c r="C2959" s="22" t="n"/>
@@ -51287,7 +51235,7 @@
       </c>
       <c r="B2969" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-alquiler-proyector-digital-zornotza-aretoa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-mantenimiento-integral-del-edificio-e-instalaciones-azkuna-zentroa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2969" s="22" t="n"/>
@@ -51298,7 +51246,7 @@
     <row r="2971" ht="30" customHeight="1">
       <c r="A2971" s="18" t="inlineStr">
         <is>
-          <t>FICHA 199: EUS-28575</t>
+          <t>FICHA 199: EUS-84876</t>
         </is>
       </c>
       <c r="B2971" s="19" t="n"/>
@@ -51331,7 +51279,7 @@
       </c>
       <c r="B2973" s="21" t="inlineStr">
         <is>
-          <t>Suministro, colocación, integración y puesta en marcha de equipos de los sistemas de seguridad del edificio Koldo Mitxelena.</t>
+          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino 1800 natural,para mobiliario urbano. (pto 21036009)</t>
         </is>
       </c>
       <c r="C2973" s="22" t="n"/>
@@ -51347,7 +51295,7 @@
       </c>
       <c r="B2974" s="21" t="inlineStr">
         <is>
-          <t>EUS-28575</t>
+          <t>EUS-84876</t>
         </is>
       </c>
       <c r="C2974" s="22" t="n"/>
@@ -51499,7 +51447,7 @@
       </c>
       <c r="B2984" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-colocacion-integracion-y-puesta-marcha-equipos-sistemas-seguridad-del-edificio-koldo-mitxelena/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/o-pto-21036009-suministro-bancos-modelo-neobarcino-1800-natural-mobiliario-urbano-pto-21036009/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2984" s="22" t="n"/>
@@ -51510,7 +51458,7 @@
     <row r="2986" ht="30" customHeight="1">
       <c r="A2986" s="18" t="inlineStr">
         <is>
-          <t>FICHA 200: EUS-74130</t>
+          <t>FICHA 200: EUS-51515</t>
         </is>
       </c>
       <c r="B2986" s="19" t="n"/>
@@ -51535,7 +51483,7 @@
       <c r="E2987" s="22" t="n"/>
       <c r="F2987" s="22" t="n"/>
     </row>
-    <row r="2988" ht="45" customHeight="1">
+    <row r="2988" ht="20" customHeight="1">
       <c r="A2988" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -51543,7 +51491,7 @@
       </c>
       <c r="B2988" s="21" t="inlineStr">
         <is>
-          <t>Levantamiento Topográfico de la Red de saneamiento y pluviales, así como inventario de arquetas del conjunto edificado del Hospital Universitario Donostia</t>
+          <t>Servicio de alquiler de proyector digital para el Zornotza Aretoa</t>
         </is>
       </c>
       <c r="C2988" s="22" t="n"/>
@@ -51559,7 +51507,7 @@
       </c>
       <c r="B2989" s="21" t="inlineStr">
         <is>
-          <t>EUS-74130</t>
+          <t>EUS-51515</t>
         </is>
       </c>
       <c r="C2989" s="22" t="n"/>
@@ -51711,7 +51659,7 @@
       </c>
       <c r="B2999" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/levantamiento-topografico-red-saneamiento-y-pluviales-asi-como-inventario-arquetas-del-conjunto-edificado-del-hospital-universitario-donostia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-alquiler-proyector-digital-zornotza-aretoa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2999" s="22" t="n"/>
@@ -51722,7 +51670,7 @@
     <row r="3001" ht="30" customHeight="1">
       <c r="A3001" s="18" t="inlineStr">
         <is>
-          <t>FICHA 201: EUS-74639</t>
+          <t>FICHA 201: EUS-20770</t>
         </is>
       </c>
       <c r="B3001" s="19" t="n"/>
@@ -51755,7 +51703,7 @@
       </c>
       <c r="B3003" s="21" t="inlineStr">
         <is>
-          <t>Obras de adecuación a la protección contra incendios en el Edificio Anexo del Hospital de Leza</t>
+          <t>Suministro, colocación, integración y puesta en marcha de equipos de los sistemas de seguridad del edificio Koldo Mitxelena.</t>
         </is>
       </c>
       <c r="C3003" s="22" t="n"/>
@@ -51771,7 +51719,7 @@
       </c>
       <c r="B3004" s="21" t="inlineStr">
         <is>
-          <t>EUS-74639</t>
+          <t>EUS-20770</t>
         </is>
       </c>
       <c r="C3004" s="22" t="n"/>
@@ -51923,7 +51871,7 @@
       </c>
       <c r="B3014" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/obras-adecuacion-proteccion-incendios-edificio-anexo-del-hospital-leza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-colocacion-integracion-y-puesta-marcha-equipos-sistemas-seguridad-del-edificio-koldo-mitxelena/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3014" s="22" t="n"/>
@@ -51934,7 +51882,7 @@
     <row r="3016" ht="30" customHeight="1">
       <c r="A3016" s="18" t="inlineStr">
         <is>
-          <t>FICHA 202: EUS-61809</t>
+          <t>FICHA 202: EUS-12021</t>
         </is>
       </c>
       <c r="B3016" s="19" t="n"/>
@@ -51959,7 +51907,7 @@
       <c r="E3017" s="22" t="n"/>
       <c r="F3017" s="22" t="n"/>
     </row>
-    <row r="3018" ht="20" customHeight="1">
+    <row r="3018" ht="45" customHeight="1">
       <c r="A3018" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -51967,7 +51915,7 @@
       </c>
       <c r="B3018" s="21" t="inlineStr">
         <is>
-          <t>Transporte adaptado alumna.</t>
+          <t>Levantamiento Topográfico de la Red de saneamiento y pluviales, así como inventario de arquetas del conjunto edificado del Hospital Universitario Donostia</t>
         </is>
       </c>
       <c r="C3018" s="22" t="n"/>
@@ -51983,7 +51931,7 @@
       </c>
       <c r="B3019" s="21" t="inlineStr">
         <is>
-          <t>EUS-61809</t>
+          <t>EUS-12021</t>
         </is>
       </c>
       <c r="C3019" s="22" t="n"/>
@@ -52135,7 +52083,7 @@
       </c>
       <c r="B3029" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-adaptado-alumna/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/levantamiento-topografico-red-saneamiento-y-pluviales-asi-como-inventario-arquetas-del-conjunto-edificado-del-hospital-universitario-donostia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3029" s="22" t="n"/>
@@ -52143,220 +52091,8 @@
       <c r="E3029" s="22" t="n"/>
       <c r="F3029" s="22" t="n"/>
     </row>
-    <row r="3031" ht="30" customHeight="1">
-      <c r="A3031" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 203: EUS-93696</t>
-        </is>
-      </c>
-      <c r="B3031" s="19" t="n"/>
-      <c r="C3031" s="19" t="n"/>
-      <c r="D3031" s="19" t="n"/>
-      <c r="E3031" s="19" t="n"/>
-      <c r="F3031" s="19" t="n"/>
-    </row>
-    <row r="3032" ht="20" customHeight="1">
-      <c r="A3032" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B3032" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C3032" s="22" t="n"/>
-      <c r="D3032" s="22" t="n"/>
-      <c r="E3032" s="22" t="n"/>
-      <c r="F3032" s="22" t="n"/>
-    </row>
-    <row r="3033" ht="20" customHeight="1">
-      <c r="A3033" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B3033" s="21" t="inlineStr">
-        <is>
-          <t>Instalación paneles solares 10% instalación legalización</t>
-        </is>
-      </c>
-      <c r="C3033" s="22" t="n"/>
-      <c r="D3033" s="22" t="n"/>
-      <c r="E3033" s="22" t="n"/>
-      <c r="F3033" s="22" t="n"/>
-    </row>
-    <row r="3034" ht="20" customHeight="1">
-      <c r="A3034" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3034" s="21" t="inlineStr">
-        <is>
-          <t>EUS-93696</t>
-        </is>
-      </c>
-      <c r="C3034" s="22" t="n"/>
-      <c r="D3034" s="22" t="n"/>
-      <c r="E3034" s="22" t="n"/>
-      <c r="F3034" s="22" t="n"/>
-    </row>
-    <row r="3035" ht="20" customHeight="1">
-      <c r="A3035" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B3035" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C3035" s="22" t="n"/>
-      <c r="D3035" s="22" t="n"/>
-      <c r="E3035" s="22" t="n"/>
-      <c r="F3035" s="22" t="n"/>
-    </row>
-    <row r="3036" ht="20" customHeight="1">
-      <c r="A3036" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B3036" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C3036" s="22" t="n"/>
-      <c r="D3036" s="22" t="n"/>
-      <c r="E3036" s="22" t="n"/>
-      <c r="F3036" s="22" t="n"/>
-    </row>
-    <row r="3037" ht="20" customHeight="1">
-      <c r="A3037" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B3037" s="21" t="inlineStr"/>
-      <c r="C3037" s="22" t="n"/>
-      <c r="D3037" s="22" t="n"/>
-      <c r="E3037" s="22" t="n"/>
-      <c r="F3037" s="22" t="n"/>
-    </row>
-    <row r="3038" ht="20" customHeight="1">
-      <c r="A3038" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B3038" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C3038" s="22" t="n"/>
-      <c r="D3038" s="22" t="n"/>
-      <c r="E3038" s="22" t="n"/>
-      <c r="F3038" s="22" t="n"/>
-    </row>
-    <row r="3039" ht="20" customHeight="1">
-      <c r="A3039" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B3039" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C3039" s="22" t="n"/>
-      <c r="D3039" s="22" t="n"/>
-      <c r="E3039" s="22" t="n"/>
-      <c r="F3039" s="22" t="n"/>
-    </row>
-    <row r="3040" ht="20" customHeight="1">
-      <c r="A3040" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B3040" s="21" t="inlineStr"/>
-      <c r="C3040" s="22" t="n"/>
-      <c r="D3040" s="22" t="n"/>
-      <c r="E3040" s="22" t="n"/>
-      <c r="F3040" s="22" t="n"/>
-    </row>
-    <row r="3041" ht="20" customHeight="1">
-      <c r="A3041" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B3041" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C3041" s="22" t="n"/>
-      <c r="D3041" s="22" t="n"/>
-      <c r="E3041" s="22" t="n"/>
-      <c r="F3041" s="22" t="n"/>
-    </row>
-    <row r="3042" ht="20" customHeight="1">
-      <c r="A3042" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B3042" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C3042" s="22" t="n"/>
-      <c r="D3042" s="22" t="n"/>
-      <c r="E3042" s="22" t="n"/>
-      <c r="F3042" s="22" t="n"/>
-    </row>
-    <row r="3043" ht="20" customHeight="1">
-      <c r="A3043" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B3043" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C3043" s="22" t="n"/>
-      <c r="D3043" s="22" t="n"/>
-      <c r="E3043" s="22" t="n"/>
-      <c r="F3043" s="22" t="n"/>
-    </row>
-    <row r="3044" ht="45" customHeight="1">
-      <c r="A3044" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B3044" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/instalacion-paneles-solares-10-instalacion-legalizacion/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C3044" s="22" t="n"/>
-      <c r="D3044" s="22" t="n"/>
-      <c r="E3044" s="22" t="n"/>
-      <c r="F3044" s="22" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="2842">
+  <mergeCells count="2828">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B2192:F2192"/>
     <mergeCell ref="B1765:F1765"/>
@@ -52817,9 +52553,7 @@
     <mergeCell ref="B921:F921"/>
     <mergeCell ref="B606:F606"/>
     <mergeCell ref="B2741:F2741"/>
-    <mergeCell ref="B3039:F3039"/>
     <mergeCell ref="B2007:F2007"/>
-    <mergeCell ref="B3033:F3033"/>
     <mergeCell ref="B2436:F2436"/>
     <mergeCell ref="A1276:F1276"/>
     <mergeCell ref="B2770:F2770"/>
@@ -53018,7 +52752,6 @@
     <mergeCell ref="A2731:F2731"/>
     <mergeCell ref="B2246:F2246"/>
     <mergeCell ref="A946:F946"/>
-    <mergeCell ref="A3031:F3031"/>
     <mergeCell ref="A631:F631"/>
     <mergeCell ref="B117:F117"/>
     <mergeCell ref="B1783:F1783"/>
@@ -53096,7 +52829,6 @@
     <mergeCell ref="B2155:F2155"/>
     <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B368:F368"/>
-    <mergeCell ref="B3041:F3041"/>
     <mergeCell ref="B1254:F1254"/>
     <mergeCell ref="B1430:F1430"/>
     <mergeCell ref="B1552:F1552"/>
@@ -53279,7 +53011,6 @@
     <mergeCell ref="B1304:F1304"/>
     <mergeCell ref="B1608:F1608"/>
     <mergeCell ref="B2695:F2695"/>
-    <mergeCell ref="B3037:F3037"/>
     <mergeCell ref="B1967:F1967"/>
     <mergeCell ref="B908:F908"/>
     <mergeCell ref="B883:F883"/>
@@ -53728,7 +53459,6 @@
     <mergeCell ref="A2491:F2491"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
-    <mergeCell ref="B3036:F3036"/>
     <mergeCell ref="B1249:F1249"/>
     <mergeCell ref="B524:F524"/>
     <mergeCell ref="B1854:F1854"/>
@@ -53736,7 +53466,6 @@
     <mergeCell ref="B67:F67"/>
     <mergeCell ref="B2012:F2012"/>
     <mergeCell ref="B953:F953"/>
-    <mergeCell ref="B3038:F3038"/>
     <mergeCell ref="B1251:F1251"/>
     <mergeCell ref="B1549:F1549"/>
     <mergeCell ref="B1856:F1856"/>
@@ -53822,7 +53551,6 @@
     <mergeCell ref="B891:F891"/>
     <mergeCell ref="B3009:F3009"/>
     <mergeCell ref="B1191:F1191"/>
-    <mergeCell ref="B3034:F3034"/>
     <mergeCell ref="B609:F609"/>
     <mergeCell ref="B1247:F1247"/>
     <mergeCell ref="B1977:F1977"/>
@@ -53840,7 +53568,6 @@
     <mergeCell ref="B1547:F1547"/>
     <mergeCell ref="B1207:F1207"/>
     <mergeCell ref="B490:F490"/>
-    <mergeCell ref="B3035:F3035"/>
     <mergeCell ref="B1338:F1338"/>
     <mergeCell ref="B3029:F3029"/>
     <mergeCell ref="B604:F604"/>
@@ -54443,7 +54170,6 @@
     <mergeCell ref="B1315:F1315"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B2377:F2377"/>
-    <mergeCell ref="B3042:F3042"/>
     <mergeCell ref="B1649:F1649"/>
     <mergeCell ref="B590:F590"/>
     <mergeCell ref="B888:F888"/>
@@ -54467,7 +54193,6 @@
     <mergeCell ref="B512:F512"/>
     <mergeCell ref="B2734:F2734"/>
     <mergeCell ref="B2728:F2728"/>
-    <mergeCell ref="B3032:F3032"/>
     <mergeCell ref="B2000:F2000"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="B941:F941"/>
@@ -54907,7 +54632,6 @@
     <mergeCell ref="B318:F318"/>
     <mergeCell ref="A1741:F1741"/>
     <mergeCell ref="B1098:F1098"/>
-    <mergeCell ref="B3043:F3043"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B1256:F1256"/>
@@ -54927,7 +54651,6 @@
     <mergeCell ref="B1562:F1562"/>
     <mergeCell ref="B2317:F2317"/>
     <mergeCell ref="B1556:F1556"/>
-    <mergeCell ref="B3044:F3044"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
@@ -55027,7 +54750,6 @@
     <mergeCell ref="B197:F197"/>
     <mergeCell ref="B2104:F2104"/>
     <mergeCell ref="B153:F153"/>
-    <mergeCell ref="B3040:F3040"/>
     <mergeCell ref="B1343:F1343"/>
     <mergeCell ref="B1641:F1641"/>
     <mergeCell ref="B2315:F2315"/>
@@ -55403,7 +55125,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2999" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3014" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3029" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3044" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -55415,7 +55136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J204"/>
+  <dimension ref="A1:J203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -61633,7 +61354,7 @@
     <row r="193" ht="28" customHeight="1">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>EUS-47015</t>
+          <t>EUS-71187</t>
         </is>
       </c>
       <c r="B193" s="6" t="inlineStr">
@@ -61669,7 +61390,7 @@
     <row r="194" ht="28" customHeight="1">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>EUS-18875</t>
+          <t>EUS-18280</t>
         </is>
       </c>
       <c r="B194" s="6" t="inlineStr">
@@ -61705,7 +61426,7 @@
     <row r="195" ht="28" customHeight="1">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>EUS-03901</t>
+          <t>EUS-83528</t>
         </is>
       </c>
       <c r="B195" s="6" t="inlineStr">
@@ -61741,7 +61462,7 @@
     <row r="196" ht="28" customHeight="1">
       <c r="A196" s="6" t="inlineStr">
         <is>
-          <t>EUS-17248</t>
+          <t>EUS-58263</t>
         </is>
       </c>
       <c r="B196" s="6" t="inlineStr">
@@ -61777,7 +61498,7 @@
     <row r="197" ht="28" customHeight="1">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>EUS-36047</t>
+          <t>EUS-37780</t>
         </is>
       </c>
       <c r="B197" s="6" t="inlineStr">
@@ -61813,12 +61534,12 @@
     <row r="198" ht="28" customHeight="1">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>EUS-38592</t>
+          <t>EUS-87782</t>
         </is>
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino</t>
+          <t>Servicio de limpieza a prestar en las instalaciones del CENT</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
@@ -61849,12 +61570,12 @@
     <row r="199" ht="28" customHeight="1">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>EUS-51365</t>
+          <t>EUS-48229</t>
         </is>
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>Servicio de alquiler de proyector digital para el Zornotza A</t>
+          <t>Servicio de mantenimiento integral del edificio e instalacio</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
@@ -61885,12 +61606,12 @@
     <row r="200" ht="28" customHeight="1">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>EUS-28575</t>
+          <t>EUS-84876</t>
         </is>
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t>Suministro, colocación, integración y puesta en marcha de eq</t>
+          <t>O. (pto 21036009); ; suministro de bancos ,modelo neobarcino</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
@@ -61921,12 +61642,12 @@
     <row r="201" ht="28" customHeight="1">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>EUS-74130</t>
+          <t>EUS-51515</t>
         </is>
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>Levantamiento Topográfico de la Red de saneamiento y pluvial</t>
+          <t>Servicio de alquiler de proyector digital para el Zornotza A</t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
@@ -61957,12 +61678,12 @@
     <row r="202" ht="28" customHeight="1">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>EUS-74639</t>
+          <t>EUS-20770</t>
         </is>
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>Obras de adecuación a la protección contra incendios en el E</t>
+          <t>Suministro, colocación, integración y puesta en marcha de eq</t>
         </is>
       </c>
       <c r="C202" s="6" t="inlineStr">
@@ -61993,12 +61714,12 @@
     <row r="203" ht="28" customHeight="1">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>EUS-61809</t>
+          <t>EUS-12021</t>
         </is>
       </c>
       <c r="B203" s="6" t="inlineStr">
         <is>
-          <t>Transporte adaptado alumna.</t>
+          <t>Levantamiento Topográfico de la Red de saneamiento y pluvial</t>
         </is>
       </c>
       <c r="C203" s="6" t="inlineStr">
@@ -62026,44 +61747,8 @@
       <c r="I203" s="6" t="inlineStr"/>
       <c r="J203" s="6" t="inlineStr"/>
     </row>
-    <row r="204" ht="28" customHeight="1">
-      <c r="A204" s="6" t="inlineStr">
-        <is>
-          <t>EUS-93696</t>
-        </is>
-      </c>
-      <c r="B204" s="6" t="inlineStr">
-        <is>
-          <t>Instalación paneles solares 10% instalación legalización</t>
-        </is>
-      </c>
-      <c r="C204" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D204" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E204" s="6" t="inlineStr"/>
-      <c r="F204" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G204" s="6" t="inlineStr"/>
-      <c r="H204" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I204" s="6" t="inlineStr"/>
-      <c r="J204" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J204"/>
+  <autoFilter ref="A1:J203"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-10-06
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$191</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M191"/>
+  <dimension ref="A1:M190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 05/10/2026 12:49 - 185 convocatorias - 11 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 06/10/2026 12:18 - 184 convocatorias - 10 nuevas</t>
         </is>
       </c>
     </row>
@@ -3341,19 +3341,15 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr"/>
       <c r="E60" s="10" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -3374,7 +3370,7 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr"/>
@@ -3392,15 +3388,19 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="inlineStr"/>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -4007,12 +4007,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr"/>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr"/>
@@ -4054,12 +4054,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -4101,12 +4101,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr"/>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="L76" s="6" t="inlineStr"/>
@@ -4148,12 +4148,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr"/>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr"/>
@@ -6968,12 +6968,12 @@
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>925388828</t>
+          <t>934294980</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>THOMSON POWER EUROPE LTD</t>
+          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr"/>
@@ -6997,7 +6997,7 @@
       </c>
       <c r="K137" s="6" t="inlineStr">
         <is>
-          <t>THOMSON POWER EUROPE LTD</t>
+          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
         </is>
       </c>
       <c r="L137" s="6" t="inlineStr"/>
@@ -7015,12 +7015,12 @@
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>934294980</t>
+          <t>925388828</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
+          <t>THOMSON POWER EUROPE LTD</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr"/>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="K138" s="6" t="inlineStr">
         <is>
-          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
+          <t>THOMSON POWER EUROPE LTD</t>
         </is>
       </c>
       <c r="L138" s="6" t="inlineStr"/>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="B181" s="6" t="inlineStr">
         <is>
-          <t>EUS-43735</t>
+          <t>EUS-47596</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>EUS-23831</t>
+          <t>EUS-51067</t>
         </is>
       </c>
       <c r="C182" s="6" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="B183" s="6" t="inlineStr">
         <is>
-          <t>EUS-89429</t>
+          <t>EUS-92303</t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>Licitación, mediante procedimiento negociado sin publicidad, para la contratación de servicios de creación y edición de obra literaria y su divulgación para la Asociación BC3 Basque Centre for Climate</t>
+          <t>Servicio de retirada, transporte y gestión de los residuos Sandach de la cámara frigorífica situada en el Garbigune de Eibar</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
@@ -9161,12 +9161,12 @@
       </c>
       <c r="B184" s="6" t="inlineStr">
         <is>
-          <t>EUS-69995</t>
+          <t>EUS-86597</t>
         </is>
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
+          <t>Rehabilitacion parrales del barrio San Bartolome (zona Bizezko)</t>
         </is>
       </c>
       <c r="D184" s="6" t="inlineStr">
@@ -9183,12 +9183,12 @@
       <c r="G184" s="6" t="inlineStr"/>
       <c r="H184" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I184" s="11" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J184" s="6" t="inlineStr"/>
@@ -9216,12 +9216,12 @@
       </c>
       <c r="B185" s="6" t="inlineStr">
         <is>
-          <t>EUS-59844</t>
+          <t>EUS-60193</t>
         </is>
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
         </is>
       </c>
       <c r="D185" s="6" t="inlineStr">
@@ -9271,12 +9271,12 @@
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>EUS-33760</t>
+          <t>EUS-65298</t>
         </is>
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>Aprobar la contratación de los trabajos de "Integración de levantamientos topográficos en la base topográfica urbana de Álava", como contrato menor de servicios.</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="D186" s="6" t="inlineStr">
@@ -9293,7 +9293,7 @@
       <c r="G186" s="6" t="inlineStr"/>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I186" s="11" t="inlineStr">
@@ -9326,12 +9326,12 @@
       </c>
       <c r="B187" s="6" t="inlineStr">
         <is>
-          <t>EUS-93831</t>
+          <t>EUS-77322</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Contratación del servicio de asistencia técnica y gestión de venta de los ahorros energéticos generados por la empresa de Transporte Urbano de Vitoria-Gasteiz (TUVISA)</t>
+          <t>Redacción del proyecto y dirección de las obras de renovación de la red de distribución de agua en distintas zonas del centro de Irun</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
@@ -9381,12 +9381,12 @@
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>EUS-16126</t>
+          <t>EUS-36090</t>
         </is>
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>Obras del proyecto de construcción de itinerario peatonal paralelo a la calzada entre los PK 1,810 y 2,030 de la  GI-3131 a Goroeta en Aretxabaleta (14-SV-79/2025 2LIC)</t>
+          <t>Obras de rehabilitación del edificio del Emisario submarino de Monpas</t>
         </is>
       </c>
       <c r="D188" s="6" t="inlineStr">
@@ -9436,12 +9436,12 @@
       </c>
       <c r="B189" s="6" t="inlineStr">
         <is>
-          <t>EUS-08987</t>
+          <t>EUS-09001</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>reparación y puesta en servicio de red de fecales y pluviales en el centro CEIP Cantarrana Eskola HLHI</t>
+          <t>Servicio para la elaboración de un estudio medioambiental de la zona costera de Mompás y del estuario del río Oiartzun</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
@@ -9491,12 +9491,12 @@
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>EUS-71383</t>
+          <t>EUS-57679</t>
         </is>
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>Suministro e instalación de un portón industrial enrollable para el edificio AIC Ermua</t>
+          <t>Plan de comunicacion y Sistema de Portavocias de la Agencia Vasca del Agua</t>
         </is>
       </c>
       <c r="D190" s="6" t="inlineStr">
@@ -9538,63 +9538,8 @@
         </is>
       </c>
     </row>
-    <row r="191" ht="40" customHeight="1">
-      <c r="A191" s="14" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B191" s="6" t="inlineStr">
-        <is>
-          <t>EUS-06475</t>
-        </is>
-      </c>
-      <c r="C191" s="6" t="inlineStr">
-        <is>
-          <t>ANS para determinadas aplicaciones implementadas por Izfe para el Departamento de Equilibrio Territorial Verde de la GFA-DFG para la gestión de la identificación, registro, saneamiento y movimiento an</t>
-        </is>
-      </c>
-      <c r="D191" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E191" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F191" s="6" t="inlineStr"/>
-      <c r="G191" s="6" t="inlineStr"/>
-      <c r="H191" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I191" s="11" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J191" s="6" t="inlineStr"/>
-      <c r="K191" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L191" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M191" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M191"/>
+  <autoFilter ref="A4:M190"/>
   <mergeCells count="4">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A180:M180"/>
@@ -9786,7 +9731,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId185"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9798,7 +9742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2774"/>
+  <dimension ref="A1:F2759"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20912,7 +20856,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="16" t="inlineStr">
         <is>
-          <t>FICHA 55: HORIZON</t>
+          <t>FICHA 55: ERASMUS2027</t>
         </is>
       </c>
       <c r="B811" s="17" t="n"/>
@@ -20945,7 +20889,7 @@
       </c>
       <c r="B813" s="19" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="C813" s="20" t="n"/>
@@ -20961,7 +20905,7 @@
       </c>
       <c r="B814" s="19" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="C814" s="20" t="n"/>
@@ -20975,11 +20919,7 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B815" s="19" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+      <c r="B815" s="19" t="inlineStr"/>
       <c r="C815" s="20" t="n"/>
       <c r="D815" s="20" t="n"/>
       <c r="E815" s="20" t="n"/>
@@ -21053,7 +20993,7 @@
       </c>
       <c r="B820" s="19" t="inlineStr">
         <is>
-          <t>HORIZON-MISS-2021-CIT-02</t>
+          <t>ERASMUS-EDU-2022-PI-ALL-INNO</t>
         </is>
       </c>
       <c r="C820" s="20" t="n"/>
@@ -21069,7 +21009,7 @@
       </c>
       <c r="B821" s="19" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="C821" s="20" t="n"/>
@@ -21113,7 +21053,7 @@
       </c>
       <c r="B824" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/ERASMUS2027</t>
         </is>
       </c>
       <c r="C824" s="20" t="n"/>
@@ -21124,7 +21064,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="16" t="inlineStr">
         <is>
-          <t>FICHA 56: ERASMUS2027</t>
+          <t>FICHA 56: HORIZON</t>
         </is>
       </c>
       <c r="B826" s="17" t="n"/>
@@ -21157,7 +21097,7 @@
       </c>
       <c r="B828" s="19" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="C828" s="20" t="n"/>
@@ -21173,7 +21113,7 @@
       </c>
       <c r="B829" s="19" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="C829" s="20" t="n"/>
@@ -21187,7 +21127,11 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B830" s="19" t="inlineStr"/>
+      <c r="B830" s="19" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="C830" s="20" t="n"/>
       <c r="D830" s="20" t="n"/>
       <c r="E830" s="20" t="n"/>
@@ -21261,7 +21205,7 @@
       </c>
       <c r="B835" s="19" t="inlineStr">
         <is>
-          <t>ERASMUS-EDU-2022-PI-ALL-INNO</t>
+          <t>HORIZON-MISS-2021-CIT-02</t>
         </is>
       </c>
       <c r="C835" s="20" t="n"/>
@@ -21277,7 +21221,7 @@
       </c>
       <c r="B836" s="19" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="C836" s="20" t="n"/>
@@ -21321,7 +21265,7 @@
       </c>
       <c r="B839" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/ERASMUS2027</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON</t>
         </is>
       </c>
       <c r="C839" s="20" t="n"/>
@@ -23796,7 +23740,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="16" t="inlineStr">
         <is>
-          <t>FICHA 69: 928447529</t>
+          <t>FICHA 69: 917779760</t>
         </is>
       </c>
       <c r="B1021" s="17" t="n"/>
@@ -23829,7 +23773,7 @@
       </c>
       <c r="B1023" s="19" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C1023" s="20" t="n"/>
@@ -23845,7 +23789,7 @@
       </c>
       <c r="B1024" s="19" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="C1024" s="20" t="n"/>
@@ -23945,7 +23889,7 @@
       </c>
       <c r="B1031" s="19" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C1031" s="20" t="n"/>
@@ -23989,7 +23933,7 @@
       </c>
       <c r="B1034" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928447529</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917779760</t>
         </is>
       </c>
       <c r="C1034" s="20" t="n"/>
@@ -24000,7 +23944,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="16" t="inlineStr">
         <is>
-          <t>FICHA 70: 917671508</t>
+          <t>FICHA 70: 920115617</t>
         </is>
       </c>
       <c r="B1036" s="17" t="n"/>
@@ -24033,7 +23977,7 @@
       </c>
       <c r="B1038" s="19" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C1038" s="20" t="n"/>
@@ -24049,7 +23993,7 @@
       </c>
       <c r="B1039" s="19" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="C1039" s="20" t="n"/>
@@ -24149,7 +24093,7 @@
       </c>
       <c r="B1046" s="19" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C1046" s="20" t="n"/>
@@ -24193,7 +24137,7 @@
       </c>
       <c r="B1049" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917671508</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/920115617</t>
         </is>
       </c>
       <c r="C1049" s="20" t="n"/>
@@ -24204,7 +24148,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="16" t="inlineStr">
         <is>
-          <t>FICHA 71: 917779760</t>
+          <t>FICHA 71: 917671508</t>
         </is>
       </c>
       <c r="B1051" s="17" t="n"/>
@@ -24237,7 +24181,7 @@
       </c>
       <c r="B1053" s="19" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C1053" s="20" t="n"/>
@@ -24253,7 +24197,7 @@
       </c>
       <c r="B1054" s="19" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="C1054" s="20" t="n"/>
@@ -24353,7 +24297,7 @@
       </c>
       <c r="B1061" s="19" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C1061" s="20" t="n"/>
@@ -24397,7 +24341,7 @@
       </c>
       <c r="B1064" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917779760</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917671508</t>
         </is>
       </c>
       <c r="C1064" s="20" t="n"/>
@@ -24408,7 +24352,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: 920115617</t>
+          <t>FICHA 72: 928447529</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -24441,7 +24385,7 @@
       </c>
       <c r="B1068" s="19" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C1068" s="20" t="n"/>
@@ -24457,7 +24401,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -24557,7 +24501,7 @@
       </c>
       <c r="B1076" s="19" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C1076" s="20" t="n"/>
@@ -24601,7 +24545,7 @@
       </c>
       <c r="B1079" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/920115617</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928447529</t>
         </is>
       </c>
       <c r="C1079" s="20" t="n"/>
@@ -36676,7 +36620,7 @@
     <row r="1966" ht="30" customHeight="1">
       <c r="A1966" s="16" t="inlineStr">
         <is>
-          <t>FICHA 132: 925388828</t>
+          <t>FICHA 132: 934294980</t>
         </is>
       </c>
       <c r="B1966" s="17" t="n"/>
@@ -36709,7 +36653,7 @@
       </c>
       <c r="B1968" s="19" t="inlineStr">
         <is>
-          <t>THOMSON POWER EUROPE LTD</t>
+          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
         </is>
       </c>
       <c r="C1968" s="20" t="n"/>
@@ -36725,7 +36669,7 @@
       </c>
       <c r="B1969" s="19" t="inlineStr">
         <is>
-          <t>925388828</t>
+          <t>934294980</t>
         </is>
       </c>
       <c r="C1969" s="20" t="n"/>
@@ -36825,7 +36769,7 @@
       </c>
       <c r="B1976" s="19" t="inlineStr">
         <is>
-          <t>THOMSON POWER EUROPE LTD</t>
+          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
         </is>
       </c>
       <c r="C1976" s="20" t="n"/>
@@ -36869,7 +36813,7 @@
       </c>
       <c r="B1979" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/925388828</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/934294980</t>
         </is>
       </c>
       <c r="C1979" s="20" t="n"/>
@@ -36880,7 +36824,7 @@
     <row r="1981" ht="30" customHeight="1">
       <c r="A1981" s="16" t="inlineStr">
         <is>
-          <t>FICHA 133: 934294980</t>
+          <t>FICHA 133: 925388828</t>
         </is>
       </c>
       <c r="B1981" s="17" t="n"/>
@@ -36913,7 +36857,7 @@
       </c>
       <c r="B1983" s="19" t="inlineStr">
         <is>
-          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
+          <t>THOMSON POWER EUROPE LTD</t>
         </is>
       </c>
       <c r="C1983" s="20" t="n"/>
@@ -36929,7 +36873,7 @@
       </c>
       <c r="B1984" s="19" t="inlineStr">
         <is>
-          <t>934294980</t>
+          <t>925388828</t>
         </is>
       </c>
       <c r="C1984" s="20" t="n"/>
@@ -37029,7 +36973,7 @@
       </c>
       <c r="B1991" s="19" t="inlineStr">
         <is>
-          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
+          <t>THOMSON POWER EUROPE LTD</t>
         </is>
       </c>
       <c r="C1991" s="20" t="n"/>
@@ -37073,7 +37017,7 @@
       </c>
       <c r="B1994" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/934294980</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/925388828</t>
         </is>
       </c>
       <c r="C1994" s="20" t="n"/>
@@ -45460,7 +45404,7 @@
     <row r="2611" ht="30" customHeight="1">
       <c r="A2611" s="16" t="inlineStr">
         <is>
-          <t>FICHA 175: EUS-43735</t>
+          <t>FICHA 175: EUS-47596</t>
         </is>
       </c>
       <c r="B2611" s="17" t="n"/>
@@ -45509,7 +45453,7 @@
       </c>
       <c r="B2614" s="19" t="inlineStr">
         <is>
-          <t>EUS-43735</t>
+          <t>EUS-47596</t>
         </is>
       </c>
       <c r="C2614" s="20" t="n"/>
@@ -45672,7 +45616,7 @@
     <row r="2626" ht="30" customHeight="1">
       <c r="A2626" s="16" t="inlineStr">
         <is>
-          <t>FICHA 176: EUS-23831</t>
+          <t>FICHA 176: EUS-51067</t>
         </is>
       </c>
       <c r="B2626" s="17" t="n"/>
@@ -45721,7 +45665,7 @@
       </c>
       <c r="B2629" s="19" t="inlineStr">
         <is>
-          <t>EUS-23831</t>
+          <t>EUS-51067</t>
         </is>
       </c>
       <c r="C2629" s="20" t="n"/>
@@ -45884,7 +45828,7 @@
     <row r="2641" ht="30" customHeight="1">
       <c r="A2641" s="16" t="inlineStr">
         <is>
-          <t>FICHA 177: EUS-89429</t>
+          <t>FICHA 177: EUS-92303</t>
         </is>
       </c>
       <c r="B2641" s="17" t="n"/>
@@ -45917,7 +45861,7 @@
       </c>
       <c r="B2643" s="19" t="inlineStr">
         <is>
-          <t>Licitación, mediante procedimiento negociado sin publicidad, para la contratación de servicios de creación y edición de obra literaria y su divulgación para la Asociación BC3 Basque Centre for Climate</t>
+          <t>Servicio de retirada, transporte y gestión de los residuos Sandach de la cámara frigorífica situada en el Garbigune de Eibar</t>
         </is>
       </c>
       <c r="C2643" s="20" t="n"/>
@@ -45933,7 +45877,7 @@
       </c>
       <c r="B2644" s="19" t="inlineStr">
         <is>
-          <t>EUS-89429</t>
+          <t>EUS-92303</t>
         </is>
       </c>
       <c r="C2644" s="20" t="n"/>
@@ -46085,7 +46029,7 @@
       </c>
       <c r="B2654" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/licitacion-mediante-procedimiento-negociado-publicidad-contratacion-servicios-creacion-y-edicion-obra-literaria-y-su-divulgacion-asociacion-bc3-basque-centre-for-climate-change-klima-aldaketa-ikergai/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-retirada-transporte-y-gestion-residuos-sandach-camara-frigorifica-situada-garbigune-eibar/expjaso743728/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2654" s="20" t="n"/>
@@ -46096,7 +46040,7 @@
     <row r="2656" ht="30" customHeight="1">
       <c r="A2656" s="16" t="inlineStr">
         <is>
-          <t>FICHA 178: EUS-69995</t>
+          <t>FICHA 178: EUS-86597</t>
         </is>
       </c>
       <c r="B2656" s="17" t="n"/>
@@ -46121,7 +46065,7 @@
       <c r="E2657" s="20" t="n"/>
       <c r="F2657" s="20" t="n"/>
     </row>
-    <row r="2658" ht="45" customHeight="1">
+    <row r="2658" ht="20" customHeight="1">
       <c r="A2658" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -46129,7 +46073,7 @@
       </c>
       <c r="B2658" s="19" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
+          <t>Rehabilitacion parrales del barrio San Bartolome (zona Bizezko)</t>
         </is>
       </c>
       <c r="C2658" s="20" t="n"/>
@@ -46145,7 +46089,7 @@
       </c>
       <c r="B2659" s="19" t="inlineStr">
         <is>
-          <t>EUS-69995</t>
+          <t>EUS-86597</t>
         </is>
       </c>
       <c r="C2659" s="20" t="n"/>
@@ -46221,7 +46165,7 @@
       </c>
       <c r="B2664" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C2664" s="20" t="n"/>
@@ -46279,9 +46223,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B2668" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B2668" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C2668" s="20" t="n"/>
@@ -46297,7 +46241,7 @@
       </c>
       <c r="B2669" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/bioaniztasunfundaziohirin/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/rehabilitacion-parrales-del-barrio-san-bartolome-zona-bizezko/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2669" s="20" t="n"/>
@@ -46308,7 +46252,7 @@
     <row r="2671" ht="30" customHeight="1">
       <c r="A2671" s="16" t="inlineStr">
         <is>
-          <t>FICHA 179: EUS-59844</t>
+          <t>FICHA 179: EUS-60193</t>
         </is>
       </c>
       <c r="B2671" s="17" t="n"/>
@@ -46333,7 +46277,7 @@
       <c r="E2672" s="20" t="n"/>
       <c r="F2672" s="20" t="n"/>
     </row>
-    <row r="2673" ht="20" customHeight="1">
+    <row r="2673" ht="45" customHeight="1">
       <c r="A2673" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -46341,7 +46285,7 @@
       </c>
       <c r="B2673" s="19" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
         </is>
       </c>
       <c r="C2673" s="20" t="n"/>
@@ -46357,7 +46301,7 @@
       </c>
       <c r="B2674" s="19" t="inlineStr">
         <is>
-          <t>EUS-59844</t>
+          <t>EUS-60193</t>
         </is>
       </c>
       <c r="C2674" s="20" t="n"/>
@@ -46509,7 +46453,7 @@
       </c>
       <c r="B2684" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/comunicacion-previs-digitalizacion-2027/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/bioaniztasunfundaziohirin/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2684" s="20" t="n"/>
@@ -46520,7 +46464,7 @@
     <row r="2686" ht="30" customHeight="1">
       <c r="A2686" s="16" t="inlineStr">
         <is>
-          <t>FICHA 180: EUS-33760</t>
+          <t>FICHA 180: EUS-65298</t>
         </is>
       </c>
       <c r="B2686" s="17" t="n"/>
@@ -46545,7 +46489,7 @@
       <c r="E2687" s="20" t="n"/>
       <c r="F2687" s="20" t="n"/>
     </row>
-    <row r="2688" ht="45" customHeight="1">
+    <row r="2688" ht="20" customHeight="1">
       <c r="A2688" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -46553,7 +46497,7 @@
       </c>
       <c r="B2688" s="19" t="inlineStr">
         <is>
-          <t>Aprobar la contratación de los trabajos de "Integración de levantamientos topográficos en la base topográfica urbana de Álava", como contrato menor de servicios.</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="C2688" s="20" t="n"/>
@@ -46569,7 +46513,7 @@
       </c>
       <c r="B2689" s="19" t="inlineStr">
         <is>
-          <t>EUS-33760</t>
+          <t>EUS-65298</t>
         </is>
       </c>
       <c r="C2689" s="20" t="n"/>
@@ -46645,7 +46589,7 @@
       </c>
       <c r="B2694" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C2694" s="20" t="n"/>
@@ -46721,7 +46665,7 @@
       </c>
       <c r="B2699" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/aprobar-contratacion-trabajos-integracion-levantamientos-topograficos-base-topografica-urbana-alava-como-contrato-menor-servicios/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/comunicacion-previs-digitalizacion-2027/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2699" s="20" t="n"/>
@@ -46732,7 +46676,7 @@
     <row r="2701" ht="30" customHeight="1">
       <c r="A2701" s="16" t="inlineStr">
         <is>
-          <t>FICHA 181: EUS-93831</t>
+          <t>FICHA 181: EUS-77322</t>
         </is>
       </c>
       <c r="B2701" s="17" t="n"/>
@@ -46765,7 +46709,7 @@
       </c>
       <c r="B2703" s="19" t="inlineStr">
         <is>
-          <t>Contratación del servicio de asistencia técnica y gestión de venta de los ahorros energéticos generados por la empresa de Transporte Urbano de Vitoria-Gasteiz (TUVISA)</t>
+          <t>Redacción del proyecto y dirección de las obras de renovación de la red de distribución de agua en distintas zonas del centro de Irun</t>
         </is>
       </c>
       <c r="C2703" s="20" t="n"/>
@@ -46781,7 +46725,7 @@
       </c>
       <c r="B2704" s="19" t="inlineStr">
         <is>
-          <t>EUS-93831</t>
+          <t>EUS-77322</t>
         </is>
       </c>
       <c r="C2704" s="20" t="n"/>
@@ -46933,7 +46877,7 @@
       </c>
       <c r="B2714" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-del-servicio-asistencia-tecnica-y-gestion-venta-ahorros-energeticos-generados-empresa-transporte-urbano-vitoria-gasteiz-tuvisa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-del-proyecto-y-direccion-obras-renovacion-red-distribucion-agua-distintas-zonas-del-centro-irun/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2714" s="20" t="n"/>
@@ -46944,7 +46888,7 @@
     <row r="2716" ht="30" customHeight="1">
       <c r="A2716" s="16" t="inlineStr">
         <is>
-          <t>FICHA 182: EUS-16126</t>
+          <t>FICHA 182: EUS-36090</t>
         </is>
       </c>
       <c r="B2716" s="17" t="n"/>
@@ -46969,7 +46913,7 @@
       <c r="E2717" s="20" t="n"/>
       <c r="F2717" s="20" t="n"/>
     </row>
-    <row r="2718" ht="45" customHeight="1">
+    <row r="2718" ht="20" customHeight="1">
       <c r="A2718" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -46977,7 +46921,7 @@
       </c>
       <c r="B2718" s="19" t="inlineStr">
         <is>
-          <t>Obras del proyecto de construcción de itinerario peatonal paralelo a la calzada entre los PK 1,810 y 2,030 de la  GI-3131 a Goroeta en Aretxabaleta (14-SV-79/2025 2LIC)</t>
+          <t>Obras de rehabilitación del edificio del Emisario submarino de Monpas</t>
         </is>
       </c>
       <c r="C2718" s="20" t="n"/>
@@ -46993,7 +46937,7 @@
       </c>
       <c r="B2719" s="19" t="inlineStr">
         <is>
-          <t>EUS-16126</t>
+          <t>EUS-36090</t>
         </is>
       </c>
       <c r="C2719" s="20" t="n"/>
@@ -47145,7 +47089,7 @@
       </c>
       <c r="B2729" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/obras-del-proyecto-construccion-itinerario-peatonal-paralelo-calzada-pk-1-810-y-2-030-gi-3131-goroeta-aretxabaleta-14-sv-79-2025-2lic/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-rehabilitacion-del-edificio-del-emisario-submarino-monpas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2729" s="20" t="n"/>
@@ -47156,7 +47100,7 @@
     <row r="2731" ht="30" customHeight="1">
       <c r="A2731" s="16" t="inlineStr">
         <is>
-          <t>FICHA 183: EUS-08987</t>
+          <t>FICHA 183: EUS-09001</t>
         </is>
       </c>
       <c r="B2731" s="17" t="n"/>
@@ -47189,7 +47133,7 @@
       </c>
       <c r="B2733" s="19" t="inlineStr">
         <is>
-          <t>reparación y puesta en servicio de red de fecales y pluviales en el centro CEIP Cantarrana Eskola HLHI</t>
+          <t>Servicio para la elaboración de un estudio medioambiental de la zona costera de Mompás y del estuario del río Oiartzun</t>
         </is>
       </c>
       <c r="C2733" s="20" t="n"/>
@@ -47205,7 +47149,7 @@
       </c>
       <c r="B2734" s="19" t="inlineStr">
         <is>
-          <t>EUS-08987</t>
+          <t>EUS-09001</t>
         </is>
       </c>
       <c r="C2734" s="20" t="n"/>
@@ -47357,7 +47301,7 @@
       </c>
       <c r="B2744" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-y-puesta-servicio-red-fecales-y-pluviales-centro-ceip-cantarrana-eskola-hlhi/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-elaboracion-estudio-medioambiental-zona-costera-mompas-y-del-estuario-del-rio-oiartzun/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2744" s="20" t="n"/>
@@ -47368,7 +47312,7 @@
     <row r="2746" ht="30" customHeight="1">
       <c r="A2746" s="16" t="inlineStr">
         <is>
-          <t>FICHA 184: EUS-71383</t>
+          <t>FICHA 184: EUS-57679</t>
         </is>
       </c>
       <c r="B2746" s="17" t="n"/>
@@ -47393,7 +47337,7 @@
       <c r="E2747" s="20" t="n"/>
       <c r="F2747" s="20" t="n"/>
     </row>
-    <row r="2748" ht="45" customHeight="1">
+    <row r="2748" ht="20" customHeight="1">
       <c r="A2748" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -47401,7 +47345,7 @@
       </c>
       <c r="B2748" s="19" t="inlineStr">
         <is>
-          <t>Suministro e instalación de un portón industrial enrollable para el edificio AIC Ermua</t>
+          <t>Plan de comunicacion y Sistema de Portavocias de la Agencia Vasca del Agua</t>
         </is>
       </c>
       <c r="C2748" s="20" t="n"/>
@@ -47417,7 +47361,7 @@
       </c>
       <c r="B2749" s="19" t="inlineStr">
         <is>
-          <t>EUS-71383</t>
+          <t>EUS-57679</t>
         </is>
       </c>
       <c r="C2749" s="20" t="n"/>
@@ -47569,7 +47513,7 @@
       </c>
       <c r="B2759" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-e-instalacion-porton-industrial-enrollable-edificio-aic-ermua/expjaso747486/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/plan-comunicacion-y-sistema-portavocias-agencia-vasca-del-agua/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2759" s="20" t="n"/>
@@ -47577,220 +47521,8 @@
       <c r="E2759" s="20" t="n"/>
       <c r="F2759" s="20" t="n"/>
     </row>
-    <row r="2761" ht="30" customHeight="1">
-      <c r="A2761" s="16" t="inlineStr">
-        <is>
-          <t>FICHA 185: EUS-06475</t>
-        </is>
-      </c>
-      <c r="B2761" s="17" t="n"/>
-      <c r="C2761" s="17" t="n"/>
-      <c r="D2761" s="17" t="n"/>
-      <c r="E2761" s="17" t="n"/>
-      <c r="F2761" s="17" t="n"/>
-    </row>
-    <row r="2762" ht="20" customHeight="1">
-      <c r="A2762" s="18" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B2762" s="19" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C2762" s="20" t="n"/>
-      <c r="D2762" s="20" t="n"/>
-      <c r="E2762" s="20" t="n"/>
-      <c r="F2762" s="20" t="n"/>
-    </row>
-    <row r="2763" ht="45" customHeight="1">
-      <c r="A2763" s="18" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B2763" s="19" t="inlineStr">
-        <is>
-          <t>ANS para determinadas aplicaciones implementadas por Izfe para el Departamento de Equilibrio Territorial Verde de la GFA-DFG para la gestión de la identificación, registro, saneamiento y movimiento an</t>
-        </is>
-      </c>
-      <c r="C2763" s="20" t="n"/>
-      <c r="D2763" s="20" t="n"/>
-      <c r="E2763" s="20" t="n"/>
-      <c r="F2763" s="20" t="n"/>
-    </row>
-    <row r="2764" ht="20" customHeight="1">
-      <c r="A2764" s="18" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B2764" s="19" t="inlineStr">
-        <is>
-          <t>EUS-06475</t>
-        </is>
-      </c>
-      <c r="C2764" s="20" t="n"/>
-      <c r="D2764" s="20" t="n"/>
-      <c r="E2764" s="20" t="n"/>
-      <c r="F2764" s="20" t="n"/>
-    </row>
-    <row r="2765" ht="20" customHeight="1">
-      <c r="A2765" s="18" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B2765" s="19" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C2765" s="20" t="n"/>
-      <c r="D2765" s="20" t="n"/>
-      <c r="E2765" s="20" t="n"/>
-      <c r="F2765" s="20" t="n"/>
-    </row>
-    <row r="2766" ht="20" customHeight="1">
-      <c r="A2766" s="18" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B2766" s="19" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C2766" s="20" t="n"/>
-      <c r="D2766" s="20" t="n"/>
-      <c r="E2766" s="20" t="n"/>
-      <c r="F2766" s="20" t="n"/>
-    </row>
-    <row r="2767" ht="20" customHeight="1">
-      <c r="A2767" s="18" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B2767" s="19" t="inlineStr"/>
-      <c r="C2767" s="20" t="n"/>
-      <c r="D2767" s="20" t="n"/>
-      <c r="E2767" s="20" t="n"/>
-      <c r="F2767" s="20" t="n"/>
-    </row>
-    <row r="2768" ht="20" customHeight="1">
-      <c r="A2768" s="18" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B2768" s="19" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C2768" s="20" t="n"/>
-      <c r="D2768" s="20" t="n"/>
-      <c r="E2768" s="20" t="n"/>
-      <c r="F2768" s="20" t="n"/>
-    </row>
-    <row r="2769" ht="20" customHeight="1">
-      <c r="A2769" s="18" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B2769" s="19" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C2769" s="20" t="n"/>
-      <c r="D2769" s="20" t="n"/>
-      <c r="E2769" s="20" t="n"/>
-      <c r="F2769" s="20" t="n"/>
-    </row>
-    <row r="2770" ht="20" customHeight="1">
-      <c r="A2770" s="18" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B2770" s="19" t="inlineStr"/>
-      <c r="C2770" s="20" t="n"/>
-      <c r="D2770" s="20" t="n"/>
-      <c r="E2770" s="20" t="n"/>
-      <c r="F2770" s="20" t="n"/>
-    </row>
-    <row r="2771" ht="20" customHeight="1">
-      <c r="A2771" s="18" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B2771" s="19" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C2771" s="20" t="n"/>
-      <c r="D2771" s="20" t="n"/>
-      <c r="E2771" s="20" t="n"/>
-      <c r="F2771" s="20" t="n"/>
-    </row>
-    <row r="2772" ht="20" customHeight="1">
-      <c r="A2772" s="18" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B2772" s="19" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C2772" s="20" t="n"/>
-      <c r="D2772" s="20" t="n"/>
-      <c r="E2772" s="20" t="n"/>
-      <c r="F2772" s="20" t="n"/>
-    </row>
-    <row r="2773" ht="20" customHeight="1">
-      <c r="A2773" s="18" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B2773" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C2773" s="20" t="n"/>
-      <c r="D2773" s="20" t="n"/>
-      <c r="E2773" s="20" t="n"/>
-      <c r="F2773" s="20" t="n"/>
-    </row>
-    <row r="2774" ht="45" customHeight="1">
-      <c r="A2774" s="18" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B2774" s="22" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/ans-determinadas-aplicaciones-implementadas-izfe-departamento-equilibrio-territorial-verde-gfa-dfg-gestion-identificacion-registro-saneamiento-y-movimiento-animal/expjaso739026/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C2774" s="20" t="n"/>
-      <c r="D2774" s="20" t="n"/>
-      <c r="E2774" s="20" t="n"/>
-      <c r="F2774" s="20" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="2590">
+  <mergeCells count="2576">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B2192:F2192"/>
     <mergeCell ref="B1765:F1765"/>
@@ -47892,7 +47624,6 @@
     <mergeCell ref="B243:F243"/>
     <mergeCell ref="B2465:F2465"/>
     <mergeCell ref="B2150:F2150"/>
-    <mergeCell ref="B2763:F2763"/>
     <mergeCell ref="B678:F678"/>
     <mergeCell ref="B363:F363"/>
     <mergeCell ref="B1731:F1731"/>
@@ -48029,7 +47760,6 @@
     <mergeCell ref="B1626:F1626"/>
     <mergeCell ref="B1582:F1582"/>
     <mergeCell ref="B1924:F1924"/>
-    <mergeCell ref="B2772:F2772"/>
     <mergeCell ref="B863:F863"/>
     <mergeCell ref="B2231:F2231"/>
     <mergeCell ref="B857:F857"/>
@@ -48211,7 +47941,6 @@
     <mergeCell ref="B2007:F2007"/>
     <mergeCell ref="B2436:F2436"/>
     <mergeCell ref="A1276:F1276"/>
-    <mergeCell ref="B2770:F2770"/>
     <mergeCell ref="B2307:F2307"/>
     <mergeCell ref="B2736:F2736"/>
     <mergeCell ref="B36:F36"/>
@@ -48590,13 +48319,11 @@
     <mergeCell ref="B1596:F1596"/>
     <mergeCell ref="B1281:F1281"/>
     <mergeCell ref="B1579:F1579"/>
-    <mergeCell ref="B2769:F2769"/>
     <mergeCell ref="B1589:F1589"/>
     <mergeCell ref="B2342:F2342"/>
     <mergeCell ref="B1283:F1283"/>
     <mergeCell ref="B257:F257"/>
     <mergeCell ref="B2464:F2464"/>
-    <mergeCell ref="B2771:F2771"/>
     <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B1162:F1162"/>
     <mergeCell ref="B92:F92"/>
@@ -48604,7 +48331,6 @@
     <mergeCell ref="B2675:F2675"/>
     <mergeCell ref="B1282:F1282"/>
     <mergeCell ref="B2335:F2335"/>
-    <mergeCell ref="B2764:F2764"/>
     <mergeCell ref="B557:F557"/>
     <mergeCell ref="B2248:F2248"/>
     <mergeCell ref="B2223:F2223"/>
@@ -48776,7 +48502,6 @@
     <mergeCell ref="B2433:F2433"/>
     <mergeCell ref="B1401:F1401"/>
     <mergeCell ref="B2427:F2427"/>
-    <mergeCell ref="B2767:F2767"/>
     <mergeCell ref="B2006:F2006"/>
     <mergeCell ref="B2304:F2304"/>
     <mergeCell ref="B219:F219"/>
@@ -48785,7 +48510,6 @@
     <mergeCell ref="B2733:F2733"/>
     <mergeCell ref="B1701:F1701"/>
     <mergeCell ref="B760:F760"/>
-    <mergeCell ref="B2762:F2762"/>
     <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="A2026:F2026"/>
     <mergeCell ref="B333:F333"/>
@@ -48939,7 +48663,6 @@
     <mergeCell ref="B1438:F1438"/>
     <mergeCell ref="B683:F683"/>
     <mergeCell ref="B1742:F1742"/>
-    <mergeCell ref="B2768:F2768"/>
     <mergeCell ref="B1527:F1527"/>
     <mergeCell ref="B2043:F2043"/>
     <mergeCell ref="A1036:F1036"/>
@@ -49005,7 +48728,6 @@
     <mergeCell ref="B1624:F1624"/>
     <mergeCell ref="B2110:F2110"/>
     <mergeCell ref="A991:F991"/>
-    <mergeCell ref="A2761:F2761"/>
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B2283:F2283"/>
@@ -49520,7 +49242,6 @@
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="B2620:F2620"/>
     <mergeCell ref="B1277:F1277"/>
-    <mergeCell ref="B2765:F2765"/>
     <mergeCell ref="B2249:F2249"/>
     <mergeCell ref="B2547:F2547"/>
     <mergeCell ref="B850:F850"/>
@@ -49885,7 +49606,6 @@
     <mergeCell ref="B2337:F2337"/>
     <mergeCell ref="B252:F252"/>
     <mergeCell ref="B2495:F2495"/>
-    <mergeCell ref="B2766:F2766"/>
     <mergeCell ref="B2451:F2451"/>
     <mergeCell ref="B366:F366"/>
     <mergeCell ref="B979:F979"/>
@@ -50120,7 +49840,6 @@
     <mergeCell ref="B835:F835"/>
     <mergeCell ref="B829:F829"/>
     <mergeCell ref="B74:F74"/>
-    <mergeCell ref="B2774:F2774"/>
     <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B68:F68"/>
     <mergeCell ref="B372:F372"/>
@@ -50269,7 +49988,6 @@
     <mergeCell ref="B872:F872"/>
     <mergeCell ref="B866:F866"/>
     <mergeCell ref="B111:F111"/>
-    <mergeCell ref="B2773:F2773"/>
     <mergeCell ref="B1301:F1301"/>
     <mergeCell ref="B986:F986"/>
     <mergeCell ref="B1024:F1024"/>
@@ -50567,7 +50285,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2729" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2744" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2759" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2774" r:id="rId185"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -50579,7 +50296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -52401,19 +52118,15 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIE</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+          <t>Circular design for bio-based innovation towards climate-neu</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr"/>
       <c r="D56" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -52437,15 +52150,19 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neu</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr"/>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIE</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -52857,12 +52574,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr"/>
@@ -52889,12 +52606,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr"/>
@@ -52921,12 +52638,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr"/>
@@ -52953,12 +52670,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr"/>
@@ -54873,12 +54590,12 @@
     <row r="133" ht="28" customHeight="1">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>925388828</t>
+          <t>934294980</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>THOMSON POWER EUROPE LTD</t>
+          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr"/>
@@ -54905,12 +54622,12 @@
     <row r="134" ht="28" customHeight="1">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>934294980</t>
+          <t>925388828</t>
         </is>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>SCHIAFFINI TRAVEL SOCIETA' PER AZIONI</t>
+          <t>THOMSON POWER EUROPE LTD</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr"/>
@@ -56249,7 +55966,7 @@
     <row r="176" ht="28" customHeight="1">
       <c r="A176" s="6" t="inlineStr">
         <is>
-          <t>EUS-43735</t>
+          <t>EUS-47596</t>
         </is>
       </c>
       <c r="B176" s="6" t="inlineStr">
@@ -56285,7 +56002,7 @@
     <row r="177" ht="28" customHeight="1">
       <c r="A177" s="6" t="inlineStr">
         <is>
-          <t>EUS-23831</t>
+          <t>EUS-51067</t>
         </is>
       </c>
       <c r="B177" s="6" t="inlineStr">
@@ -56321,12 +56038,12 @@
     <row r="178" ht="28" customHeight="1">
       <c r="A178" s="6" t="inlineStr">
         <is>
-          <t>EUS-89429</t>
+          <t>EUS-92303</t>
         </is>
       </c>
       <c r="B178" s="6" t="inlineStr">
         <is>
-          <t>Licitación, mediante procedimiento negociado sin publicidad,</t>
+          <t>Servicio de retirada, transporte y gestión de los residuos S</t>
         </is>
       </c>
       <c r="C178" s="6" t="inlineStr">
@@ -56357,12 +56074,12 @@
     <row r="179" ht="28" customHeight="1">
       <c r="A179" s="6" t="inlineStr">
         <is>
-          <t>EUS-69995</t>
+          <t>EUS-86597</t>
         </is>
       </c>
       <c r="B179" s="6" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Euro</t>
+          <t>Rehabilitacion parrales del barrio San Bartolome (zona Bizez</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
@@ -56378,7 +56095,7 @@
       <c r="E179" s="6" t="inlineStr"/>
       <c r="F179" s="25" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G179" s="6" t="inlineStr"/>
@@ -56393,12 +56110,12 @@
     <row r="180" ht="28" customHeight="1">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>EUS-59844</t>
+          <t>EUS-60193</t>
         </is>
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Euro</t>
         </is>
       </c>
       <c r="C180" s="6" t="inlineStr">
@@ -56429,12 +56146,12 @@
     <row r="181" ht="28" customHeight="1">
       <c r="A181" s="6" t="inlineStr">
         <is>
-          <t>EUS-33760</t>
+          <t>EUS-65298</t>
         </is>
       </c>
       <c r="B181" s="6" t="inlineStr">
         <is>
-          <t>Aprobar la contratación de los trabajos de "Integración de l</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
@@ -56465,12 +56182,12 @@
     <row r="182" ht="28" customHeight="1">
       <c r="A182" s="6" t="inlineStr">
         <is>
-          <t>EUS-93831</t>
+          <t>EUS-77322</t>
         </is>
       </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>Contratación del servicio de asistencia técnica y gestión de</t>
+          <t>Redacción del proyecto y dirección de las obras de renovació</t>
         </is>
       </c>
       <c r="C182" s="6" t="inlineStr">
@@ -56501,12 +56218,12 @@
     <row r="183" ht="28" customHeight="1">
       <c r="A183" s="6" t="inlineStr">
         <is>
-          <t>EUS-16126</t>
+          <t>EUS-36090</t>
         </is>
       </c>
       <c r="B183" s="6" t="inlineStr">
         <is>
-          <t>Obras del proyecto de construcción de itinerario peatonal pa</t>
+          <t xml:space="preserve">Obras de rehabilitación del edificio del Emisario submarino </t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
@@ -56537,12 +56254,12 @@
     <row r="184" ht="28" customHeight="1">
       <c r="A184" s="6" t="inlineStr">
         <is>
-          <t>EUS-08987</t>
+          <t>EUS-09001</t>
         </is>
       </c>
       <c r="B184" s="6" t="inlineStr">
         <is>
-          <t>reparación y puesta en servicio de red de fecales y pluviale</t>
+          <t>Servicio para la elaboración de un estudio medioambiental de</t>
         </is>
       </c>
       <c r="C184" s="6" t="inlineStr">
@@ -56573,12 +56290,12 @@
     <row r="185" ht="28" customHeight="1">
       <c r="A185" s="6" t="inlineStr">
         <is>
-          <t>EUS-71383</t>
+          <t>EUS-57679</t>
         </is>
       </c>
       <c r="B185" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro e instalación de un portón industrial enrollable </t>
+          <t xml:space="preserve">Plan de comunicacion y Sistema de Portavocias de la Agencia </t>
         </is>
       </c>
       <c r="C185" s="6" t="inlineStr">
@@ -56606,44 +56323,8 @@
       <c r="I185" s="6" t="inlineStr"/>
       <c r="J185" s="6" t="inlineStr"/>
     </row>
-    <row r="186" ht="28" customHeight="1">
-      <c r="A186" s="6" t="inlineStr">
-        <is>
-          <t>EUS-06475</t>
-        </is>
-      </c>
-      <c r="B186" s="6" t="inlineStr">
-        <is>
-          <t>ANS para determinadas aplicaciones implementadas por Izfe pa</t>
-        </is>
-      </c>
-      <c r="C186" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D186" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E186" s="6" t="inlineStr"/>
-      <c r="F186" s="25" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G186" s="6" t="inlineStr"/>
-      <c r="H186" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I186" s="6" t="inlineStr"/>
-      <c r="J186" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J186"/>
+  <autoFilter ref="A1:J185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-10-19
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$209</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$206</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M209"/>
+  <dimension ref="A1:M206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 18/10/2026 10:00 - 203 convocatorias - 14 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 19/10/2026 11:22 - 200 convocatorias - 14 nuevas</t>
         </is>
       </c>
     </row>
@@ -6713,12 +6713,12 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>njaunzdz</t>
+          <t>14587</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Mr. Dzintars Jaunzems</t>
+          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="K132" s="6" t="inlineStr">
         <is>
-          <t>Mr. Dzintars Jaunzems</t>
+          <t xml:space="preserve">A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance </t>
         </is>
       </c>
       <c r="L132" s="6" t="inlineStr"/>
@@ -6760,12 +6760,12 @@
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>14587</t>
+          <t>njaunzdz</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
+          <t>Mr. Dzintars Jaunzems</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr"/>
@@ -6789,7 +6789,7 @@
       </c>
       <c r="K133" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance </t>
+          <t>Mr. Dzintars Jaunzems</t>
         </is>
       </c>
       <c r="L133" s="6" t="inlineStr"/>
@@ -8264,12 +8264,12 @@
       </c>
       <c r="B165" s="6" t="inlineStr">
         <is>
-          <t>928057492</t>
+          <t>928211140</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA RODOPI</t>
+          <t>OBSHTINA PARVOMAY</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr"/>
@@ -8293,7 +8293,7 @@
       </c>
       <c r="K165" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA RODOPI</t>
+          <t>OBSHTINA PARVOMAY</t>
         </is>
       </c>
       <c r="L165" s="6" t="inlineStr"/>
@@ -8311,12 +8311,12 @@
       </c>
       <c r="B166" s="6" t="inlineStr">
         <is>
-          <t>926227393</t>
+          <t>928057492</t>
         </is>
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA SVILENGRAD</t>
+          <t>OBSHTINA RODOPI</t>
         </is>
       </c>
       <c r="D166" s="6" t="inlineStr"/>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="K166" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA SVILENGRAD</t>
+          <t>OBSHTINA RODOPI</t>
         </is>
       </c>
       <c r="L166" s="6" t="inlineStr"/>
@@ -8358,12 +8358,12 @@
       </c>
       <c r="B167" s="6" t="inlineStr">
         <is>
-          <t>928211140</t>
+          <t>926227393</t>
         </is>
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA PARVOMAY</t>
+          <t>OBSHTINA SVILENGRAD</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr"/>
@@ -8387,7 +8387,7 @@
       </c>
       <c r="K167" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA PARVOMAY</t>
+          <t>OBSHTINA SVILENGRAD</t>
         </is>
       </c>
       <c r="L167" s="6" t="inlineStr"/>
@@ -9439,12 +9439,12 @@
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>892931076</t>
+          <t>936518123</t>
         </is>
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VILA DE REI</t>
+          <t>Urban Initiative</t>
         </is>
       </c>
       <c r="D190" s="6" t="inlineStr"/>
@@ -9468,7 +9468,7 @@
       </c>
       <c r="K190" s="6" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VILA DE REI</t>
+          <t>Urban Initiative</t>
         </is>
       </c>
       <c r="L190" s="6" t="inlineStr"/>
@@ -9486,12 +9486,12 @@
       </c>
       <c r="B191" s="6" t="inlineStr">
         <is>
-          <t>936518123</t>
+          <t>892931076</t>
         </is>
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Urban Initiative</t>
+          <t>MUNICIPIO DE VILA DE REI</t>
         </is>
       </c>
       <c r="D191" s="6" t="inlineStr"/>
@@ -9515,7 +9515,7 @@
       </c>
       <c r="K191" s="6" t="inlineStr">
         <is>
-          <t>Urban Initiative</t>
+          <t>MUNICIPIO DE VILA DE REI</t>
         </is>
       </c>
       <c r="L191" s="6" t="inlineStr"/>
@@ -9525,57 +9525,65 @@
         </is>
       </c>
     </row>
-    <row r="192" ht="40" customHeight="1">
-      <c r="A192" s="5" t="inlineStr">
-        <is>
-          <t>Europa</t>
-        </is>
-      </c>
-      <c r="B192" s="6" t="inlineStr">
-        <is>
-          <t>EU4H</t>
-        </is>
-      </c>
-      <c r="C192" s="6" t="inlineStr">
-        <is>
-          <t>European Linkage of Initiative from Science to Action in Health</t>
-        </is>
-      </c>
-      <c r="D192" s="6" t="inlineStr"/>
-      <c r="E192" s="10" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F192" s="6" t="inlineStr"/>
-      <c r="G192" s="6" t="inlineStr"/>
-      <c r="H192" s="6" t="inlineStr"/>
-      <c r="I192" s="10" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J192" s="6" t="inlineStr">
-        <is>
-          <t>Revisar relevancia para el Ayuntamiento de Bilbao.</t>
-        </is>
-      </c>
-      <c r="K192" s="6" t="inlineStr">
-        <is>
-          <t>European Linkage of Initiative from Science to Action in Health</t>
-        </is>
-      </c>
-      <c r="L192" s="6" t="inlineStr"/>
-      <c r="M192" s="9" t="inlineStr">
+    <row r="192" ht="28" customHeight="1">
+      <c r="A192" s="13" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="40" customHeight="1">
+      <c r="A193" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B193" s="6" t="inlineStr">
+        <is>
+          <t>EUS-45445</t>
+        </is>
+      </c>
+      <c r="C193" s="6" t="inlineStr">
+        <is>
+          <t>Coordinación de seguridad y salud en las obras de reparación de escudo en la fachada principal de CIPF EMILIO CAMPUZANO de Bilbao (Bizkaia</t>
+        </is>
+      </c>
+      <c r="D193" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E193" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F193" s="6" t="inlineStr"/>
+      <c r="G193" s="6" t="inlineStr"/>
+      <c r="H193" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I193" s="11" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
+        </is>
+      </c>
+      <c r="J193" s="6" t="inlineStr"/>
+      <c r="K193" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L193" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M193" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="193" ht="28" customHeight="1">
-      <c r="A193" s="13" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
@@ -9587,12 +9595,15 @@
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>EUS-75332</t>
+          <t>EUS-92164</t>
         </is>
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Renovación de las licencias o suscripciones de software VMWare actualmente implantadas en la infraestructura tecnológica del Ayuntamiento de Eibar</t>
+          <t>Coordinación de
+seguridad y salud en las obras de desinfección y
+cierre de huecos en cancha cubierta en el IES
+IBARREKOLANDA de Bilbao (Bizkaia)</t>
         </is>
       </c>
       <c r="D194" s="6" t="inlineStr">
@@ -9642,7 +9653,7 @@
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>EUS-52813</t>
+          <t>EUS-64887</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
@@ -9697,7 +9708,7 @@
       </c>
       <c r="B196" s="6" t="inlineStr">
         <is>
-          <t>EUS-91123</t>
+          <t>EUS-78605</t>
         </is>
       </c>
       <c r="C196" s="6" t="inlineStr">
@@ -9752,12 +9763,12 @@
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>EUS-55604</t>
+          <t>EUS-19539</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Redacción del proyecto básico, de ejecución y la dirección facultativa para la construcción de aproximadamente 32 viviendas de protección oficial en la parcela SZR-1 y 11 alojamientos dotacionales en </t>
+          <t>coordinación de seguridad y salud en la obra de renovación y mejora de la eficiencia energética del alumbrado público</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
@@ -9807,12 +9818,12 @@
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t>EUS-64978</t>
+          <t>EUS-34915</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
         <is>
-          <t>Ayudas para la adquisición e implantación de sistemas de nuevas tecnologías y de seguridad en el sector del transporte público 2026.</t>
+          <t>1-alquiler camión cesta- (j9/01/2025) / seguro diario / gestión de residuos y limpieza plataforma / gasoil consumido 14</t>
         </is>
       </c>
       <c r="D198" s="6" t="inlineStr">
@@ -9829,12 +9840,12 @@
       <c r="G198" s="6" t="inlineStr"/>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I198" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I198" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J198" s="6" t="inlineStr"/>
@@ -9862,12 +9873,12 @@
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-66515</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y sociosanitaria) y 2 líneas (de retos y plataformas) son los ejes de una nueva convocatoria del Gobierno Vasco que persigue colaboración de E</t>
+          <t>Ayudas para la adquisición e implantación de sistemas de nuevas tecnologías y de seguridad en el sector del transporte público 2026.</t>
         </is>
       </c>
       <c r="D199" s="6" t="inlineStr">
@@ -9898,7 +9909,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L199" s="6" t="inlineStr"/>
+      <c r="L199" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M199" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -9913,12 +9928,12 @@
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t>EUS-29689</t>
+          <t>EUS-12421</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
+          <t>9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y sociosanitaria) y 2 líneas (de retos y plataformas) son los ejes de una nueva convocatoria del Gobierno Vasco que persigue colaboración de E</t>
         </is>
       </c>
       <c r="D200" s="6" t="inlineStr">
@@ -9968,12 +9983,12 @@
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>EUS-96720</t>
+          <t>EUS-30744</t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
         </is>
       </c>
       <c r="D201" s="6" t="inlineStr">
@@ -10023,12 +10038,12 @@
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>EUS-38676</t>
+          <t>EUS-39957</t>
         </is>
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>Servicio público de transporte urbano de viajeros en autobús de Arrasate</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="D202" s="6" t="inlineStr">
@@ -10045,7 +10060,7 @@
       <c r="G202" s="6" t="inlineStr"/>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I202" s="12" t="inlineStr">
@@ -10078,12 +10093,12 @@
       </c>
       <c r="B203" s="6" t="inlineStr">
         <is>
-          <t>EUS-18235</t>
+          <t>EUS-35301</t>
         </is>
       </c>
       <c r="C203" s="6" t="inlineStr">
         <is>
-          <t>Mantenimiento de la jardinería y limpieza de los parques de Monterron y Santa Barbara de Arrasate (reservado a centros especiales de empleo de iniciativa social y empresas de inserción)</t>
+          <t>transporte autobús histórico centenario funicular</t>
         </is>
       </c>
       <c r="D203" s="6" t="inlineStr">
@@ -10133,12 +10148,12 @@
       </c>
       <c r="B204" s="6" t="inlineStr">
         <is>
-          <t>EUS-95301</t>
+          <t>EUS-05161</t>
         </is>
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>Productos de limpieza para andretxea</t>
+          <t>suministro artículos de limpieza</t>
         </is>
       </c>
       <c r="D204" s="6" t="inlineStr">
@@ -10188,12 +10203,12 @@
       </c>
       <c r="B205" s="6" t="inlineStr">
         <is>
-          <t>EUS-12012</t>
+          <t>EUS-89367</t>
         </is>
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Menaje para las viviendas municipales</t>
+          <t>diorama estación kontxa ut 980 inaguación pasante</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
@@ -10243,12 +10258,12 @@
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>EUS-26392</t>
+          <t>EUS-18525</t>
         </is>
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>Menaje de hogar para viviendas municipales</t>
+          <t>trabajos y transportes de mercancías</t>
         </is>
       </c>
       <c r="D206" s="6" t="inlineStr">
@@ -10290,171 +10305,10 @@
         </is>
       </c>
     </row>
-    <row r="207" ht="40" customHeight="1">
-      <c r="A207" s="14" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B207" s="6" t="inlineStr">
-        <is>
-          <t>EUS-09152</t>
-        </is>
-      </c>
-      <c r="C207" s="6" t="inlineStr">
-        <is>
-          <t>Paraguas como obsequio para el día de aitites-amamas en fiestas</t>
-        </is>
-      </c>
-      <c r="D207" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E207" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F207" s="6" t="inlineStr"/>
-      <c r="G207" s="6" t="inlineStr"/>
-      <c r="H207" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I207" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J207" s="6" t="inlineStr"/>
-      <c r="K207" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L207" s="6" t="inlineStr"/>
-      <c r="M207" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" ht="40" customHeight="1">
-      <c r="A208" s="14" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B208" s="6" t="inlineStr">
-        <is>
-          <t>EUS-46833</t>
-        </is>
-      </c>
-      <c r="C208" s="6" t="inlineStr">
-        <is>
-          <t>Suministro e instalación de 27 farolas led de alumbrado solar autónomo</t>
-        </is>
-      </c>
-      <c r="D208" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E208" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F208" s="6" t="inlineStr"/>
-      <c r="G208" s="6" t="inlineStr"/>
-      <c r="H208" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I208" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J208" s="6" t="inlineStr"/>
-      <c r="K208" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L208" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M208" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="209" ht="40" customHeight="1">
-      <c r="A209" s="14" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B209" s="6" t="inlineStr">
-        <is>
-          <t>EUS-10725</t>
-        </is>
-      </c>
-      <c r="C209" s="6" t="inlineStr">
-        <is>
-          <t>Suministro en régimen de alquiler de 2 contenedores y 1 caseta vestuario con 2 duchas para uso de la brigada municipal de obras</t>
-        </is>
-      </c>
-      <c r="D209" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E209" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F209" s="6" t="inlineStr"/>
-      <c r="G209" s="6" t="inlineStr"/>
-      <c r="H209" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I209" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J209" s="6" t="inlineStr"/>
-      <c r="K209" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L209" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M209" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M209"/>
+  <autoFilter ref="A4:M206"/>
   <mergeCells count="4">
-    <mergeCell ref="A193:M193"/>
+    <mergeCell ref="A192:M192"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -10646,7 +10500,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId190"/>
@@ -10660,9 +10514,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M204" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M205" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M206" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M207" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M208" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M209" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10674,7 +10525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3044"/>
+  <dimension ref="A1:F2999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36500,7 +36351,7 @@
     <row r="1891" ht="30" customHeight="1">
       <c r="A1891" s="16" t="inlineStr">
         <is>
-          <t>FICHA 127: njaunzdz</t>
+          <t>FICHA 127: 14587</t>
         </is>
       </c>
       <c r="B1891" s="17" t="n"/>
@@ -36525,7 +36376,7 @@
       <c r="E1892" s="20" t="n"/>
       <c r="F1892" s="20" t="n"/>
     </row>
-    <row r="1893" ht="20" customHeight="1">
+    <row r="1893" ht="45" customHeight="1">
       <c r="A1893" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -36533,7 +36384,7 @@
       </c>
       <c r="B1893" s="19" t="inlineStr">
         <is>
-          <t>Mr. Dzintars Jaunzems</t>
+          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
         </is>
       </c>
       <c r="C1893" s="20" t="n"/>
@@ -36549,7 +36400,7 @@
       </c>
       <c r="B1894" s="19" t="inlineStr">
         <is>
-          <t>njaunzdz</t>
+          <t>14587</t>
         </is>
       </c>
       <c r="C1894" s="20" t="n"/>
@@ -36641,7 +36492,7 @@
       <c r="E1900" s="20" t="n"/>
       <c r="F1900" s="20" t="n"/>
     </row>
-    <row r="1901" ht="20" customHeight="1">
+    <row r="1901" ht="45" customHeight="1">
       <c r="A1901" s="18" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -36649,7 +36500,7 @@
       </c>
       <c r="B1901" s="19" t="inlineStr">
         <is>
-          <t>Mr. Dzintars Jaunzems</t>
+          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
         </is>
       </c>
       <c r="C1901" s="20" t="n"/>
@@ -36693,7 +36544,7 @@
       </c>
       <c r="B1904" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/njaunzdz</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/14587</t>
         </is>
       </c>
       <c r="C1904" s="20" t="n"/>
@@ -36704,7 +36555,7 @@
     <row r="1906" ht="30" customHeight="1">
       <c r="A1906" s="16" t="inlineStr">
         <is>
-          <t>FICHA 128: 14587</t>
+          <t>FICHA 128: njaunzdz</t>
         </is>
       </c>
       <c r="B1906" s="17" t="n"/>
@@ -36729,7 +36580,7 @@
       <c r="E1907" s="20" t="n"/>
       <c r="F1907" s="20" t="n"/>
     </row>
-    <row r="1908" ht="45" customHeight="1">
+    <row r="1908" ht="20" customHeight="1">
       <c r="A1908" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -36737,7 +36588,7 @@
       </c>
       <c r="B1908" s="19" t="inlineStr">
         <is>
-          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
+          <t>Mr. Dzintars Jaunzems</t>
         </is>
       </c>
       <c r="C1908" s="20" t="n"/>
@@ -36753,7 +36604,7 @@
       </c>
       <c r="B1909" s="19" t="inlineStr">
         <is>
-          <t>14587</t>
+          <t>njaunzdz</t>
         </is>
       </c>
       <c r="C1909" s="20" t="n"/>
@@ -36845,7 +36696,7 @@
       <c r="E1915" s="20" t="n"/>
       <c r="F1915" s="20" t="n"/>
     </row>
-    <row r="1916" ht="45" customHeight="1">
+    <row r="1916" ht="20" customHeight="1">
       <c r="A1916" s="18" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -36853,7 +36704,7 @@
       </c>
       <c r="B1916" s="19" t="inlineStr">
         <is>
-          <t>A project intends to build an innovative renewable energy production plant combined with an innovative electricity storage to provide controllable RES-E generation. How is the GHG emissions avoidance calculated in this case?</t>
+          <t>Mr. Dzintars Jaunzems</t>
         </is>
       </c>
       <c r="C1916" s="20" t="n"/>
@@ -36897,7 +36748,7 @@
       </c>
       <c r="B1919" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/14587</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/njaunzdz</t>
         </is>
       </c>
       <c r="C1919" s="20" t="n"/>
@@ -43232,7 +43083,7 @@
     <row r="2386" ht="30" customHeight="1">
       <c r="A2386" s="16" t="inlineStr">
         <is>
-          <t>FICHA 160: 928057492</t>
+          <t>FICHA 160: 928211140</t>
         </is>
       </c>
       <c r="B2386" s="17" t="n"/>
@@ -43265,7 +43116,7 @@
       </c>
       <c r="B2388" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA RODOPI</t>
+          <t>OBSHTINA PARVOMAY</t>
         </is>
       </c>
       <c r="C2388" s="20" t="n"/>
@@ -43281,7 +43132,7 @@
       </c>
       <c r="B2389" s="19" t="inlineStr">
         <is>
-          <t>928057492</t>
+          <t>928211140</t>
         </is>
       </c>
       <c r="C2389" s="20" t="n"/>
@@ -43381,7 +43232,7 @@
       </c>
       <c r="B2396" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA RODOPI</t>
+          <t>OBSHTINA PARVOMAY</t>
         </is>
       </c>
       <c r="C2396" s="20" t="n"/>
@@ -43425,7 +43276,7 @@
       </c>
       <c r="B2399" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928057492</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928211140</t>
         </is>
       </c>
       <c r="C2399" s="20" t="n"/>
@@ -43436,7 +43287,7 @@
     <row r="2401" ht="30" customHeight="1">
       <c r="A2401" s="16" t="inlineStr">
         <is>
-          <t>FICHA 161: 926227393</t>
+          <t>FICHA 161: 928057492</t>
         </is>
       </c>
       <c r="B2401" s="17" t="n"/>
@@ -43469,7 +43320,7 @@
       </c>
       <c r="B2403" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA SVILENGRAD</t>
+          <t>OBSHTINA RODOPI</t>
         </is>
       </c>
       <c r="C2403" s="20" t="n"/>
@@ -43485,7 +43336,7 @@
       </c>
       <c r="B2404" s="19" t="inlineStr">
         <is>
-          <t>926227393</t>
+          <t>928057492</t>
         </is>
       </c>
       <c r="C2404" s="20" t="n"/>
@@ -43585,7 +43436,7 @@
       </c>
       <c r="B2411" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA SVILENGRAD</t>
+          <t>OBSHTINA RODOPI</t>
         </is>
       </c>
       <c r="C2411" s="20" t="n"/>
@@ -43629,7 +43480,7 @@
       </c>
       <c r="B2414" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/926227393</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928057492</t>
         </is>
       </c>
       <c r="C2414" s="20" t="n"/>
@@ -43640,7 +43491,7 @@
     <row r="2416" ht="30" customHeight="1">
       <c r="A2416" s="16" t="inlineStr">
         <is>
-          <t>FICHA 162: 928211140</t>
+          <t>FICHA 162: 926227393</t>
         </is>
       </c>
       <c r="B2416" s="17" t="n"/>
@@ -43673,7 +43524,7 @@
       </c>
       <c r="B2418" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA PARVOMAY</t>
+          <t>OBSHTINA SVILENGRAD</t>
         </is>
       </c>
       <c r="C2418" s="20" t="n"/>
@@ -43689,7 +43540,7 @@
       </c>
       <c r="B2419" s="19" t="inlineStr">
         <is>
-          <t>928211140</t>
+          <t>926227393</t>
         </is>
       </c>
       <c r="C2419" s="20" t="n"/>
@@ -43789,7 +43640,7 @@
       </c>
       <c r="B2426" s="19" t="inlineStr">
         <is>
-          <t>OBSHTINA PARVOMAY</t>
+          <t>OBSHTINA SVILENGRAD</t>
         </is>
       </c>
       <c r="C2426" s="20" t="n"/>
@@ -43833,7 +43684,7 @@
       </c>
       <c r="B2429" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928211140</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/926227393</t>
         </is>
       </c>
       <c r="C2429" s="20" t="n"/>
@@ -48340,7 +48191,7 @@
     <row r="2761" ht="30" customHeight="1">
       <c r="A2761" s="16" t="inlineStr">
         <is>
-          <t>FICHA 185: 892931076</t>
+          <t>FICHA 185: 936518123</t>
         </is>
       </c>
       <c r="B2761" s="17" t="n"/>
@@ -48373,7 +48224,7 @@
       </c>
       <c r="B2763" s="19" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VILA DE REI</t>
+          <t>Urban Initiative</t>
         </is>
       </c>
       <c r="C2763" s="20" t="n"/>
@@ -48389,7 +48240,7 @@
       </c>
       <c r="B2764" s="19" t="inlineStr">
         <is>
-          <t>892931076</t>
+          <t>936518123</t>
         </is>
       </c>
       <c r="C2764" s="20" t="n"/>
@@ -48489,7 +48340,7 @@
       </c>
       <c r="B2771" s="19" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VILA DE REI</t>
+          <t>Urban Initiative</t>
         </is>
       </c>
       <c r="C2771" s="20" t="n"/>
@@ -48533,7 +48384,7 @@
       </c>
       <c r="B2774" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/892931076</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/936518123</t>
         </is>
       </c>
       <c r="C2774" s="20" t="n"/>
@@ -48544,7 +48395,7 @@
     <row r="2776" ht="30" customHeight="1">
       <c r="A2776" s="16" t="inlineStr">
         <is>
-          <t>FICHA 186: 936518123</t>
+          <t>FICHA 186: 892931076</t>
         </is>
       </c>
       <c r="B2776" s="17" t="n"/>
@@ -48577,7 +48428,7 @@
       </c>
       <c r="B2778" s="19" t="inlineStr">
         <is>
-          <t>Urban Initiative</t>
+          <t>MUNICIPIO DE VILA DE REI</t>
         </is>
       </c>
       <c r="C2778" s="20" t="n"/>
@@ -48593,7 +48444,7 @@
       </c>
       <c r="B2779" s="19" t="inlineStr">
         <is>
-          <t>936518123</t>
+          <t>892931076</t>
         </is>
       </c>
       <c r="C2779" s="20" t="n"/>
@@ -48693,7 +48544,7 @@
       </c>
       <c r="B2786" s="19" t="inlineStr">
         <is>
-          <t>Urban Initiative</t>
+          <t>MUNICIPIO DE VILA DE REI</t>
         </is>
       </c>
       <c r="C2786" s="20" t="n"/>
@@ -48737,7 +48588,7 @@
       </c>
       <c r="B2789" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/936518123</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/892931076</t>
         </is>
       </c>
       <c r="C2789" s="20" t="n"/>
@@ -48748,7 +48599,7 @@
     <row r="2791" ht="30" customHeight="1">
       <c r="A2791" s="16" t="inlineStr">
         <is>
-          <t>FICHA 187: EU4H</t>
+          <t>FICHA 187: EUS-45445</t>
         </is>
       </c>
       <c r="B2791" s="17" t="n"/>
@@ -48765,7 +48616,7 @@
       </c>
       <c r="B2792" s="19" t="inlineStr">
         <is>
-          <t>🇪🇺 Europa</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C2792" s="20" t="n"/>
@@ -48773,7 +48624,7 @@
       <c r="E2792" s="20" t="n"/>
       <c r="F2792" s="20" t="n"/>
     </row>
-    <row r="2793" ht="20" customHeight="1">
+    <row r="2793" ht="45" customHeight="1">
       <c r="A2793" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -48781,7 +48632,7 @@
       </c>
       <c r="B2793" s="19" t="inlineStr">
         <is>
-          <t>European Linkage of Initiative from Science to Action in Health</t>
+          <t>Coordinación de seguridad y salud en las obras de reparación de escudo en la fachada principal de CIPF EMILIO CAMPUZANO de Bilbao (Bizkaia</t>
         </is>
       </c>
       <c r="C2793" s="20" t="n"/>
@@ -48797,7 +48648,7 @@
       </c>
       <c r="B2794" s="19" t="inlineStr">
         <is>
-          <t>EU4H</t>
+          <t>EUS-45445</t>
         </is>
       </c>
       <c r="C2794" s="20" t="n"/>
@@ -48811,7 +48662,11 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B2795" s="19" t="inlineStr"/>
+      <c r="B2795" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
       <c r="C2795" s="20" t="n"/>
       <c r="D2795" s="20" t="n"/>
       <c r="E2795" s="20" t="n"/>
@@ -48825,7 +48680,7 @@
       </c>
       <c r="B2796" s="19" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="C2796" s="20" t="n"/>
@@ -48869,7 +48724,7 @@
       </c>
       <c r="B2799" s="19" t="inlineStr">
         <is>
-          <t>No disponible</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C2799" s="20" t="n"/>
@@ -48883,11 +48738,7 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B2800" s="19" t="inlineStr">
-        <is>
-          <t>EU4H-2022-PJ-3</t>
-        </is>
-      </c>
+      <c r="B2800" s="19" t="inlineStr"/>
       <c r="C2800" s="20" t="n"/>
       <c r="D2800" s="20" t="n"/>
       <c r="E2800" s="20" t="n"/>
@@ -48901,7 +48752,7 @@
       </c>
       <c r="B2801" s="19" t="inlineStr">
         <is>
-          <t>European Linkage of Initiative from Science to Action in Health</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C2801" s="20" t="n"/>
@@ -48915,7 +48766,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B2802" s="19" t="inlineStr"/>
+      <c r="B2802" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C2802" s="20" t="n"/>
       <c r="D2802" s="20" t="n"/>
       <c r="E2802" s="20" t="n"/>
@@ -48927,9 +48782,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B2803" s="19" t="inlineStr">
-        <is>
-          <t>INFO — Revisar relevancia para el Ayuntamiento de Bilbao.</t>
+      <c r="B2803" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C2803" s="20" t="n"/>
@@ -48945,7 +48800,7 @@
       </c>
       <c r="B2804" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/EU4H</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-obras-reparacion-escudo-fachada-principal-cipf-emilio-campuzano-bilbao-bizkaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2804" s="20" t="n"/>
@@ -48956,7 +48811,7 @@
     <row r="2806" ht="30" customHeight="1">
       <c r="A2806" s="16" t="inlineStr">
         <is>
-          <t>FICHA 188: EUS-75332</t>
+          <t>FICHA 188: EUS-92164</t>
         </is>
       </c>
       <c r="B2806" s="17" t="n"/>
@@ -48989,7 +48844,10 @@
       </c>
       <c r="B2808" s="19" t="inlineStr">
         <is>
-          <t>Renovación de las licencias o suscripciones de software VMWare actualmente implantadas en la infraestructura tecnológica del Ayuntamiento de Eibar</t>
+          <t>Coordinación de
+seguridad y salud en las obras de desinfección y
+cierre de huecos en cancha cubierta en el IES
+IBARREKOLANDA de Bilbao (Bizkaia)</t>
         </is>
       </c>
       <c r="C2808" s="20" t="n"/>
@@ -49005,7 +48863,7 @@
       </c>
       <c r="B2809" s="19" t="inlineStr">
         <is>
-          <t>EUS-75332</t>
+          <t>EUS-92164</t>
         </is>
       </c>
       <c r="C2809" s="20" t="n"/>
@@ -49157,7 +49015,7 @@
       </c>
       <c r="B2819" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/renovacion-licencias-o-suscripciones-software-vmware-actualmente-implantadas-infraestructura-tecnologica-del-ayuntamiento-eibar/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-obras-desinfeccion-y-cierre-huecos-cancha-cubierta-ies-ibarrekolanda-bilbao-bizkaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2819" s="20" t="n"/>
@@ -49168,7 +49026,7 @@
     <row r="2821" ht="30" customHeight="1">
       <c r="A2821" s="16" t="inlineStr">
         <is>
-          <t>FICHA 189: EUS-52813</t>
+          <t>FICHA 189: EUS-64887</t>
         </is>
       </c>
       <c r="B2821" s="17" t="n"/>
@@ -49217,7 +49075,7 @@
       </c>
       <c r="B2824" s="19" t="inlineStr">
         <is>
-          <t>EUS-52813</t>
+          <t>EUS-64887</t>
         </is>
       </c>
       <c r="C2824" s="20" t="n"/>
@@ -49380,7 +49238,7 @@
     <row r="2836" ht="30" customHeight="1">
       <c r="A2836" s="16" t="inlineStr">
         <is>
-          <t>FICHA 190: EUS-91123</t>
+          <t>FICHA 190: EUS-78605</t>
         </is>
       </c>
       <c r="B2836" s="17" t="n"/>
@@ -49429,7 +49287,7 @@
       </c>
       <c r="B2839" s="19" t="inlineStr">
         <is>
-          <t>EUS-91123</t>
+          <t>EUS-78605</t>
         </is>
       </c>
       <c r="C2839" s="20" t="n"/>
@@ -49592,7 +49450,7 @@
     <row r="2851" ht="30" customHeight="1">
       <c r="A2851" s="16" t="inlineStr">
         <is>
-          <t>FICHA 191: EUS-55604</t>
+          <t>FICHA 191: EUS-19539</t>
         </is>
       </c>
       <c r="B2851" s="17" t="n"/>
@@ -49625,7 +49483,7 @@
       </c>
       <c r="B2853" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Redacción del proyecto básico, de ejecución y la dirección facultativa para la construcción de aproximadamente 32 viviendas de protección oficial en la parcela SZR-1 y 11 alojamientos dotacionales en </t>
+          <t>coordinación de seguridad y salud en la obra de renovación y mejora de la eficiencia energética del alumbrado público</t>
         </is>
       </c>
       <c r="C2853" s="20" t="n"/>
@@ -49641,7 +49499,7 @@
       </c>
       <c r="B2854" s="19" t="inlineStr">
         <is>
-          <t>EUS-55604</t>
+          <t>EUS-19539</t>
         </is>
       </c>
       <c r="C2854" s="20" t="n"/>
@@ -49793,7 +49651,7 @@
       </c>
       <c r="B2864" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-del-proyecto-basico-ejecucion-y-direccion-facultativa-construccion-aproximadamente-32-viviendas-proteccion-oficial-parcela-szr-1-y-11-alojamientos-dotacionales-parcela-ead-1-portugalete-bizkaia-acorde-metodologia-trabajo-bim-teniendo-cuenta-pri/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-obra-renovacion-y-mejora-eficiencia-energetica-del-alumbrado-publico/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2864" s="20" t="n"/>
@@ -49804,7 +49662,7 @@
     <row r="2866" ht="30" customHeight="1">
       <c r="A2866" s="16" t="inlineStr">
         <is>
-          <t>FICHA 192: EUS-64978</t>
+          <t>FICHA 192: EUS-34915</t>
         </is>
       </c>
       <c r="B2866" s="17" t="n"/>
@@ -49837,7 +49695,7 @@
       </c>
       <c r="B2868" s="19" t="inlineStr">
         <is>
-          <t>Ayudas para la adquisición e implantación de sistemas de nuevas tecnologías y de seguridad en el sector del transporte público 2026.</t>
+          <t>1-alquiler camión cesta- (j9/01/2025) / seguro diario / gestión de residuos y limpieza plataforma / gasoil consumido 14</t>
         </is>
       </c>
       <c r="C2868" s="20" t="n"/>
@@ -49853,7 +49711,7 @@
       </c>
       <c r="B2869" s="19" t="inlineStr">
         <is>
-          <t>EUS-64978</t>
+          <t>EUS-34915</t>
         </is>
       </c>
       <c r="C2869" s="20" t="n"/>
@@ -49929,7 +49787,7 @@
       </c>
       <c r="B2874" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C2874" s="20" t="n"/>
@@ -49987,9 +49845,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B2878" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B2878" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C2878" s="20" t="n"/>
@@ -50005,7 +49863,7 @@
       </c>
       <c r="B2879" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/nuevas-tecnologias-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/1-alquiler-camion-cesta-j9-01-2025-seguro-diario-gestion-residuos-y-limpieza-plataforma-gasoil-consumido-14/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2879" s="20" t="n"/>
@@ -50016,7 +49874,7 @@
     <row r="2881" ht="30" customHeight="1">
       <c r="A2881" s="16" t="inlineStr">
         <is>
-          <t>FICHA 193: EUS-61815</t>
+          <t>FICHA 193: EUS-66515</t>
         </is>
       </c>
       <c r="B2881" s="17" t="n"/>
@@ -50049,7 +49907,7 @@
       </c>
       <c r="B2883" s="19" t="inlineStr">
         <is>
-          <t>9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y sociosanitaria) y 2 líneas (de retos y plataformas) son los ejes de una nueva convocatoria del Gobierno Vasco que persigue colaboración de E</t>
+          <t>Ayudas para la adquisición e implantación de sistemas de nuevas tecnologías y de seguridad en el sector del transporte público 2026.</t>
         </is>
       </c>
       <c r="C2883" s="20" t="n"/>
@@ -50065,7 +49923,7 @@
       </c>
       <c r="B2884" s="19" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-66515</t>
         </is>
       </c>
       <c r="C2884" s="20" t="n"/>
@@ -50217,7 +50075,7 @@
       </c>
       <c r="B2894" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/berrikuntzaitsasargierron/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/nuevas-tecnologias-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2894" s="20" t="n"/>
@@ -50228,7 +50086,7 @@
     <row r="2896" ht="30" customHeight="1">
       <c r="A2896" s="16" t="inlineStr">
         <is>
-          <t>FICHA 194: EUS-29689</t>
+          <t>FICHA 194: EUS-12421</t>
         </is>
       </c>
       <c r="B2896" s="17" t="n"/>
@@ -50261,7 +50119,7 @@
       </c>
       <c r="B2898" s="19" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
+          <t>9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y sociosanitaria) y 2 líneas (de retos y plataformas) son los ejes de una nueva convocatoria del Gobierno Vasco que persigue colaboración de E</t>
         </is>
       </c>
       <c r="C2898" s="20" t="n"/>
@@ -50277,7 +50135,7 @@
       </c>
       <c r="B2899" s="19" t="inlineStr">
         <is>
-          <t>EUS-29689</t>
+          <t>EUS-12421</t>
         </is>
       </c>
       <c r="C2899" s="20" t="n"/>
@@ -50429,7 +50287,7 @@
       </c>
       <c r="B2909" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/bioaniztasunfundaziohirin/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/berrikuntzaitsasargierron/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2909" s="20" t="n"/>
@@ -50440,7 +50298,7 @@
     <row r="2911" ht="30" customHeight="1">
       <c r="A2911" s="16" t="inlineStr">
         <is>
-          <t>FICHA 195: EUS-96720</t>
+          <t>FICHA 195: EUS-30744</t>
         </is>
       </c>
       <c r="B2911" s="17" t="n"/>
@@ -50465,7 +50323,7 @@
       <c r="E2912" s="20" t="n"/>
       <c r="F2912" s="20" t="n"/>
     </row>
-    <row r="2913" ht="20" customHeight="1">
+    <row r="2913" ht="45" customHeight="1">
       <c r="A2913" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -50473,7 +50331,7 @@
       </c>
       <c r="B2913" s="19" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Europeo de Desarrollo Regional y la Fundación Biodiversidad, en favor de la renaturalización urbana, infraestructura verde, conectividad de espa</t>
         </is>
       </c>
       <c r="C2913" s="20" t="n"/>
@@ -50489,7 +50347,7 @@
       </c>
       <c r="B2914" s="19" t="inlineStr">
         <is>
-          <t>EUS-96720</t>
+          <t>EUS-30744</t>
         </is>
       </c>
       <c r="C2914" s="20" t="n"/>
@@ -50641,7 +50499,7 @@
       </c>
       <c r="B2924" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/comunicacion-previs-digitalizacion-2027/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/bioaniztasunfundaziohirin/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2924" s="20" t="n"/>
@@ -50652,7 +50510,7 @@
     <row r="2926" ht="30" customHeight="1">
       <c r="A2926" s="16" t="inlineStr">
         <is>
-          <t>FICHA 196: EUS-38676</t>
+          <t>FICHA 196: EUS-39957</t>
         </is>
       </c>
       <c r="B2926" s="17" t="n"/>
@@ -50685,7 +50543,7 @@
       </c>
       <c r="B2928" s="19" t="inlineStr">
         <is>
-          <t>Servicio público de transporte urbano de viajeros en autobús de Arrasate</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="C2928" s="20" t="n"/>
@@ -50701,7 +50559,7 @@
       </c>
       <c r="B2929" s="19" t="inlineStr">
         <is>
-          <t>EUS-38676</t>
+          <t>EUS-39957</t>
         </is>
       </c>
       <c r="C2929" s="20" t="n"/>
@@ -50777,7 +50635,7 @@
       </c>
       <c r="B2934" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C2934" s="20" t="n"/>
@@ -50853,7 +50711,7 @@
       </c>
       <c r="B2939" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-publico-transporte-urbano-viajeros-autobus-arrasate/expjaso750179/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/comunicacion-previs-digitalizacion-2027/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2939" s="20" t="n"/>
@@ -50864,7 +50722,7 @@
     <row r="2941" ht="30" customHeight="1">
       <c r="A2941" s="16" t="inlineStr">
         <is>
-          <t>FICHA 197: EUS-18235</t>
+          <t>FICHA 197: EUS-35301</t>
         </is>
       </c>
       <c r="B2941" s="17" t="n"/>
@@ -50889,7 +50747,7 @@
       <c r="E2942" s="20" t="n"/>
       <c r="F2942" s="20" t="n"/>
     </row>
-    <row r="2943" ht="45" customHeight="1">
+    <row r="2943" ht="20" customHeight="1">
       <c r="A2943" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -50897,7 +50755,7 @@
       </c>
       <c r="B2943" s="19" t="inlineStr">
         <is>
-          <t>Mantenimiento de la jardinería y limpieza de los parques de Monterron y Santa Barbara de Arrasate (reservado a centros especiales de empleo de iniciativa social y empresas de inserción)</t>
+          <t>transporte autobús histórico centenario funicular</t>
         </is>
       </c>
       <c r="C2943" s="20" t="n"/>
@@ -50913,7 +50771,7 @@
       </c>
       <c r="B2944" s="19" t="inlineStr">
         <is>
-          <t>EUS-18235</t>
+          <t>EUS-35301</t>
         </is>
       </c>
       <c r="C2944" s="20" t="n"/>
@@ -51065,7 +50923,7 @@
       </c>
       <c r="B2954" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-jardineria-y-limpieza-parques-monterron-y-santa-barbara-arrasate-reservado-centros-especiales-empleo-iniciativa-social-y-empresas-insercion/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-autobus-historico-centenario-funicular/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2954" s="20" t="n"/>
@@ -51076,7 +50934,7 @@
     <row r="2956" ht="30" customHeight="1">
       <c r="A2956" s="16" t="inlineStr">
         <is>
-          <t>FICHA 198: EUS-95301</t>
+          <t>FICHA 198: EUS-05161</t>
         </is>
       </c>
       <c r="B2956" s="17" t="n"/>
@@ -51109,7 +50967,7 @@
       </c>
       <c r="B2958" s="19" t="inlineStr">
         <is>
-          <t>Productos de limpieza para andretxea</t>
+          <t>suministro artículos de limpieza</t>
         </is>
       </c>
       <c r="C2958" s="20" t="n"/>
@@ -51125,7 +50983,7 @@
       </c>
       <c r="B2959" s="19" t="inlineStr">
         <is>
-          <t>EUS-95301</t>
+          <t>EUS-05161</t>
         </is>
       </c>
       <c r="C2959" s="20" t="n"/>
@@ -51277,7 +51135,7 @@
       </c>
       <c r="B2969" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/productos-limpieza-andretxea/expgeeibar22008/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-articulos-limpieza/expcm539280/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2969" s="20" t="n"/>
@@ -51288,7 +51146,7 @@
     <row r="2971" ht="30" customHeight="1">
       <c r="A2971" s="16" t="inlineStr">
         <is>
-          <t>FICHA 199: EUS-12012</t>
+          <t>FICHA 199: EUS-89367</t>
         </is>
       </c>
       <c r="B2971" s="17" t="n"/>
@@ -51321,7 +51179,7 @@
       </c>
       <c r="B2973" s="19" t="inlineStr">
         <is>
-          <t>Menaje para las viviendas municipales</t>
+          <t>diorama estación kontxa ut 980 inaguación pasante</t>
         </is>
       </c>
       <c r="C2973" s="20" t="n"/>
@@ -51337,7 +51195,7 @@
       </c>
       <c r="B2974" s="19" t="inlineStr">
         <is>
-          <t>EUS-12012</t>
+          <t>EUS-89367</t>
         </is>
       </c>
       <c r="C2974" s="20" t="n"/>
@@ -51489,7 +51347,7 @@
       </c>
       <c r="B2984" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/menaje-viviendas-municipales/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/diorama-estacion-kontxa-ut-980-inaguacion-pasante/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2984" s="20" t="n"/>
@@ -51500,7 +51358,7 @@
     <row r="2986" ht="30" customHeight="1">
       <c r="A2986" s="16" t="inlineStr">
         <is>
-          <t>FICHA 200: EUS-26392</t>
+          <t>FICHA 200: EUS-18525</t>
         </is>
       </c>
       <c r="B2986" s="17" t="n"/>
@@ -51533,7 +51391,7 @@
       </c>
       <c r="B2988" s="19" t="inlineStr">
         <is>
-          <t>Menaje de hogar para viviendas municipales</t>
+          <t>trabajos y transportes de mercancías</t>
         </is>
       </c>
       <c r="C2988" s="20" t="n"/>
@@ -51549,7 +51407,7 @@
       </c>
       <c r="B2989" s="19" t="inlineStr">
         <is>
-          <t>EUS-26392</t>
+          <t>EUS-18525</t>
         </is>
       </c>
       <c r="C2989" s="20" t="n"/>
@@ -51701,7 +51559,7 @@
       </c>
       <c r="B2999" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/menaje-hogar-viviendas-municipales/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/trabajos-y-transportes-mercancias/expcm539272/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2999" s="20" t="n"/>
@@ -51709,644 +51567,8 @@
       <c r="E2999" s="20" t="n"/>
       <c r="F2999" s="20" t="n"/>
     </row>
-    <row r="3001" ht="30" customHeight="1">
-      <c r="A3001" s="16" t="inlineStr">
-        <is>
-          <t>FICHA 201: EUS-09152</t>
-        </is>
-      </c>
-      <c r="B3001" s="17" t="n"/>
-      <c r="C3001" s="17" t="n"/>
-      <c r="D3001" s="17" t="n"/>
-      <c r="E3001" s="17" t="n"/>
-      <c r="F3001" s="17" t="n"/>
-    </row>
-    <row r="3002" ht="20" customHeight="1">
-      <c r="A3002" s="18" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B3002" s="19" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C3002" s="20" t="n"/>
-      <c r="D3002" s="20" t="n"/>
-      <c r="E3002" s="20" t="n"/>
-      <c r="F3002" s="20" t="n"/>
-    </row>
-    <row r="3003" ht="20" customHeight="1">
-      <c r="A3003" s="18" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B3003" s="19" t="inlineStr">
-        <is>
-          <t>Paraguas como obsequio para el día de aitites-amamas en fiestas</t>
-        </is>
-      </c>
-      <c r="C3003" s="20" t="n"/>
-      <c r="D3003" s="20" t="n"/>
-      <c r="E3003" s="20" t="n"/>
-      <c r="F3003" s="20" t="n"/>
-    </row>
-    <row r="3004" ht="20" customHeight="1">
-      <c r="A3004" s="18" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3004" s="19" t="inlineStr">
-        <is>
-          <t>EUS-09152</t>
-        </is>
-      </c>
-      <c r="C3004" s="20" t="n"/>
-      <c r="D3004" s="20" t="n"/>
-      <c r="E3004" s="20" t="n"/>
-      <c r="F3004" s="20" t="n"/>
-    </row>
-    <row r="3005" ht="20" customHeight="1">
-      <c r="A3005" s="18" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B3005" s="19" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C3005" s="20" t="n"/>
-      <c r="D3005" s="20" t="n"/>
-      <c r="E3005" s="20" t="n"/>
-      <c r="F3005" s="20" t="n"/>
-    </row>
-    <row r="3006" ht="20" customHeight="1">
-      <c r="A3006" s="18" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B3006" s="19" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C3006" s="20" t="n"/>
-      <c r="D3006" s="20" t="n"/>
-      <c r="E3006" s="20" t="n"/>
-      <c r="F3006" s="20" t="n"/>
-    </row>
-    <row r="3007" ht="20" customHeight="1">
-      <c r="A3007" s="18" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B3007" s="19" t="inlineStr"/>
-      <c r="C3007" s="20" t="n"/>
-      <c r="D3007" s="20" t="n"/>
-      <c r="E3007" s="20" t="n"/>
-      <c r="F3007" s="20" t="n"/>
-    </row>
-    <row r="3008" ht="20" customHeight="1">
-      <c r="A3008" s="18" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B3008" s="19" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C3008" s="20" t="n"/>
-      <c r="D3008" s="20" t="n"/>
-      <c r="E3008" s="20" t="n"/>
-      <c r="F3008" s="20" t="n"/>
-    </row>
-    <row r="3009" ht="20" customHeight="1">
-      <c r="A3009" s="18" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B3009" s="19" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C3009" s="20" t="n"/>
-      <c r="D3009" s="20" t="n"/>
-      <c r="E3009" s="20" t="n"/>
-      <c r="F3009" s="20" t="n"/>
-    </row>
-    <row r="3010" ht="20" customHeight="1">
-      <c r="A3010" s="18" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B3010" s="19" t="inlineStr"/>
-      <c r="C3010" s="20" t="n"/>
-      <c r="D3010" s="20" t="n"/>
-      <c r="E3010" s="20" t="n"/>
-      <c r="F3010" s="20" t="n"/>
-    </row>
-    <row r="3011" ht="20" customHeight="1">
-      <c r="A3011" s="18" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B3011" s="19" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C3011" s="20" t="n"/>
-      <c r="D3011" s="20" t="n"/>
-      <c r="E3011" s="20" t="n"/>
-      <c r="F3011" s="20" t="n"/>
-    </row>
-    <row r="3012" ht="20" customHeight="1">
-      <c r="A3012" s="18" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B3012" s="19" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C3012" s="20" t="n"/>
-      <c r="D3012" s="20" t="n"/>
-      <c r="E3012" s="20" t="n"/>
-      <c r="F3012" s="20" t="n"/>
-    </row>
-    <row r="3013" ht="20" customHeight="1">
-      <c r="A3013" s="18" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B3013" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C3013" s="20" t="n"/>
-      <c r="D3013" s="20" t="n"/>
-      <c r="E3013" s="20" t="n"/>
-      <c r="F3013" s="20" t="n"/>
-    </row>
-    <row r="3014" ht="45" customHeight="1">
-      <c r="A3014" s="18" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B3014" s="22" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/paraguas-como-obsequio-dia-aitites-amamas-fiestas/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C3014" s="20" t="n"/>
-      <c r="D3014" s="20" t="n"/>
-      <c r="E3014" s="20" t="n"/>
-      <c r="F3014" s="20" t="n"/>
-    </row>
-    <row r="3016" ht="30" customHeight="1">
-      <c r="A3016" s="16" t="inlineStr">
-        <is>
-          <t>FICHA 202: EUS-46833</t>
-        </is>
-      </c>
-      <c r="B3016" s="17" t="n"/>
-      <c r="C3016" s="17" t="n"/>
-      <c r="D3016" s="17" t="n"/>
-      <c r="E3016" s="17" t="n"/>
-      <c r="F3016" s="17" t="n"/>
-    </row>
-    <row r="3017" ht="20" customHeight="1">
-      <c r="A3017" s="18" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B3017" s="19" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C3017" s="20" t="n"/>
-      <c r="D3017" s="20" t="n"/>
-      <c r="E3017" s="20" t="n"/>
-      <c r="F3017" s="20" t="n"/>
-    </row>
-    <row r="3018" ht="20" customHeight="1">
-      <c r="A3018" s="18" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B3018" s="19" t="inlineStr">
-        <is>
-          <t>Suministro e instalación de 27 farolas led de alumbrado solar autónomo</t>
-        </is>
-      </c>
-      <c r="C3018" s="20" t="n"/>
-      <c r="D3018" s="20" t="n"/>
-      <c r="E3018" s="20" t="n"/>
-      <c r="F3018" s="20" t="n"/>
-    </row>
-    <row r="3019" ht="20" customHeight="1">
-      <c r="A3019" s="18" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3019" s="19" t="inlineStr">
-        <is>
-          <t>EUS-46833</t>
-        </is>
-      </c>
-      <c r="C3019" s="20" t="n"/>
-      <c r="D3019" s="20" t="n"/>
-      <c r="E3019" s="20" t="n"/>
-      <c r="F3019" s="20" t="n"/>
-    </row>
-    <row r="3020" ht="20" customHeight="1">
-      <c r="A3020" s="18" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B3020" s="19" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C3020" s="20" t="n"/>
-      <c r="D3020" s="20" t="n"/>
-      <c r="E3020" s="20" t="n"/>
-      <c r="F3020" s="20" t="n"/>
-    </row>
-    <row r="3021" ht="20" customHeight="1">
-      <c r="A3021" s="18" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B3021" s="19" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C3021" s="20" t="n"/>
-      <c r="D3021" s="20" t="n"/>
-      <c r="E3021" s="20" t="n"/>
-      <c r="F3021" s="20" t="n"/>
-    </row>
-    <row r="3022" ht="20" customHeight="1">
-      <c r="A3022" s="18" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B3022" s="19" t="inlineStr"/>
-      <c r="C3022" s="20" t="n"/>
-      <c r="D3022" s="20" t="n"/>
-      <c r="E3022" s="20" t="n"/>
-      <c r="F3022" s="20" t="n"/>
-    </row>
-    <row r="3023" ht="20" customHeight="1">
-      <c r="A3023" s="18" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B3023" s="19" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C3023" s="20" t="n"/>
-      <c r="D3023" s="20" t="n"/>
-      <c r="E3023" s="20" t="n"/>
-      <c r="F3023" s="20" t="n"/>
-    </row>
-    <row r="3024" ht="20" customHeight="1">
-      <c r="A3024" s="18" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B3024" s="19" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C3024" s="20" t="n"/>
-      <c r="D3024" s="20" t="n"/>
-      <c r="E3024" s="20" t="n"/>
-      <c r="F3024" s="20" t="n"/>
-    </row>
-    <row r="3025" ht="20" customHeight="1">
-      <c r="A3025" s="18" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B3025" s="19" t="inlineStr"/>
-      <c r="C3025" s="20" t="n"/>
-      <c r="D3025" s="20" t="n"/>
-      <c r="E3025" s="20" t="n"/>
-      <c r="F3025" s="20" t="n"/>
-    </row>
-    <row r="3026" ht="20" customHeight="1">
-      <c r="A3026" s="18" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B3026" s="19" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C3026" s="20" t="n"/>
-      <c r="D3026" s="20" t="n"/>
-      <c r="E3026" s="20" t="n"/>
-      <c r="F3026" s="20" t="n"/>
-    </row>
-    <row r="3027" ht="20" customHeight="1">
-      <c r="A3027" s="18" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B3027" s="19" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C3027" s="20" t="n"/>
-      <c r="D3027" s="20" t="n"/>
-      <c r="E3027" s="20" t="n"/>
-      <c r="F3027" s="20" t="n"/>
-    </row>
-    <row r="3028" ht="20" customHeight="1">
-      <c r="A3028" s="18" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B3028" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C3028" s="20" t="n"/>
-      <c r="D3028" s="20" t="n"/>
-      <c r="E3028" s="20" t="n"/>
-      <c r="F3028" s="20" t="n"/>
-    </row>
-    <row r="3029" ht="45" customHeight="1">
-      <c r="A3029" s="18" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B3029" s="22" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-e-instalacion-27-farolas-led-alumbrado-solar-autonomo/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C3029" s="20" t="n"/>
-      <c r="D3029" s="20" t="n"/>
-      <c r="E3029" s="20" t="n"/>
-      <c r="F3029" s="20" t="n"/>
-    </row>
-    <row r="3031" ht="30" customHeight="1">
-      <c r="A3031" s="16" t="inlineStr">
-        <is>
-          <t>FICHA 203: EUS-10725</t>
-        </is>
-      </c>
-      <c r="B3031" s="17" t="n"/>
-      <c r="C3031" s="17" t="n"/>
-      <c r="D3031" s="17" t="n"/>
-      <c r="E3031" s="17" t="n"/>
-      <c r="F3031" s="17" t="n"/>
-    </row>
-    <row r="3032" ht="20" customHeight="1">
-      <c r="A3032" s="18" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B3032" s="19" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C3032" s="20" t="n"/>
-      <c r="D3032" s="20" t="n"/>
-      <c r="E3032" s="20" t="n"/>
-      <c r="F3032" s="20" t="n"/>
-    </row>
-    <row r="3033" ht="45" customHeight="1">
-      <c r="A3033" s="18" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B3033" s="19" t="inlineStr">
-        <is>
-          <t>Suministro en régimen de alquiler de 2 contenedores y 1 caseta vestuario con 2 duchas para uso de la brigada municipal de obras</t>
-        </is>
-      </c>
-      <c r="C3033" s="20" t="n"/>
-      <c r="D3033" s="20" t="n"/>
-      <c r="E3033" s="20" t="n"/>
-      <c r="F3033" s="20" t="n"/>
-    </row>
-    <row r="3034" ht="20" customHeight="1">
-      <c r="A3034" s="18" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3034" s="19" t="inlineStr">
-        <is>
-          <t>EUS-10725</t>
-        </is>
-      </c>
-      <c r="C3034" s="20" t="n"/>
-      <c r="D3034" s="20" t="n"/>
-      <c r="E3034" s="20" t="n"/>
-      <c r="F3034" s="20" t="n"/>
-    </row>
-    <row r="3035" ht="20" customHeight="1">
-      <c r="A3035" s="18" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B3035" s="19" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C3035" s="20" t="n"/>
-      <c r="D3035" s="20" t="n"/>
-      <c r="E3035" s="20" t="n"/>
-      <c r="F3035" s="20" t="n"/>
-    </row>
-    <row r="3036" ht="20" customHeight="1">
-      <c r="A3036" s="18" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B3036" s="19" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C3036" s="20" t="n"/>
-      <c r="D3036" s="20" t="n"/>
-      <c r="E3036" s="20" t="n"/>
-      <c r="F3036" s="20" t="n"/>
-    </row>
-    <row r="3037" ht="20" customHeight="1">
-      <c r="A3037" s="18" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B3037" s="19" t="inlineStr"/>
-      <c r="C3037" s="20" t="n"/>
-      <c r="D3037" s="20" t="n"/>
-      <c r="E3037" s="20" t="n"/>
-      <c r="F3037" s="20" t="n"/>
-    </row>
-    <row r="3038" ht="20" customHeight="1">
-      <c r="A3038" s="18" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B3038" s="19" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C3038" s="20" t="n"/>
-      <c r="D3038" s="20" t="n"/>
-      <c r="E3038" s="20" t="n"/>
-      <c r="F3038" s="20" t="n"/>
-    </row>
-    <row r="3039" ht="20" customHeight="1">
-      <c r="A3039" s="18" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B3039" s="19" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C3039" s="20" t="n"/>
-      <c r="D3039" s="20" t="n"/>
-      <c r="E3039" s="20" t="n"/>
-      <c r="F3039" s="20" t="n"/>
-    </row>
-    <row r="3040" ht="20" customHeight="1">
-      <c r="A3040" s="18" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B3040" s="19" t="inlineStr"/>
-      <c r="C3040" s="20" t="n"/>
-      <c r="D3040" s="20" t="n"/>
-      <c r="E3040" s="20" t="n"/>
-      <c r="F3040" s="20" t="n"/>
-    </row>
-    <row r="3041" ht="20" customHeight="1">
-      <c r="A3041" s="18" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B3041" s="19" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C3041" s="20" t="n"/>
-      <c r="D3041" s="20" t="n"/>
-      <c r="E3041" s="20" t="n"/>
-      <c r="F3041" s="20" t="n"/>
-    </row>
-    <row r="3042" ht="20" customHeight="1">
-      <c r="A3042" s="18" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B3042" s="19" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C3042" s="20" t="n"/>
-      <c r="D3042" s="20" t="n"/>
-      <c r="E3042" s="20" t="n"/>
-      <c r="F3042" s="20" t="n"/>
-    </row>
-    <row r="3043" ht="20" customHeight="1">
-      <c r="A3043" s="18" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B3043" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C3043" s="20" t="n"/>
-      <c r="D3043" s="20" t="n"/>
-      <c r="E3043" s="20" t="n"/>
-      <c r="F3043" s="20" t="n"/>
-    </row>
-    <row r="3044" ht="45" customHeight="1">
-      <c r="A3044" s="18" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B3044" s="22" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-regimen-alquiler-2-contenedores-y-1-caseta-vestuario-2-duchas-uso-brigada-municipal-obras/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C3044" s="20" t="n"/>
-      <c r="D3044" s="20" t="n"/>
-      <c r="E3044" s="20" t="n"/>
-      <c r="F3044" s="20" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="2842">
+  <mergeCells count="2800">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B2192:F2192"/>
     <mergeCell ref="B1765:F1765"/>
@@ -52528,7 +51750,6 @@
     <mergeCell ref="B2858:F2858"/>
     <mergeCell ref="B2103:F2103"/>
     <mergeCell ref="A976:F976"/>
-    <mergeCell ref="B3003:F3003"/>
     <mergeCell ref="B2242:F2242"/>
     <mergeCell ref="B157:F157"/>
     <mergeCell ref="B455:F455"/>
@@ -52537,7 +51758,6 @@
     <mergeCell ref="B762:F762"/>
     <mergeCell ref="B1821:F1821"/>
     <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B3005:F3005"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B1973:F1973"/>
     <mergeCell ref="B1218:F1218"/>
@@ -52656,11 +51876,9 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B2275:F2275"/>
     <mergeCell ref="B2573:F2573"/>
-    <mergeCell ref="B3002:F3002"/>
     <mergeCell ref="B2996:F2996"/>
     <mergeCell ref="B1184:F1184"/>
     <mergeCell ref="B2270:F2270"/>
-    <mergeCell ref="B3027:F3027"/>
     <mergeCell ref="B2699:F2699"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -52670,7 +51888,6 @@
     <mergeCell ref="B902:F902"/>
     <mergeCell ref="B2724:F2724"/>
     <mergeCell ref="B1331:F1331"/>
-    <mergeCell ref="B3022:F3022"/>
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B1629:F1629"/>
     <mergeCell ref="B597:F597"/>
@@ -52775,7 +51992,6 @@
     <mergeCell ref="B1654:F1654"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1925:F1925"/>
-    <mergeCell ref="B3020:F3020"/>
     <mergeCell ref="B893:F893"/>
     <mergeCell ref="B2838:F2838"/>
     <mergeCell ref="B2083:F2083"/>
@@ -52807,9 +52023,7 @@
     <mergeCell ref="B921:F921"/>
     <mergeCell ref="B606:F606"/>
     <mergeCell ref="B2741:F2741"/>
-    <mergeCell ref="B3039:F3039"/>
     <mergeCell ref="B2007:F2007"/>
-    <mergeCell ref="B3033:F3033"/>
     <mergeCell ref="B2436:F2436"/>
     <mergeCell ref="A1276:F1276"/>
     <mergeCell ref="B2770:F2770"/>
@@ -52878,7 +52092,6 @@
     <mergeCell ref="B2073:F2073"/>
     <mergeCell ref="B2048:F2048"/>
     <mergeCell ref="B261:F261"/>
-    <mergeCell ref="A3016:F3016"/>
     <mergeCell ref="B2379:F2379"/>
     <mergeCell ref="B2193:F2193"/>
     <mergeCell ref="A616:F616"/>
@@ -53008,7 +52221,6 @@
     <mergeCell ref="A2731:F2731"/>
     <mergeCell ref="B2246:F2246"/>
     <mergeCell ref="A946:F946"/>
-    <mergeCell ref="A3031:F3031"/>
     <mergeCell ref="A631:F631"/>
     <mergeCell ref="B117:F117"/>
     <mergeCell ref="B1783:F1783"/>
@@ -53047,7 +52259,6 @@
     <mergeCell ref="B1804:F1804"/>
     <mergeCell ref="B2882:F2882"/>
     <mergeCell ref="B797:F797"/>
-    <mergeCell ref="B3013:F3013"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="A2011:F2011"/>
     <mergeCell ref="B2592:F2592"/>
@@ -53057,11 +52268,9 @@
     <mergeCell ref="B2884:F2884"/>
     <mergeCell ref="B799:F799"/>
     <mergeCell ref="B2129:F2129"/>
-    <mergeCell ref="B3021:F3021"/>
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B2585:F2585"/>
     <mergeCell ref="B1526:F1526"/>
-    <mergeCell ref="B3014:F3014"/>
     <mergeCell ref="B2473:F2473"/>
     <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B2915:F2915"/>
@@ -53086,7 +52295,6 @@
     <mergeCell ref="B2155:F2155"/>
     <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B368:F368"/>
-    <mergeCell ref="B3041:F3041"/>
     <mergeCell ref="B1254:F1254"/>
     <mergeCell ref="B1430:F1430"/>
     <mergeCell ref="B1552:F1552"/>
@@ -53269,7 +52477,6 @@
     <mergeCell ref="B1304:F1304"/>
     <mergeCell ref="B1608:F1608"/>
     <mergeCell ref="B2695:F2695"/>
-    <mergeCell ref="B3037:F3037"/>
     <mergeCell ref="B1967:F1967"/>
     <mergeCell ref="B908:F908"/>
     <mergeCell ref="B883:F883"/>
@@ -53287,7 +52494,6 @@
     <mergeCell ref="B1353:F1353"/>
     <mergeCell ref="B636:F636"/>
     <mergeCell ref="B2721:F2721"/>
-    <mergeCell ref="B3019:F3019"/>
     <mergeCell ref="B296:F296"/>
     <mergeCell ref="B934:F934"/>
     <mergeCell ref="B1232:F1232"/>
@@ -53406,7 +52612,6 @@
     <mergeCell ref="B2801:F2801"/>
     <mergeCell ref="B2837:F2837"/>
     <mergeCell ref="B2720:F2720"/>
-    <mergeCell ref="B3018:F3018"/>
     <mergeCell ref="B289:F289"/>
     <mergeCell ref="B1479:F1479"/>
     <mergeCell ref="B1777:F1777"/>
@@ -53687,7 +52892,6 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B2283:F2283"/>
-    <mergeCell ref="B3010:F3010"/>
     <mergeCell ref="B925:F925"/>
     <mergeCell ref="B1223:F1223"/>
     <mergeCell ref="B164:F164"/>
@@ -53699,13 +52903,11 @@
     <mergeCell ref="B498:F498"/>
     <mergeCell ref="B1986:F1986"/>
     <mergeCell ref="B2599:F2599"/>
-    <mergeCell ref="B3012:F3012"/>
     <mergeCell ref="B2284:F2284"/>
     <mergeCell ref="B1225:F1225"/>
     <mergeCell ref="B1523:F1523"/>
     <mergeCell ref="B2891:F2891"/>
     <mergeCell ref="B2713:F2713"/>
-    <mergeCell ref="B3011:F3011"/>
     <mergeCell ref="B1979:F1979"/>
     <mergeCell ref="A2191:F2191"/>
     <mergeCell ref="B2286:F2286"/>
@@ -53718,7 +52920,6 @@
     <mergeCell ref="A2491:F2491"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
-    <mergeCell ref="B3036:F3036"/>
     <mergeCell ref="B1249:F1249"/>
     <mergeCell ref="B524:F524"/>
     <mergeCell ref="B1854:F1854"/>
@@ -53726,7 +52927,6 @@
     <mergeCell ref="B67:F67"/>
     <mergeCell ref="B2012:F2012"/>
     <mergeCell ref="B953:F953"/>
-    <mergeCell ref="B3038:F3038"/>
     <mergeCell ref="B1251:F1251"/>
     <mergeCell ref="B1549:F1549"/>
     <mergeCell ref="B1856:F1856"/>
@@ -53810,9 +53010,7 @@
     <mergeCell ref="B1652:F1652"/>
     <mergeCell ref="B2678:F2678"/>
     <mergeCell ref="B891:F891"/>
-    <mergeCell ref="B3009:F3009"/>
     <mergeCell ref="B1191:F1191"/>
-    <mergeCell ref="B3034:F3034"/>
     <mergeCell ref="B609:F609"/>
     <mergeCell ref="B1247:F1247"/>
     <mergeCell ref="B1977:F1977"/>
@@ -53830,9 +53028,7 @@
     <mergeCell ref="B1547:F1547"/>
     <mergeCell ref="B1207:F1207"/>
     <mergeCell ref="B490:F490"/>
-    <mergeCell ref="B3035:F3035"/>
     <mergeCell ref="B1338:F1338"/>
-    <mergeCell ref="B3029:F3029"/>
     <mergeCell ref="B604:F604"/>
     <mergeCell ref="A61:F61"/>
     <mergeCell ref="B2608:F2608"/>
@@ -53999,7 +53195,6 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1303:F1303"/>
     <mergeCell ref="B1297:F1297"/>
-    <mergeCell ref="A3001:F3001"/>
     <mergeCell ref="B2487:F2487"/>
     <mergeCell ref="B2514:F2514"/>
     <mergeCell ref="B2785:F2785"/>
@@ -54115,7 +53310,6 @@
     <mergeCell ref="B2153:F2153"/>
     <mergeCell ref="B1838:F1838"/>
     <mergeCell ref="B779:F779"/>
-    <mergeCell ref="B3028:F3028"/>
     <mergeCell ref="B2810:F2810"/>
     <mergeCell ref="B358:F358"/>
     <mergeCell ref="B2138:F2138"/>
@@ -54322,14 +53516,12 @@
     <mergeCell ref="B1204:F1204"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="B134:F134"/>
-    <mergeCell ref="B3007:F3007"/>
     <mergeCell ref="B922:F922"/>
     <mergeCell ref="B167:F167"/>
     <mergeCell ref="B2290:F2290"/>
     <mergeCell ref="B1220:F1220"/>
     <mergeCell ref="B503:F503"/>
     <mergeCell ref="B2588:F2588"/>
-    <mergeCell ref="B3017:F3017"/>
     <mergeCell ref="B932:F932"/>
     <mergeCell ref="B2702:F2702"/>
     <mergeCell ref="B617:F617"/>
@@ -54433,7 +53625,6 @@
     <mergeCell ref="B1315:F1315"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B2377:F2377"/>
-    <mergeCell ref="B3042:F3042"/>
     <mergeCell ref="B1649:F1649"/>
     <mergeCell ref="B590:F590"/>
     <mergeCell ref="B888:F888"/>
@@ -54457,14 +53648,12 @@
     <mergeCell ref="B512:F512"/>
     <mergeCell ref="B2734:F2734"/>
     <mergeCell ref="B2728:F2728"/>
-    <mergeCell ref="B3032:F3032"/>
     <mergeCell ref="B2000:F2000"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="B941:F941"/>
     <mergeCell ref="A1726:F1726"/>
     <mergeCell ref="B1239:F1239"/>
     <mergeCell ref="B484:F484"/>
-    <mergeCell ref="B3026:F3026"/>
     <mergeCell ref="B2429:F2429"/>
     <mergeCell ref="B732:F732"/>
     <mergeCell ref="B2605:F2605"/>
@@ -54590,7 +53779,6 @@
     <mergeCell ref="B1782:F1782"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
-    <mergeCell ref="B3025:F3025"/>
     <mergeCell ref="B2112:F2112"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B2568:F2568"/>
@@ -54738,7 +53926,6 @@
     <mergeCell ref="B2708:F2708"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="A2461:F2461"/>
-    <mergeCell ref="B3006:F3006"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B1097:F1097"/>
     <mergeCell ref="B2579:F2579"/>
@@ -54750,7 +53937,6 @@
     <mergeCell ref="B1090:F1090"/>
     <mergeCell ref="B1361:F1361"/>
     <mergeCell ref="B2122:F2122"/>
-    <mergeCell ref="B3008:F3008"/>
     <mergeCell ref="B1221:F1221"/>
     <mergeCell ref="B1397:F1397"/>
     <mergeCell ref="B1519:F1519"/>
@@ -54845,7 +54031,6 @@
     <mergeCell ref="B307:F307"/>
     <mergeCell ref="B429:F429"/>
     <mergeCell ref="B1034:F1034"/>
-    <mergeCell ref="B3004:F3004"/>
     <mergeCell ref="B2979:F2979"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B1947:F1947"/>
@@ -54882,7 +54067,6 @@
     <mergeCell ref="B144:F144"/>
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B1116:F1116"/>
-    <mergeCell ref="B3023:F3023"/>
     <mergeCell ref="B1414:F1414"/>
     <mergeCell ref="B2604:F2604"/>
     <mergeCell ref="B907:F907"/>
@@ -54897,7 +54081,6 @@
     <mergeCell ref="B318:F318"/>
     <mergeCell ref="A1741:F1741"/>
     <mergeCell ref="B1098:F1098"/>
-    <mergeCell ref="B3043:F3043"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B1256:F1256"/>
@@ -54917,7 +54100,6 @@
     <mergeCell ref="B1562:F1562"/>
     <mergeCell ref="B2317:F2317"/>
     <mergeCell ref="B1556:F1556"/>
-    <mergeCell ref="B3044:F3044"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
@@ -55017,7 +54199,6 @@
     <mergeCell ref="B197:F197"/>
     <mergeCell ref="B2104:F2104"/>
     <mergeCell ref="B153:F153"/>
-    <mergeCell ref="B3040:F3040"/>
     <mergeCell ref="B1343:F1343"/>
     <mergeCell ref="B1641:F1641"/>
     <mergeCell ref="B2315:F2315"/>
@@ -55145,7 +54326,6 @@
     <mergeCell ref="B2428:F2428"/>
     <mergeCell ref="B2726:F2726"/>
     <mergeCell ref="B1694:F1694"/>
-    <mergeCell ref="B3024:F3024"/>
     <mergeCell ref="B2878:F2878"/>
     <mergeCell ref="B2123:F2123"/>
     <mergeCell ref="B2457:F2457"/>
@@ -55391,9 +54571,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2969" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2984" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2999" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3014" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3029" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3044" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -55405,7 +54582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J204"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59527,12 +58704,12 @@
     <row r="128" ht="28" customHeight="1">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>njaunzdz</t>
+          <t>14587</t>
         </is>
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>Mr. Dzintars Jaunzems</t>
+          <t>A project intends to build an innovative renewable energy pr</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr"/>
@@ -59559,12 +58736,12 @@
     <row r="129" ht="28" customHeight="1">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>14587</t>
+          <t>njaunzdz</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>A project intends to build an innovative renewable energy pr</t>
+          <t>Mr. Dzintars Jaunzems</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr"/>
@@ -60583,12 +59760,12 @@
     <row r="161" ht="28" customHeight="1">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>928057492</t>
+          <t>928211140</t>
         </is>
       </c>
       <c r="B161" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA RODOPI</t>
+          <t>OBSHTINA PARVOMAY</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr"/>
@@ -60615,12 +59792,12 @@
     <row r="162" ht="28" customHeight="1">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>926227393</t>
+          <t>928057492</t>
         </is>
       </c>
       <c r="B162" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA SVILENGRAD</t>
+          <t>OBSHTINA RODOPI</t>
         </is>
       </c>
       <c r="C162" s="6" t="inlineStr"/>
@@ -60647,12 +59824,12 @@
     <row r="163" ht="28" customHeight="1">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>928211140</t>
+          <t>926227393</t>
         </is>
       </c>
       <c r="B163" s="6" t="inlineStr">
         <is>
-          <t>OBSHTINA PARVOMAY</t>
+          <t>OBSHTINA SVILENGRAD</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr"/>
@@ -61383,12 +60560,12 @@
     <row r="186" ht="28" customHeight="1">
       <c r="A186" s="6" t="inlineStr">
         <is>
-          <t>892931076</t>
+          <t>936518123</t>
         </is>
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VILA DE REI</t>
+          <t>Urban Initiative</t>
         </is>
       </c>
       <c r="C186" s="6" t="inlineStr"/>
@@ -61415,12 +60592,12 @@
     <row r="187" ht="28" customHeight="1">
       <c r="A187" s="6" t="inlineStr">
         <is>
-          <t>936518123</t>
+          <t>892931076</t>
         </is>
       </c>
       <c r="B187" s="6" t="inlineStr">
         <is>
-          <t>Urban Initiative</t>
+          <t>MUNICIPIO DE VILA DE REI</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr"/>
@@ -61447,24 +60624,28 @@
     <row r="188" ht="28" customHeight="1">
       <c r="A188" s="6" t="inlineStr">
         <is>
-          <t>EU4H</t>
+          <t>EUS-45445</t>
         </is>
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>European Linkage of Initiative from Science to Action in Hea</t>
-        </is>
-      </c>
-      <c r="C188" s="6" t="inlineStr"/>
+          <t>Coordinación de seguridad y salud en las obras de reparación</t>
+        </is>
+      </c>
+      <c r="C188" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
       <c r="D188" s="6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr"/>
       <c r="F188" s="25" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G188" s="6" t="inlineStr"/>
@@ -61479,12 +60660,13 @@
     <row r="189" ht="28" customHeight="1">
       <c r="A189" s="6" t="inlineStr">
         <is>
-          <t>EUS-75332</t>
+          <t>EUS-92164</t>
         </is>
       </c>
       <c r="B189" s="6" t="inlineStr">
         <is>
-          <t>Renovación de las licencias o suscripciones de software VMWa</t>
+          <t>Coordinación de
+seguridad y salud en las obras de desinfecci</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
@@ -61515,7 +60697,7 @@
     <row r="190" ht="28" customHeight="1">
       <c r="A190" s="6" t="inlineStr">
         <is>
-          <t>EUS-52813</t>
+          <t>EUS-64887</t>
         </is>
       </c>
       <c r="B190" s="6" t="inlineStr">
@@ -61551,7 +60733,7 @@
     <row r="191" ht="28" customHeight="1">
       <c r="A191" s="6" t="inlineStr">
         <is>
-          <t>EUS-91123</t>
+          <t>EUS-78605</t>
         </is>
       </c>
       <c r="B191" s="6" t="inlineStr">
@@ -61587,12 +60769,12 @@
     <row r="192" ht="28" customHeight="1">
       <c r="A192" s="6" t="inlineStr">
         <is>
-          <t>EUS-55604</t>
+          <t>EUS-19539</t>
         </is>
       </c>
       <c r="B192" s="6" t="inlineStr">
         <is>
-          <t>Redacción del proyecto básico, de ejecución y la dirección f</t>
+          <t>coordinación de seguridad y salud en la obra de renovación y</t>
         </is>
       </c>
       <c r="C192" s="6" t="inlineStr">
@@ -61623,12 +60805,12 @@
     <row r="193" ht="28" customHeight="1">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>EUS-64978</t>
+          <t>EUS-34915</t>
         </is>
       </c>
       <c r="B193" s="6" t="inlineStr">
         <is>
-          <t>Ayudas para la adquisición e implantación de sistemas de nue</t>
+          <t>1-alquiler camión cesta- (j9/01/2025) / seguro diario / gest</t>
         </is>
       </c>
       <c r="C193" s="6" t="inlineStr">
@@ -61644,7 +60826,7 @@
       <c r="E193" s="6" t="inlineStr"/>
       <c r="F193" s="25" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G193" s="6" t="inlineStr"/>
@@ -61659,12 +60841,12 @@
     <row r="194" ht="28" customHeight="1">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-66515</t>
         </is>
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y </t>
+          <t>Ayudas para la adquisición e implantación de sistemas de nue</t>
         </is>
       </c>
       <c r="C194" s="6" t="inlineStr">
@@ -61695,12 +60877,12 @@
     <row r="195" ht="28" customHeight="1">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>EUS-29689</t>
+          <t>EUS-12421</t>
         </is>
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Euro</t>
+          <t xml:space="preserve">9 FAROS DE INNOVACIÓN, 3 transiciones (digital, ecológica y </t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
@@ -61731,12 +60913,12 @@
     <row r="196" ht="28" customHeight="1">
       <c r="A196" s="6" t="inlineStr">
         <is>
-          <t>EUS-96720</t>
+          <t>EUS-30744</t>
         </is>
       </c>
       <c r="B196" s="6" t="inlineStr">
         <is>
-          <t>Comunicación previa - Digitalización 2027</t>
+          <t>MEDIO AMBIENTE URBANO Y FEDER. Ayudas mediante el Fondo Euro</t>
         </is>
       </c>
       <c r="C196" s="6" t="inlineStr">
@@ -61767,12 +60949,12 @@
     <row r="197" ht="28" customHeight="1">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>EUS-38676</t>
+          <t>EUS-39957</t>
         </is>
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>Servicio público de transporte urbano de viajeros en autobús</t>
+          <t>Comunicación previa - Digitalización 2027</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
@@ -61803,12 +60985,12 @@
     <row r="198" ht="28" customHeight="1">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>EUS-18235</t>
+          <t>EUS-35301</t>
         </is>
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mantenimiento de la jardinería y limpieza de los parques de </t>
+          <t>transporte autobús histórico centenario funicular</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
@@ -61839,12 +61021,12 @@
     <row r="199" ht="28" customHeight="1">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>EUS-95301</t>
+          <t>EUS-05161</t>
         </is>
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>Productos de limpieza para andretxea</t>
+          <t>suministro artículos de limpieza</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
@@ -61875,12 +61057,12 @@
     <row r="200" ht="28" customHeight="1">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>EUS-12012</t>
+          <t>EUS-89367</t>
         </is>
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t>Menaje para las viviendas municipales</t>
+          <t>diorama estación kontxa ut 980 inaguación pasante</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
@@ -61911,12 +61093,12 @@
     <row r="201" ht="28" customHeight="1">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>EUS-26392</t>
+          <t>EUS-18525</t>
         </is>
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>Menaje de hogar para viviendas municipales</t>
+          <t>trabajos y transportes de mercancías</t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
@@ -61944,116 +61126,8 @@
       <c r="I201" s="6" t="inlineStr"/>
       <c r="J201" s="6" t="inlineStr"/>
     </row>
-    <row r="202" ht="28" customHeight="1">
-      <c r="A202" s="6" t="inlineStr">
-        <is>
-          <t>EUS-09152</t>
-        </is>
-      </c>
-      <c r="B202" s="6" t="inlineStr">
-        <is>
-          <t>Paraguas como obsequio para el día de aitites-amamas en fies</t>
-        </is>
-      </c>
-      <c r="C202" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D202" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E202" s="6" t="inlineStr"/>
-      <c r="F202" s="25" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G202" s="6" t="inlineStr"/>
-      <c r="H202" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I202" s="6" t="inlineStr"/>
-      <c r="J202" s="6" t="inlineStr"/>
-    </row>
-    <row r="203" ht="28" customHeight="1">
-      <c r="A203" s="6" t="inlineStr">
-        <is>
-          <t>EUS-46833</t>
-        </is>
-      </c>
-      <c r="B203" s="6" t="inlineStr">
-        <is>
-          <t>Suministro e instalación de 27 farolas led de alumbrado sola</t>
-        </is>
-      </c>
-      <c r="C203" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D203" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E203" s="6" t="inlineStr"/>
-      <c r="F203" s="25" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G203" s="6" t="inlineStr"/>
-      <c r="H203" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I203" s="6" t="inlineStr"/>
-      <c r="J203" s="6" t="inlineStr"/>
-    </row>
-    <row r="204" ht="28" customHeight="1">
-      <c r="A204" s="6" t="inlineStr">
-        <is>
-          <t>EUS-10725</t>
-        </is>
-      </c>
-      <c r="B204" s="6" t="inlineStr">
-        <is>
-          <t>Suministro en régimen de alquiler de 2 contenedores y 1 case</t>
-        </is>
-      </c>
-      <c r="C204" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D204" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E204" s="6" t="inlineStr"/>
-      <c r="F204" s="25" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G204" s="6" t="inlineStr"/>
-      <c r="H204" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I204" s="6" t="inlineStr"/>
-      <c r="J204" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J204"/>
+  <autoFilter ref="A1:J201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-10-25
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$216</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$211</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M216"/>
+  <dimension ref="A1:M218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 24/10/2026 09:55 - 210 convocatorias - 12 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 25/10/2026 10:15 - 212 convocatorias - 13 nuevas</t>
         </is>
       </c>
     </row>
@@ -4120,19 +4120,15 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr"/>
       <c r="E77" s="10" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -4153,7 +4149,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr"/>
@@ -4171,15 +4167,19 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr"/>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="L78" s="6" t="inlineStr"/>
@@ -4692,12 +4692,12 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr"/>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="L89" s="6" t="inlineStr"/>
@@ -4739,12 +4739,12 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr"/>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="L90" s="6" t="inlineStr"/>
@@ -4786,12 +4786,12 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr"/>
@@ -4833,12 +4833,12 @@
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="L92" s="6" t="inlineStr"/>
@@ -8734,12 +8734,12 @@
       </c>
       <c r="B175" s="6" t="inlineStr">
         <is>
-          <t>877682967</t>
+          <t>UCPM</t>
         </is>
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
+          <t>RIsk WATER flooding  EXercise</t>
         </is>
       </c>
       <c r="D175" s="6" t="inlineStr"/>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="K175" s="6" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
+          <t>RIsk WATER flooding EXercise</t>
         </is>
       </c>
       <c r="L175" s="6" t="inlineStr"/>
@@ -8781,12 +8781,12 @@
       </c>
       <c r="B176" s="6" t="inlineStr">
         <is>
-          <t>UCPM</t>
+          <t>877682967</t>
         </is>
       </c>
       <c r="C176" s="6" t="inlineStr">
         <is>
-          <t>RIsk WATER flooding  EXercise</t>
+          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
         </is>
       </c>
       <c r="D176" s="6" t="inlineStr"/>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="K176" s="6" t="inlineStr">
         <is>
-          <t>RIsk WATER flooding EXercise</t>
+          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
         </is>
       </c>
       <c r="L176" s="6" t="inlineStr"/>
@@ -10104,12 +10104,13 @@
       </c>
       <c r="B205" s="6" t="inlineStr">
         <is>
-          <t>EUS-93732</t>
+          <t>EUS-18844</t>
         </is>
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
+          <t>Contratación del servicio de mantenimiento integral e inspección de las instalaciones térmicas en edificios e instalaciones 
+municipales del Ayuntamiento de Amorebieta-Etxano</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
@@ -10126,12 +10127,12 @@
       <c r="G205" s="6" t="inlineStr"/>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I205" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I205" s="11" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J205" s="6" t="inlineStr"/>
@@ -10159,12 +10160,12 @@
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>EUS-28838</t>
+          <t>EUS-01951</t>
         </is>
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocatorias transversales ligadas a multitud de líneas innovadoras, que atañen a inteligencia artificial y digitalización, energía y descarbonizació</t>
+          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
         </is>
       </c>
       <c r="D206" s="6" t="inlineStr">
@@ -10214,12 +10215,12 @@
       </c>
       <c r="B207" s="6" t="inlineStr">
         <is>
-          <t>EUS-72505</t>
+          <t>EUS-56052</t>
         </is>
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>Asistencia técnica para la elaboración del Plan de Movilidad Sostenible de la Diputación Foral de Álava</t>
+          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocatorias transversales ligadas a multitud de líneas innovadoras, que atañen a inteligencia artificial y digitalización, energía y descarbonizació</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
@@ -10236,7 +10237,7 @@
       <c r="G207" s="6" t="inlineStr"/>
       <c r="H207" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I207" s="8" t="inlineStr">
@@ -10269,12 +10270,12 @@
       </c>
       <c r="B208" s="6" t="inlineStr">
         <is>
-          <t>EUS-51417</t>
+          <t>EUS-50335</t>
         </is>
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>Alquiler contenedor para residuos y su tratamiento</t>
+          <t>Asistencia técnica para la elaboración del Plan de Movilidad Sostenible de la Diputación Foral de Álava</t>
         </is>
       </c>
       <c r="D208" s="6" t="inlineStr">
@@ -10324,7 +10325,7 @@
       </c>
       <c r="B209" s="6" t="inlineStr">
         <is>
-          <t>EUS-76515</t>
+          <t>EUS-95257</t>
         </is>
       </c>
       <c r="C209" s="6" t="inlineStr">
@@ -10379,7 +10380,7 @@
       </c>
       <c r="B210" s="6" t="inlineStr">
         <is>
-          <t>EUS-69468</t>
+          <t>EUS-13959</t>
         </is>
       </c>
       <c r="C210" s="6" t="inlineStr">
@@ -10434,7 +10435,7 @@
       </c>
       <c r="B211" s="6" t="inlineStr">
         <is>
-          <t>EUS-08471</t>
+          <t>EUS-94998</t>
         </is>
       </c>
       <c r="C211" s="6" t="inlineStr">
@@ -10489,7 +10490,7 @@
       </c>
       <c r="B212" s="6" t="inlineStr">
         <is>
-          <t>EUS-98139</t>
+          <t>EUS-92809</t>
         </is>
       </c>
       <c r="C212" s="6" t="inlineStr">
@@ -10544,7 +10545,7 @@
       </c>
       <c r="B213" s="6" t="inlineStr">
         <is>
-          <t>EUS-44103</t>
+          <t>EUS-29254</t>
         </is>
       </c>
       <c r="C213" s="6" t="inlineStr">
@@ -10599,7 +10600,7 @@
       </c>
       <c r="B214" s="6" t="inlineStr">
         <is>
-          <t>EUS-99252</t>
+          <t>EUS-17441</t>
         </is>
       </c>
       <c r="C214" s="6" t="inlineStr">
@@ -10635,11 +10636,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L214" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L214" s="6" t="inlineStr"/>
       <c r="M214" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -10654,12 +10651,12 @@
       </c>
       <c r="B215" s="6" t="inlineStr">
         <is>
-          <t>EUS-62644</t>
+          <t>EUS-52186</t>
         </is>
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de ejecución para la instalación de una cubierta en Urizar</t>
+          <t>Servicio de atención y gestión integral de la vivienda Comunitaria de Laguardia</t>
         </is>
       </c>
       <c r="D215" s="6" t="inlineStr">
@@ -10709,12 +10706,12 @@
       </c>
       <c r="B216" s="6" t="inlineStr">
         <is>
-          <t>EUS-01533</t>
+          <t>EUS-87459</t>
         </is>
       </c>
       <c r="C216" s="6" t="inlineStr">
         <is>
-          <t>Estudio de detalle cubierta</t>
+          <t>Mejora del alumbrado público Fase 3</t>
         </is>
       </c>
       <c r="D216" s="6" t="inlineStr">
@@ -10756,8 +10753,118 @@
         </is>
       </c>
     </row>
+    <row r="217" ht="40" customHeight="1">
+      <c r="A217" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B217" s="6" t="inlineStr">
+        <is>
+          <t>EUS-84294</t>
+        </is>
+      </c>
+      <c r="C217" s="6" t="inlineStr">
+        <is>
+          <t>Redacción de proyecto de ejecución para la instalación de una cubierta en Urizar</t>
+        </is>
+      </c>
+      <c r="D217" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E217" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F217" s="6" t="inlineStr"/>
+      <c r="G217" s="6" t="inlineStr"/>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I217" s="12" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J217" s="6" t="inlineStr"/>
+      <c r="K217" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L217" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M217" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="40" customHeight="1">
+      <c r="A218" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B218" s="6" t="inlineStr">
+        <is>
+          <t>EUS-19207</t>
+        </is>
+      </c>
+      <c r="C218" s="6" t="inlineStr">
+        <is>
+          <t>Estudio de detalle cubierta</t>
+        </is>
+      </c>
+      <c r="D218" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E218" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F218" s="6" t="inlineStr"/>
+      <c r="G218" s="6" t="inlineStr"/>
+      <c r="H218" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I218" s="12" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J218" s="6" t="inlineStr"/>
+      <c r="K218" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L218" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M218" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M216"/>
+  <autoFilter ref="A4:M218"/>
   <mergeCells count="4">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A204:M204"/>
@@ -10975,6 +11082,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M214" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M215" r:id="rId209"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M216" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M217" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M218" r:id="rId212"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10986,7 +11095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3149"/>
+  <dimension ref="A1:F3179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -25544,7 +25653,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: HORIZON</t>
+          <t>FICHA 72: ERASMUS2027</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -25577,7 +25686,7 @@
       </c>
       <c r="B1068" s="19" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="C1068" s="20" t="n"/>
@@ -25593,7 +25702,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -25607,11 +25716,7 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B1070" s="19" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+      <c r="B1070" s="19" t="inlineStr"/>
       <c r="C1070" s="20" t="n"/>
       <c r="D1070" s="20" t="n"/>
       <c r="E1070" s="20" t="n"/>
@@ -25685,7 +25790,7 @@
       </c>
       <c r="B1075" s="19" t="inlineStr">
         <is>
-          <t>HORIZON-MISS-2021-CIT-02</t>
+          <t>ERASMUS-EDU-2022-PI-ALL-INNO</t>
         </is>
       </c>
       <c r="C1075" s="20" t="n"/>
@@ -25701,7 +25806,7 @@
       </c>
       <c r="B1076" s="19" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
+          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
         </is>
       </c>
       <c r="C1076" s="20" t="n"/>
@@ -25745,7 +25850,7 @@
       </c>
       <c r="B1079" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/ERASMUS2027</t>
         </is>
       </c>
       <c r="C1079" s="20" t="n"/>
@@ -25756,7 +25861,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="16" t="inlineStr">
         <is>
-          <t>FICHA 73: ERASMUS2027</t>
+          <t>FICHA 73: HORIZON</t>
         </is>
       </c>
       <c r="B1081" s="17" t="n"/>
@@ -25789,7 +25894,7 @@
       </c>
       <c r="B1083" s="19" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="C1083" s="20" t="n"/>
@@ -25805,7 +25910,7 @@
       </c>
       <c r="B1084" s="19" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="C1084" s="20" t="n"/>
@@ -25819,7 +25924,11 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B1085" s="19" t="inlineStr"/>
+      <c r="B1085" s="19" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="C1085" s="20" t="n"/>
       <c r="D1085" s="20" t="n"/>
       <c r="E1085" s="20" t="n"/>
@@ -25893,7 +26002,7 @@
       </c>
       <c r="B1090" s="19" t="inlineStr">
         <is>
-          <t>ERASMUS-EDU-2022-PI-ALL-INNO</t>
+          <t>HORIZON-MISS-2021-CIT-02</t>
         </is>
       </c>
       <c r="C1090" s="20" t="n"/>
@@ -25909,7 +26018,7 @@
       </c>
       <c r="B1091" s="19" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neutral cities</t>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIES IN EUROPE</t>
         </is>
       </c>
       <c r="C1091" s="20" t="n"/>
@@ -25953,7 +26062,7 @@
       </c>
       <c r="B1094" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/ERASMUS2027</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON</t>
         </is>
       </c>
       <c r="C1094" s="20" t="n"/>
@@ -28016,7 +28125,7 @@
     <row r="1246" ht="30" customHeight="1">
       <c r="A1246" s="16" t="inlineStr">
         <is>
-          <t>FICHA 84: 928447529</t>
+          <t>FICHA 84: 917779760</t>
         </is>
       </c>
       <c r="B1246" s="17" t="n"/>
@@ -28049,7 +28158,7 @@
       </c>
       <c r="B1248" s="19" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C1248" s="20" t="n"/>
@@ -28065,7 +28174,7 @@
       </c>
       <c r="B1249" s="19" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="C1249" s="20" t="n"/>
@@ -28165,7 +28274,7 @@
       </c>
       <c r="B1256" s="19" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C1256" s="20" t="n"/>
@@ -28209,7 +28318,7 @@
       </c>
       <c r="B1259" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928447529</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917779760</t>
         </is>
       </c>
       <c r="C1259" s="20" t="n"/>
@@ -28220,7 +28329,7 @@
     <row r="1261" ht="30" customHeight="1">
       <c r="A1261" s="16" t="inlineStr">
         <is>
-          <t>FICHA 85: 917671508</t>
+          <t>FICHA 85: 920115617</t>
         </is>
       </c>
       <c r="B1261" s="17" t="n"/>
@@ -28253,7 +28362,7 @@
       </c>
       <c r="B1263" s="19" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C1263" s="20" t="n"/>
@@ -28269,7 +28378,7 @@
       </c>
       <c r="B1264" s="19" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="C1264" s="20" t="n"/>
@@ -28369,7 +28478,7 @@
       </c>
       <c r="B1271" s="19" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C1271" s="20" t="n"/>
@@ -28413,7 +28522,7 @@
       </c>
       <c r="B1274" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917671508</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/920115617</t>
         </is>
       </c>
       <c r="C1274" s="20" t="n"/>
@@ -28424,7 +28533,7 @@
     <row r="1276" ht="30" customHeight="1">
       <c r="A1276" s="16" t="inlineStr">
         <is>
-          <t>FICHA 86: 917779760</t>
+          <t>FICHA 86: 917671508</t>
         </is>
       </c>
       <c r="B1276" s="17" t="n"/>
@@ -28457,7 +28566,7 @@
       </c>
       <c r="B1278" s="19" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C1278" s="20" t="n"/>
@@ -28473,7 +28582,7 @@
       </c>
       <c r="B1279" s="19" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="C1279" s="20" t="n"/>
@@ -28573,7 +28682,7 @@
       </c>
       <c r="B1286" s="19" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C1286" s="20" t="n"/>
@@ -28617,7 +28726,7 @@
       </c>
       <c r="B1289" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917779760</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/917671508</t>
         </is>
       </c>
       <c r="C1289" s="20" t="n"/>
@@ -28628,7 +28737,7 @@
     <row r="1291" ht="30" customHeight="1">
       <c r="A1291" s="16" t="inlineStr">
         <is>
-          <t>FICHA 87: 920115617</t>
+          <t>FICHA 87: 928447529</t>
         </is>
       </c>
       <c r="B1291" s="17" t="n"/>
@@ -28661,7 +28770,7 @@
       </c>
       <c r="B1293" s="19" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C1293" s="20" t="n"/>
@@ -28677,7 +28786,7 @@
       </c>
       <c r="B1294" s="19" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="C1294" s="20" t="n"/>
@@ -28777,7 +28886,7 @@
       </c>
       <c r="B1301" s="19" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C1301" s="20" t="n"/>
@@ -28821,7 +28930,7 @@
       </c>
       <c r="B1304" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/920115617</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/928447529</t>
         </is>
       </c>
       <c r="C1304" s="20" t="n"/>
@@ -45588,7 +45697,7 @@
     <row r="2536" ht="30" customHeight="1">
       <c r="A2536" s="16" t="inlineStr">
         <is>
-          <t>FICHA 170: 877682967</t>
+          <t>FICHA 170: UCPM</t>
         </is>
       </c>
       <c r="B2536" s="17" t="n"/>
@@ -45621,7 +45730,7 @@
       </c>
       <c r="B2538" s="19" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
+          <t>RIsk WATER flooding  EXercise</t>
         </is>
       </c>
       <c r="C2538" s="20" t="n"/>
@@ -45637,7 +45746,7 @@
       </c>
       <c r="B2539" s="19" t="inlineStr">
         <is>
-          <t>877682967</t>
+          <t>UCPM</t>
         </is>
       </c>
       <c r="C2539" s="20" t="n"/>
@@ -45723,7 +45832,11 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B2545" s="19" t="inlineStr"/>
+      <c r="B2545" s="19" t="inlineStr">
+        <is>
+          <t>UCPM-2017-EX-AG</t>
+        </is>
+      </c>
       <c r="C2545" s="20" t="n"/>
       <c r="D2545" s="20" t="n"/>
       <c r="E2545" s="20" t="n"/>
@@ -45737,7 +45850,7 @@
       </c>
       <c r="B2546" s="19" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
+          <t>RIsk WATER flooding EXercise</t>
         </is>
       </c>
       <c r="C2546" s="20" t="n"/>
@@ -45781,7 +45894,7 @@
       </c>
       <c r="B2549" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/877682967</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/UCPM</t>
         </is>
       </c>
       <c r="C2549" s="20" t="n"/>
@@ -45792,7 +45905,7 @@
     <row r="2551" ht="30" customHeight="1">
       <c r="A2551" s="16" t="inlineStr">
         <is>
-          <t>FICHA 171: UCPM</t>
+          <t>FICHA 171: 877682967</t>
         </is>
       </c>
       <c r="B2551" s="17" t="n"/>
@@ -45825,7 +45938,7 @@
       </c>
       <c r="B2553" s="19" t="inlineStr">
         <is>
-          <t>RIsk WATER flooding  EXercise</t>
+          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
         </is>
       </c>
       <c r="C2553" s="20" t="n"/>
@@ -45841,7 +45954,7 @@
       </c>
       <c r="B2554" s="19" t="inlineStr">
         <is>
-          <t>UCPM</t>
+          <t>877682967</t>
         </is>
       </c>
       <c r="C2554" s="20" t="n"/>
@@ -45927,11 +46040,7 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B2560" s="19" t="inlineStr">
-        <is>
-          <t>UCPM-2017-EX-AG</t>
-        </is>
-      </c>
+      <c r="B2560" s="19" t="inlineStr"/>
       <c r="C2560" s="20" t="n"/>
       <c r="D2560" s="20" t="n"/>
       <c r="E2560" s="20" t="n"/>
@@ -45945,7 +46054,7 @@
       </c>
       <c r="B2561" s="19" t="inlineStr">
         <is>
-          <t>RIsk WATER flooding EXercise</t>
+          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RIESGOS</t>
         </is>
       </c>
       <c r="C2561" s="20" t="n"/>
@@ -45989,7 +46098,7 @@
       </c>
       <c r="B2564" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/UCPM</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/877682967</t>
         </is>
       </c>
       <c r="C2564" s="20" t="n"/>
@@ -51520,7 +51629,7 @@
     <row r="2971" ht="30" customHeight="1">
       <c r="A2971" s="16" t="inlineStr">
         <is>
-          <t>FICHA 199: EUS-93732</t>
+          <t>FICHA 199: EUS-18844</t>
         </is>
       </c>
       <c r="B2971" s="17" t="n"/>
@@ -51553,7 +51662,8 @@
       </c>
       <c r="B2973" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
+          <t>Contratación del servicio de mantenimiento integral e inspección de las instalaciones térmicas en edificios e instalaciones 
+municipales del Ayuntamiento de Amorebieta-Etxano</t>
         </is>
       </c>
       <c r="C2973" s="20" t="n"/>
@@ -51569,7 +51679,7 @@
       </c>
       <c r="B2974" s="19" t="inlineStr">
         <is>
-          <t>EUS-93732</t>
+          <t>EUS-18844</t>
         </is>
       </c>
       <c r="C2974" s="20" t="n"/>
@@ -51645,7 +51755,7 @@
       </c>
       <c r="B2979" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C2979" s="20" t="n"/>
@@ -51703,9 +51813,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B2983" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B2983" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C2983" s="20" t="n"/>
@@ -51721,7 +51831,7 @@
       </c>
       <c r="B2984" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/ayudas-al-amparo-de-la-estrategia-de-desarrollo-local-participativo-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-del-servicio-mantenimiento-integral-e-inspeccion-instalaciones-termicas-edificios-e-instalaciones-municipales-del-ayuntamiento-amorebieta-etxano/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2984" s="20" t="n"/>
@@ -51732,7 +51842,7 @@
     <row r="2986" ht="30" customHeight="1">
       <c r="A2986" s="16" t="inlineStr">
         <is>
-          <t>FICHA 200: EUS-28838</t>
+          <t>FICHA 200: EUS-01951</t>
         </is>
       </c>
       <c r="B2986" s="17" t="n"/>
@@ -51765,7 +51875,7 @@
       </c>
       <c r="B2988" s="19" t="inlineStr">
         <is>
-          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocatorias transversales ligadas a multitud de líneas innovadoras, que atañen a inteligencia artificial y digitalización, energía y descarbonizació</t>
+          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
         </is>
       </c>
       <c r="C2988" s="20" t="n"/>
@@ -51781,7 +51891,7 @@
       </c>
       <c r="B2989" s="19" t="inlineStr">
         <is>
-          <t>EUS-28838</t>
+          <t>EUS-01951</t>
         </is>
       </c>
       <c r="C2989" s="20" t="n"/>
@@ -51933,7 +52043,7 @@
       </c>
       <c r="B2999" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonzeharkakodeialdiak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/ayudas-al-amparo-de-la-estrategia-de-desarrollo-local-participativo-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C2999" s="20" t="n"/>
@@ -51944,7 +52054,7 @@
     <row r="3001" ht="30" customHeight="1">
       <c r="A3001" s="16" t="inlineStr">
         <is>
-          <t>FICHA 201: EUS-72505</t>
+          <t>FICHA 201: EUS-56052</t>
         </is>
       </c>
       <c r="B3001" s="17" t="n"/>
@@ -51977,7 +52087,7 @@
       </c>
       <c r="B3003" s="19" t="inlineStr">
         <is>
-          <t>Asistencia técnica para la elaboración del Plan de Movilidad Sostenible de la Diputación Foral de Álava</t>
+          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocatorias transversales ligadas a multitud de líneas innovadoras, que atañen a inteligencia artificial y digitalización, energía y descarbonizació</t>
         </is>
       </c>
       <c r="C3003" s="20" t="n"/>
@@ -51993,7 +52103,7 @@
       </c>
       <c r="B3004" s="19" t="inlineStr">
         <is>
-          <t>EUS-72505</t>
+          <t>EUS-56052</t>
         </is>
       </c>
       <c r="C3004" s="20" t="n"/>
@@ -52069,7 +52179,7 @@
       </c>
       <c r="B3009" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C3009" s="20" t="n"/>
@@ -52145,7 +52255,7 @@
       </c>
       <c r="B3014" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/asistencia-tecnica-elaboracion-del-plan-movilidad-sostenible-diputacion-foral-alava/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonzeharkakodeialdiak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3014" s="20" t="n"/>
@@ -52156,7 +52266,7 @@
     <row r="3016" ht="30" customHeight="1">
       <c r="A3016" s="16" t="inlineStr">
         <is>
-          <t>FICHA 202: EUS-51417</t>
+          <t>FICHA 202: EUS-50335</t>
         </is>
       </c>
       <c r="B3016" s="17" t="n"/>
@@ -52181,7 +52291,7 @@
       <c r="E3017" s="20" t="n"/>
       <c r="F3017" s="20" t="n"/>
     </row>
-    <row r="3018" ht="20" customHeight="1">
+    <row r="3018" ht="45" customHeight="1">
       <c r="A3018" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -52189,7 +52299,7 @@
       </c>
       <c r="B3018" s="19" t="inlineStr">
         <is>
-          <t>Alquiler contenedor para residuos y su tratamiento</t>
+          <t>Asistencia técnica para la elaboración del Plan de Movilidad Sostenible de la Diputación Foral de Álava</t>
         </is>
       </c>
       <c r="C3018" s="20" t="n"/>
@@ -52205,7 +52315,7 @@
       </c>
       <c r="B3019" s="19" t="inlineStr">
         <is>
-          <t>EUS-51417</t>
+          <t>EUS-50335</t>
         </is>
       </c>
       <c r="C3019" s="20" t="n"/>
@@ -52357,7 +52467,7 @@
       </c>
       <c r="B3029" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/alquiler-contenedor-residuos-y-su-tratamiento/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/asistencia-tecnica-elaboracion-del-plan-movilidad-sostenible-diputacion-foral-alava/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3029" s="20" t="n"/>
@@ -52368,7 +52478,7 @@
     <row r="3031" ht="30" customHeight="1">
       <c r="A3031" s="16" t="inlineStr">
         <is>
-          <t>FICHA 203: EUS-76515</t>
+          <t>FICHA 203: EUS-95257</t>
         </is>
       </c>
       <c r="B3031" s="17" t="n"/>
@@ -52417,7 +52527,7 @@
       </c>
       <c r="B3034" s="19" t="inlineStr">
         <is>
-          <t>EUS-76515</t>
+          <t>EUS-95257</t>
         </is>
       </c>
       <c r="C3034" s="20" t="n"/>
@@ -52580,7 +52690,7 @@
     <row r="3046" ht="30" customHeight="1">
       <c r="A3046" s="16" t="inlineStr">
         <is>
-          <t>FICHA 204: EUS-69468</t>
+          <t>FICHA 204: EUS-13959</t>
         </is>
       </c>
       <c r="B3046" s="17" t="n"/>
@@ -52629,7 +52739,7 @@
       </c>
       <c r="B3049" s="19" t="inlineStr">
         <is>
-          <t>EUS-69468</t>
+          <t>EUS-13959</t>
         </is>
       </c>
       <c r="C3049" s="20" t="n"/>
@@ -52792,7 +52902,7 @@
     <row r="3061" ht="30" customHeight="1">
       <c r="A3061" s="16" t="inlineStr">
         <is>
-          <t>FICHA 205: EUS-08471</t>
+          <t>FICHA 205: EUS-94998</t>
         </is>
       </c>
       <c r="B3061" s="17" t="n"/>
@@ -52841,7 +52951,7 @@
       </c>
       <c r="B3064" s="19" t="inlineStr">
         <is>
-          <t>EUS-08471</t>
+          <t>EUS-94998</t>
         </is>
       </c>
       <c r="C3064" s="20" t="n"/>
@@ -53004,7 +53114,7 @@
     <row r="3076" ht="30" customHeight="1">
       <c r="A3076" s="16" t="inlineStr">
         <is>
-          <t>FICHA 206: EUS-98139</t>
+          <t>FICHA 206: EUS-92809</t>
         </is>
       </c>
       <c r="B3076" s="17" t="n"/>
@@ -53053,7 +53163,7 @@
       </c>
       <c r="B3079" s="19" t="inlineStr">
         <is>
-          <t>EUS-98139</t>
+          <t>EUS-92809</t>
         </is>
       </c>
       <c r="C3079" s="20" t="n"/>
@@ -53216,7 +53326,7 @@
     <row r="3091" ht="30" customHeight="1">
       <c r="A3091" s="16" t="inlineStr">
         <is>
-          <t>FICHA 207: EUS-44103</t>
+          <t>FICHA 207: EUS-29254</t>
         </is>
       </c>
       <c r="B3091" s="17" t="n"/>
@@ -53265,7 +53375,7 @@
       </c>
       <c r="B3094" s="19" t="inlineStr">
         <is>
-          <t>EUS-44103</t>
+          <t>EUS-29254</t>
         </is>
       </c>
       <c r="C3094" s="20" t="n"/>
@@ -53428,7 +53538,7 @@
     <row r="3106" ht="30" customHeight="1">
       <c r="A3106" s="16" t="inlineStr">
         <is>
-          <t>FICHA 208: EUS-99252</t>
+          <t>FICHA 208: EUS-17441</t>
         </is>
       </c>
       <c r="B3106" s="17" t="n"/>
@@ -53477,7 +53587,7 @@
       </c>
       <c r="B3109" s="19" t="inlineStr">
         <is>
-          <t>EUS-99252</t>
+          <t>EUS-17441</t>
         </is>
       </c>
       <c r="C3109" s="20" t="n"/>
@@ -53640,7 +53750,7 @@
     <row r="3121" ht="30" customHeight="1">
       <c r="A3121" s="16" t="inlineStr">
         <is>
-          <t>FICHA 209: EUS-62644</t>
+          <t>FICHA 209: EUS-52186</t>
         </is>
       </c>
       <c r="B3121" s="17" t="n"/>
@@ -53665,7 +53775,7 @@
       <c r="E3122" s="20" t="n"/>
       <c r="F3122" s="20" t="n"/>
     </row>
-    <row r="3123" ht="45" customHeight="1">
+    <row r="3123" ht="20" customHeight="1">
       <c r="A3123" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -53673,7 +53783,7 @@
       </c>
       <c r="B3123" s="19" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de ejecución para la instalación de una cubierta en Urizar</t>
+          <t>Servicio de atención y gestión integral de la vivienda Comunitaria de Laguardia</t>
         </is>
       </c>
       <c r="C3123" s="20" t="n"/>
@@ -53689,7 +53799,7 @@
       </c>
       <c r="B3124" s="19" t="inlineStr">
         <is>
-          <t>EUS-62644</t>
+          <t>EUS-52186</t>
         </is>
       </c>
       <c r="C3124" s="20" t="n"/>
@@ -53841,7 +53951,7 @@
       </c>
       <c r="B3134" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-proyecto-ejecucion-instalacion-cubierta-urizar/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-atencion-y-gestion-integral-vivienda-comunitaria-laguardia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3134" s="20" t="n"/>
@@ -53852,7 +53962,7 @@
     <row r="3136" ht="30" customHeight="1">
       <c r="A3136" s="16" t="inlineStr">
         <is>
-          <t>FICHA 210: EUS-01533</t>
+          <t>FICHA 210: EUS-87459</t>
         </is>
       </c>
       <c r="B3136" s="17" t="n"/>
@@ -53885,7 +53995,7 @@
       </c>
       <c r="B3138" s="19" t="inlineStr">
         <is>
-          <t>Estudio de detalle cubierta</t>
+          <t>Mejora del alumbrado público Fase 3</t>
         </is>
       </c>
       <c r="C3138" s="20" t="n"/>
@@ -53901,7 +54011,7 @@
       </c>
       <c r="B3139" s="19" t="inlineStr">
         <is>
-          <t>EUS-01533</t>
+          <t>EUS-87459</t>
         </is>
       </c>
       <c r="C3139" s="20" t="n"/>
@@ -54053,7 +54163,7 @@
       </c>
       <c r="B3149" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/estudio-detalle-cubierta/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mejora-del-alumbrado-publico-fase-3/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C3149" s="20" t="n"/>
@@ -54061,8 +54171,432 @@
       <c r="E3149" s="20" t="n"/>
       <c r="F3149" s="20" t="n"/>
     </row>
+    <row r="3151" ht="30" customHeight="1">
+      <c r="A3151" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 211: EUS-84294</t>
+        </is>
+      </c>
+      <c r="B3151" s="17" t="n"/>
+      <c r="C3151" s="17" t="n"/>
+      <c r="D3151" s="17" t="n"/>
+      <c r="E3151" s="17" t="n"/>
+      <c r="F3151" s="17" t="n"/>
+    </row>
+    <row r="3152" ht="20" customHeight="1">
+      <c r="A3152" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B3152" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C3152" s="20" t="n"/>
+      <c r="D3152" s="20" t="n"/>
+      <c r="E3152" s="20" t="n"/>
+      <c r="F3152" s="20" t="n"/>
+    </row>
+    <row r="3153" ht="45" customHeight="1">
+      <c r="A3153" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B3153" s="19" t="inlineStr">
+        <is>
+          <t>Redacción de proyecto de ejecución para la instalación de una cubierta en Urizar</t>
+        </is>
+      </c>
+      <c r="C3153" s="20" t="n"/>
+      <c r="D3153" s="20" t="n"/>
+      <c r="E3153" s="20" t="n"/>
+      <c r="F3153" s="20" t="n"/>
+    </row>
+    <row r="3154" ht="20" customHeight="1">
+      <c r="A3154" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3154" s="19" t="inlineStr">
+        <is>
+          <t>EUS-84294</t>
+        </is>
+      </c>
+      <c r="C3154" s="20" t="n"/>
+      <c r="D3154" s="20" t="n"/>
+      <c r="E3154" s="20" t="n"/>
+      <c r="F3154" s="20" t="n"/>
+    </row>
+    <row r="3155" ht="20" customHeight="1">
+      <c r="A3155" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B3155" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C3155" s="20" t="n"/>
+      <c r="D3155" s="20" t="n"/>
+      <c r="E3155" s="20" t="n"/>
+      <c r="F3155" s="20" t="n"/>
+    </row>
+    <row r="3156" ht="20" customHeight="1">
+      <c r="A3156" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B3156" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C3156" s="20" t="n"/>
+      <c r="D3156" s="20" t="n"/>
+      <c r="E3156" s="20" t="n"/>
+      <c r="F3156" s="20" t="n"/>
+    </row>
+    <row r="3157" ht="20" customHeight="1">
+      <c r="A3157" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B3157" s="19" t="inlineStr"/>
+      <c r="C3157" s="20" t="n"/>
+      <c r="D3157" s="20" t="n"/>
+      <c r="E3157" s="20" t="n"/>
+      <c r="F3157" s="20" t="n"/>
+    </row>
+    <row r="3158" ht="20" customHeight="1">
+      <c r="A3158" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B3158" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C3158" s="20" t="n"/>
+      <c r="D3158" s="20" t="n"/>
+      <c r="E3158" s="20" t="n"/>
+      <c r="F3158" s="20" t="n"/>
+    </row>
+    <row r="3159" ht="20" customHeight="1">
+      <c r="A3159" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B3159" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C3159" s="20" t="n"/>
+      <c r="D3159" s="20" t="n"/>
+      <c r="E3159" s="20" t="n"/>
+      <c r="F3159" s="20" t="n"/>
+    </row>
+    <row r="3160" ht="20" customHeight="1">
+      <c r="A3160" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B3160" s="19" t="inlineStr"/>
+      <c r="C3160" s="20" t="n"/>
+      <c r="D3160" s="20" t="n"/>
+      <c r="E3160" s="20" t="n"/>
+      <c r="F3160" s="20" t="n"/>
+    </row>
+    <row r="3161" ht="20" customHeight="1">
+      <c r="A3161" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B3161" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C3161" s="20" t="n"/>
+      <c r="D3161" s="20" t="n"/>
+      <c r="E3161" s="20" t="n"/>
+      <c r="F3161" s="20" t="n"/>
+    </row>
+    <row r="3162" ht="20" customHeight="1">
+      <c r="A3162" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B3162" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C3162" s="20" t="n"/>
+      <c r="D3162" s="20" t="n"/>
+      <c r="E3162" s="20" t="n"/>
+      <c r="F3162" s="20" t="n"/>
+    </row>
+    <row r="3163" ht="20" customHeight="1">
+      <c r="A3163" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B3163" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C3163" s="20" t="n"/>
+      <c r="D3163" s="20" t="n"/>
+      <c r="E3163" s="20" t="n"/>
+      <c r="F3163" s="20" t="n"/>
+    </row>
+    <row r="3164" ht="45" customHeight="1">
+      <c r="A3164" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B3164" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-proyecto-ejecucion-instalacion-cubierta-urizar/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C3164" s="20" t="n"/>
+      <c r="D3164" s="20" t="n"/>
+      <c r="E3164" s="20" t="n"/>
+      <c r="F3164" s="20" t="n"/>
+    </row>
+    <row r="3166" ht="30" customHeight="1">
+      <c r="A3166" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 212: EUS-19207</t>
+        </is>
+      </c>
+      <c r="B3166" s="17" t="n"/>
+      <c r="C3166" s="17" t="n"/>
+      <c r="D3166" s="17" t="n"/>
+      <c r="E3166" s="17" t="n"/>
+      <c r="F3166" s="17" t="n"/>
+    </row>
+    <row r="3167" ht="20" customHeight="1">
+      <c r="A3167" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B3167" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C3167" s="20" t="n"/>
+      <c r="D3167" s="20" t="n"/>
+      <c r="E3167" s="20" t="n"/>
+      <c r="F3167" s="20" t="n"/>
+    </row>
+    <row r="3168" ht="20" customHeight="1">
+      <c r="A3168" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B3168" s="19" t="inlineStr">
+        <is>
+          <t>Estudio de detalle cubierta</t>
+        </is>
+      </c>
+      <c r="C3168" s="20" t="n"/>
+      <c r="D3168" s="20" t="n"/>
+      <c r="E3168" s="20" t="n"/>
+      <c r="F3168" s="20" t="n"/>
+    </row>
+    <row r="3169" ht="20" customHeight="1">
+      <c r="A3169" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3169" s="19" t="inlineStr">
+        <is>
+          <t>EUS-19207</t>
+        </is>
+      </c>
+      <c r="C3169" s="20" t="n"/>
+      <c r="D3169" s="20" t="n"/>
+      <c r="E3169" s="20" t="n"/>
+      <c r="F3169" s="20" t="n"/>
+    </row>
+    <row r="3170" ht="20" customHeight="1">
+      <c r="A3170" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B3170" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C3170" s="20" t="n"/>
+      <c r="D3170" s="20" t="n"/>
+      <c r="E3170" s="20" t="n"/>
+      <c r="F3170" s="20" t="n"/>
+    </row>
+    <row r="3171" ht="20" customHeight="1">
+      <c r="A3171" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B3171" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C3171" s="20" t="n"/>
+      <c r="D3171" s="20" t="n"/>
+      <c r="E3171" s="20" t="n"/>
+      <c r="F3171" s="20" t="n"/>
+    </row>
+    <row r="3172" ht="20" customHeight="1">
+      <c r="A3172" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B3172" s="19" t="inlineStr"/>
+      <c r="C3172" s="20" t="n"/>
+      <c r="D3172" s="20" t="n"/>
+      <c r="E3172" s="20" t="n"/>
+      <c r="F3172" s="20" t="n"/>
+    </row>
+    <row r="3173" ht="20" customHeight="1">
+      <c r="A3173" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B3173" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C3173" s="20" t="n"/>
+      <c r="D3173" s="20" t="n"/>
+      <c r="E3173" s="20" t="n"/>
+      <c r="F3173" s="20" t="n"/>
+    </row>
+    <row r="3174" ht="20" customHeight="1">
+      <c r="A3174" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B3174" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C3174" s="20" t="n"/>
+      <c r="D3174" s="20" t="n"/>
+      <c r="E3174" s="20" t="n"/>
+      <c r="F3174" s="20" t="n"/>
+    </row>
+    <row r="3175" ht="20" customHeight="1">
+      <c r="A3175" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B3175" s="19" t="inlineStr"/>
+      <c r="C3175" s="20" t="n"/>
+      <c r="D3175" s="20" t="n"/>
+      <c r="E3175" s="20" t="n"/>
+      <c r="F3175" s="20" t="n"/>
+    </row>
+    <row r="3176" ht="20" customHeight="1">
+      <c r="A3176" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B3176" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C3176" s="20" t="n"/>
+      <c r="D3176" s="20" t="n"/>
+      <c r="E3176" s="20" t="n"/>
+      <c r="F3176" s="20" t="n"/>
+    </row>
+    <row r="3177" ht="20" customHeight="1">
+      <c r="A3177" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B3177" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C3177" s="20" t="n"/>
+      <c r="D3177" s="20" t="n"/>
+      <c r="E3177" s="20" t="n"/>
+      <c r="F3177" s="20" t="n"/>
+    </row>
+    <row r="3178" ht="20" customHeight="1">
+      <c r="A3178" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B3178" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C3178" s="20" t="n"/>
+      <c r="D3178" s="20" t="n"/>
+      <c r="E3178" s="20" t="n"/>
+      <c r="F3178" s="20" t="n"/>
+    </row>
+    <row r="3179" ht="45" customHeight="1">
+      <c r="A3179" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B3179" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/estudio-detalle-cubierta/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C3179" s="20" t="n"/>
+      <c r="D3179" s="20" t="n"/>
+      <c r="E3179" s="20" t="n"/>
+      <c r="F3179" s="20" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="2940">
+  <mergeCells count="2968">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B2192:F2192"/>
     <mergeCell ref="B1765:F1765"/>
@@ -54103,6 +54637,7 @@
     <mergeCell ref="B1664:F1664"/>
     <mergeCell ref="B2879:F2879"/>
     <mergeCell ref="B2539:F2539"/>
+    <mergeCell ref="B3152:F3152"/>
     <mergeCell ref="B725:F725"/>
     <mergeCell ref="B1067:F1067"/>
     <mergeCell ref="B1778:F1778"/>
@@ -54114,6 +54649,8 @@
     <mergeCell ref="B1794:F1794"/>
     <mergeCell ref="B1788:F1788"/>
     <mergeCell ref="B718:F718"/>
+    <mergeCell ref="B3179:F3179"/>
+    <mergeCell ref="B3154:F3154"/>
     <mergeCell ref="B2839:F2839"/>
     <mergeCell ref="B1025:F1025"/>
     <mergeCell ref="B1367:F1367"/>
@@ -54229,6 +54766,7 @@
     <mergeCell ref="B2863:F2863"/>
     <mergeCell ref="B778:F778"/>
     <mergeCell ref="B2108:F2108"/>
+    <mergeCell ref="B3161:F3161"/>
     <mergeCell ref="B1076:F1076"/>
     <mergeCell ref="B1586:F1586"/>
     <mergeCell ref="B2406:F2406"/>
@@ -54635,6 +55173,7 @@
     <mergeCell ref="B279:F279"/>
     <mergeCell ref="B2862:F2862"/>
     <mergeCell ref="B410:F410"/>
+    <mergeCell ref="B3160:F3160"/>
     <mergeCell ref="B733:F733"/>
     <mergeCell ref="B708:F708"/>
     <mergeCell ref="B1463:F1463"/>
@@ -54642,6 +55181,7 @@
     <mergeCell ref="B1978:F1978"/>
     <mergeCell ref="B281:F281"/>
     <mergeCell ref="B1972:F1972"/>
+    <mergeCell ref="B3162:F3162"/>
     <mergeCell ref="B2407:F2407"/>
     <mergeCell ref="B2092:F2092"/>
     <mergeCell ref="B1033:F1033"/>
@@ -54651,6 +55191,7 @@
     <mergeCell ref="B1362:F1362"/>
     <mergeCell ref="B759:F759"/>
     <mergeCell ref="B1057:F1057"/>
+    <mergeCell ref="B3178:F3178"/>
     <mergeCell ref="B1093:F1093"/>
     <mergeCell ref="B1364:F1364"/>
     <mergeCell ref="B2119:F2119"/>
@@ -54673,6 +55214,7 @@
     <mergeCell ref="B2875:F2875"/>
     <mergeCell ref="B790:F790"/>
     <mergeCell ref="B2120:F2120"/>
+    <mergeCell ref="B3173:F3173"/>
     <mergeCell ref="B1088:F1088"/>
     <mergeCell ref="B1359:F1359"/>
     <mergeCell ref="B2418:F2418"/>
@@ -54728,6 +55270,7 @@
     <mergeCell ref="B2518:F2518"/>
     <mergeCell ref="B1459:F1459"/>
     <mergeCell ref="B704:F704"/>
+    <mergeCell ref="B3156:F3156"/>
     <mergeCell ref="B1757:F1757"/>
     <mergeCell ref="B1002:F1002"/>
     <mergeCell ref="B2649:F2649"/>
@@ -54737,6 +55280,7 @@
     <mergeCell ref="B2213:F2213"/>
     <mergeCell ref="B399:F399"/>
     <mergeCell ref="B2642:F2642"/>
+    <mergeCell ref="B3158:F3158"/>
     <mergeCell ref="B2818:F2818"/>
     <mergeCell ref="B1759:F1759"/>
     <mergeCell ref="B1004:F1004"/>
@@ -54770,8 +55314,10 @@
     <mergeCell ref="B717:F717"/>
     <mergeCell ref="B2414:F2414"/>
     <mergeCell ref="B2846:F2846"/>
+    <mergeCell ref="B3169:F3169"/>
     <mergeCell ref="B298:F298"/>
     <mergeCell ref="B2118:F2118"/>
+    <mergeCell ref="B3171:F3171"/>
     <mergeCell ref="B1959:F1959"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
@@ -54848,6 +55394,7 @@
     <mergeCell ref="B1272:F1272"/>
     <mergeCell ref="B1570:F1570"/>
     <mergeCell ref="B809:F809"/>
+    <mergeCell ref="A3151:F3151"/>
     <mergeCell ref="A2836:F2836"/>
     <mergeCell ref="B2542:F2542"/>
     <mergeCell ref="B1143:F1143"/>
@@ -55042,6 +55589,7 @@
     <mergeCell ref="B934:F934"/>
     <mergeCell ref="B1232:F1232"/>
     <mergeCell ref="B173:F173"/>
+    <mergeCell ref="B3177:F3177"/>
     <mergeCell ref="B1539:F1539"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
@@ -55145,6 +55693,7 @@
     <mergeCell ref="B714:F714"/>
     <mergeCell ref="B2537:F2537"/>
     <mergeCell ref="B890:F890"/>
+    <mergeCell ref="B3175:F3175"/>
     <mergeCell ref="B1776:F1776"/>
     <mergeCell ref="B2080:F2080"/>
     <mergeCell ref="B2074:F2074"/>
@@ -55265,6 +55814,7 @@
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B1491:F1491"/>
     <mergeCell ref="B2859:F2859"/>
+    <mergeCell ref="B3157:F3157"/>
     <mergeCell ref="B2098:F2098"/>
     <mergeCell ref="B1370:F1370"/>
     <mergeCell ref="B311:F311"/>
@@ -55280,6 +55830,7 @@
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B1791:F1791"/>
     <mergeCell ref="B1074:F1074"/>
+    <mergeCell ref="B3159:F3159"/>
     <mergeCell ref="B1372:F1372"/>
     <mergeCell ref="B1670:F1670"/>
     <mergeCell ref="B611:F611"/>
@@ -55701,6 +56252,7 @@
     <mergeCell ref="B2718:F2718"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="B2832:F2832"/>
+    <mergeCell ref="B3174:F3174"/>
     <mergeCell ref="B2413:F2413"/>
     <mergeCell ref="B328:F328"/>
     <mergeCell ref="B1658:F1658"/>
@@ -55710,6 +56262,7 @@
     <mergeCell ref="B933:F933"/>
     <mergeCell ref="B1992:F1992"/>
     <mergeCell ref="B172:F172"/>
+    <mergeCell ref="B3176:F3176"/>
     <mergeCell ref="B2421:F2421"/>
     <mergeCell ref="B1389:F1389"/>
     <mergeCell ref="B2719:F2719"/>
@@ -55800,12 +56353,14 @@
     <mergeCell ref="B1029:F1029"/>
     <mergeCell ref="B1900:F1900"/>
     <mergeCell ref="B3116:F3116"/>
+    <mergeCell ref="B3170:F3170"/>
     <mergeCell ref="B712:F712"/>
     <mergeCell ref="B1929:F1929"/>
     <mergeCell ref="B2200:F2200"/>
     <mergeCell ref="B413:F413"/>
     <mergeCell ref="A166:F166"/>
     <mergeCell ref="B589:F589"/>
+    <mergeCell ref="B3172:F3172"/>
     <mergeCell ref="B1597:F1597"/>
     <mergeCell ref="B2417:F2417"/>
     <mergeCell ref="B1773:F1773"/>
@@ -55837,6 +56392,7 @@
     <mergeCell ref="B2711:F2711"/>
     <mergeCell ref="B584:F584"/>
     <mergeCell ref="B2114:F2114"/>
+    <mergeCell ref="B3167:F3167"/>
     <mergeCell ref="B2412:F2412"/>
     <mergeCell ref="B715:F715"/>
     <mergeCell ref="B1013:F1013"/>
@@ -56367,6 +56923,7 @@
     <mergeCell ref="B2079:F2079"/>
     <mergeCell ref="B1324:F1324"/>
     <mergeCell ref="B2394:F2394"/>
+    <mergeCell ref="B3155:F3155"/>
     <mergeCell ref="B1360:F1360"/>
     <mergeCell ref="B599:F599"/>
     <mergeCell ref="B1789:F1789"/>
@@ -56508,6 +57065,7 @@
     <mergeCell ref="A3046:F3046"/>
     <mergeCell ref="B1160:F1160"/>
     <mergeCell ref="B2111:F2111"/>
+    <mergeCell ref="B3164:F3164"/>
     <mergeCell ref="B2409:F2409"/>
     <mergeCell ref="B1377:F1377"/>
     <mergeCell ref="B1648:F1648"/>
@@ -56767,6 +57325,7 @@
     <mergeCell ref="B576:F576"/>
     <mergeCell ref="B138:F138"/>
     <mergeCell ref="B113:F113"/>
+    <mergeCell ref="A3166:F3166"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B2688:F2688"/>
     <mergeCell ref="B1933:F1933"/>
@@ -56901,6 +57460,7 @@
     <mergeCell ref="B251:F251"/>
     <mergeCell ref="A1651:F1651"/>
     <mergeCell ref="B2196:F2196"/>
+    <mergeCell ref="B3168:F3168"/>
     <mergeCell ref="B1769:F1769"/>
     <mergeCell ref="B1014:F1014"/>
     <mergeCell ref="B2067:F2067"/>
@@ -56918,9 +57478,11 @@
     <mergeCell ref="B1016:F1016"/>
     <mergeCell ref="B3128:F3128"/>
     <mergeCell ref="B2707:F2707"/>
+    <mergeCell ref="B3153:F3153"/>
     <mergeCell ref="B282:F282"/>
     <mergeCell ref="B920:F920"/>
     <mergeCell ref="B580:F580"/>
+    <mergeCell ref="B3163:F3163"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B2102:F2102"/>
@@ -57215,6 +57777,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3119" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3134" r:id="rId209"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3149" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3164" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3179" r:id="rId212"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -57226,7 +57790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J211"/>
+  <dimension ref="A1:J213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59580,19 +60144,15 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>HORIZON</t>
+          <t>ERASMUS2027</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIE</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>Horizon Europe</t>
-        </is>
-      </c>
+          <t>Circular design for bio-based innovation towards climate-neu</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr"/>
       <c r="D73" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -59616,15 +60176,19 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>ERASMUS2027</t>
+          <t>HORIZON</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Circular design for bio-based innovation towards climate-neu</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="inlineStr"/>
+          <t>SMART PUBLIC TRANSPORT INITIATIVES FOR CLIMATE-NEUTRAL CITIE</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -59972,12 +60536,12 @@
     <row r="85" ht="28" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>928447529</t>
+          <t>917779760</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
+          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr"/>
@@ -60004,12 +60568,12 @@
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>917671508</t>
+          <t>920115617</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>IN-DER-CITY-BUS GMBH</t>
+          <t>EUE APS</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr"/>
@@ -60036,12 +60600,12 @@
     <row r="87" ht="28" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>917779760</t>
+          <t>917671508</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>MAINZER VERKEHRSGESELLSCHAFT MBH</t>
+          <t>IN-DER-CITY-BUS GMBH</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr"/>
@@ -60068,12 +60632,12 @@
     <row r="88" ht="28" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>920115617</t>
+          <t>928447529</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUE APS</t>
+          <t>SASA SPA AG SOCIETA AUTOBUS SERVIZID'AREA SPA</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr"/>
@@ -62724,12 +63288,12 @@
     <row r="171" ht="28" customHeight="1">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>877682967</t>
+          <t>UCPM</t>
         </is>
       </c>
       <c r="B171" s="6" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RI</t>
+          <t>RIsk WATER flooding  EXercise</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr"/>
@@ -62756,12 +63320,12 @@
     <row r="172" ht="28" customHeight="1">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>UCPM</t>
+          <t>877682967</t>
         </is>
       </c>
       <c r="B172" s="6" t="inlineStr">
         <is>
-          <t>RIsk WATER flooding  EXercise</t>
+          <t>ASOCIACIÓN CENTRO DE INVESTIGACIÓN EN GESTIÓN INTEGRAL DE RI</t>
         </is>
       </c>
       <c r="C172" s="6" t="inlineStr"/>
@@ -63652,12 +64216,12 @@
     <row r="200" ht="28" customHeight="1">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>EUS-93732</t>
+          <t>EUS-18844</t>
         </is>
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ayudas a proyectos al amparo de la estrategia de desarrollo </t>
+          <t>Contratación del servicio de mantenimiento integral e inspec</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
@@ -63673,7 +64237,7 @@
       <c r="E200" s="6" t="inlineStr"/>
       <c r="F200" s="25" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G200" s="6" t="inlineStr"/>
@@ -63688,12 +64252,12 @@
     <row r="201" ht="28" customHeight="1">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>EUS-28838</t>
+          <t>EUS-01951</t>
         </is>
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocator</t>
+          <t xml:space="preserve">Ayudas a proyectos al amparo de la estrategia de desarrollo </t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
@@ -63724,12 +64288,12 @@
     <row r="202" ht="28" customHeight="1">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>EUS-72505</t>
+          <t>EUS-56052</t>
         </is>
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>Asistencia técnica para la elaboración del Plan de Movilidad</t>
+          <t>HORIZON. El gran Programa de I+D+i de la UE lanza convocator</t>
         </is>
       </c>
       <c r="C202" s="6" t="inlineStr">
@@ -63760,12 +64324,12 @@
     <row r="203" ht="28" customHeight="1">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>EUS-51417</t>
+          <t>EUS-50335</t>
         </is>
       </c>
       <c r="B203" s="6" t="inlineStr">
         <is>
-          <t>Alquiler contenedor para residuos y su tratamiento</t>
+          <t>Asistencia técnica para la elaboración del Plan de Movilidad</t>
         </is>
       </c>
       <c r="C203" s="6" t="inlineStr">
@@ -63796,7 +64360,7 @@
     <row r="204" ht="28" customHeight="1">
       <c r="A204" s="6" t="inlineStr">
         <is>
-          <t>EUS-76515</t>
+          <t>EUS-95257</t>
         </is>
       </c>
       <c r="B204" s="6" t="inlineStr">
@@ -63832,7 +64396,7 @@
     <row r="205" ht="28" customHeight="1">
       <c r="A205" s="6" t="inlineStr">
         <is>
-          <t>EUS-69468</t>
+          <t>EUS-13959</t>
         </is>
       </c>
       <c r="B205" s="6" t="inlineStr">
@@ -63868,7 +64432,7 @@
     <row r="206" ht="28" customHeight="1">
       <c r="A206" s="6" t="inlineStr">
         <is>
-          <t>EUS-08471</t>
+          <t>EUS-94998</t>
         </is>
       </c>
       <c r="B206" s="6" t="inlineStr">
@@ -63904,7 +64468,7 @@
     <row r="207" ht="28" customHeight="1">
       <c r="A207" s="6" t="inlineStr">
         <is>
-          <t>EUS-98139</t>
+          <t>EUS-92809</t>
         </is>
       </c>
       <c r="B207" s="6" t="inlineStr">
@@ -63940,7 +64504,7 @@
     <row r="208" ht="28" customHeight="1">
       <c r="A208" s="6" t="inlineStr">
         <is>
-          <t>EUS-44103</t>
+          <t>EUS-29254</t>
         </is>
       </c>
       <c r="B208" s="6" t="inlineStr">
@@ -63976,7 +64540,7 @@
     <row r="209" ht="28" customHeight="1">
       <c r="A209" s="6" t="inlineStr">
         <is>
-          <t>EUS-99252</t>
+          <t>EUS-17441</t>
         </is>
       </c>
       <c r="B209" s="6" t="inlineStr">
@@ -64012,12 +64576,12 @@
     <row r="210" ht="28" customHeight="1">
       <c r="A210" s="6" t="inlineStr">
         <is>
-          <t>EUS-62644</t>
+          <t>EUS-52186</t>
         </is>
       </c>
       <c r="B210" s="6" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de ejecución para la instalación de un</t>
+          <t>Servicio de atención y gestión integral de la vivienda Comun</t>
         </is>
       </c>
       <c r="C210" s="6" t="inlineStr">
@@ -64048,12 +64612,12 @@
     <row r="211" ht="28" customHeight="1">
       <c r="A211" s="6" t="inlineStr">
         <is>
-          <t>EUS-01533</t>
+          <t>EUS-87459</t>
         </is>
       </c>
       <c r="B211" s="6" t="inlineStr">
         <is>
-          <t>Estudio de detalle cubierta</t>
+          <t>Mejora del alumbrado público Fase 3</t>
         </is>
       </c>
       <c r="C211" s="6" t="inlineStr">
@@ -64081,8 +64645,80 @@
       <c r="I211" s="6" t="inlineStr"/>
       <c r="J211" s="6" t="inlineStr"/>
     </row>
+    <row r="212" ht="28" customHeight="1">
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>EUS-84294</t>
+        </is>
+      </c>
+      <c r="B212" s="6" t="inlineStr">
+        <is>
+          <t>Redacción de proyecto de ejecución para la instalación de un</t>
+        </is>
+      </c>
+      <c r="C212" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D212" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E212" s="6" t="inlineStr"/>
+      <c r="F212" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G212" s="6" t="inlineStr"/>
+      <c r="H212" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I212" s="6" t="inlineStr"/>
+      <c r="J212" s="6" t="inlineStr"/>
+    </row>
+    <row r="213" ht="28" customHeight="1">
+      <c r="A213" s="6" t="inlineStr">
+        <is>
+          <t>EUS-19207</t>
+        </is>
+      </c>
+      <c r="B213" s="6" t="inlineStr">
+        <is>
+          <t>Estudio de detalle cubierta</t>
+        </is>
+      </c>
+      <c r="C213" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E213" s="6" t="inlineStr"/>
+      <c r="F213" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G213" s="6" t="inlineStr"/>
+      <c r="H213" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I213" s="6" t="inlineStr"/>
+      <c r="J213" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J211"/>
+  <autoFilter ref="A1:J213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>